<commit_message>
added some coop events
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Configurations/Cards.xlsx
+++ b/Assets/StreamingAssets/Configurations/Cards.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29029"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity\VTuberSim\Assets\StreamingAssets\Configurations\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{688C71BD-0AE5-418B-B638-597A12AAA34E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView windowWidth="24750" windowHeight="10480"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cards" sheetId="1" r:id="rId1"/>
@@ -24,8 +30,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -935,167 +939,17 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="20">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="35">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1114,194 +968,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="11">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -1327,251 +995,9 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
   <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -1586,71 +1012,27 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="49">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
-    <cellStyle name="货币" xfId="2" builtinId="4"/>
-    <cellStyle name="百分比" xfId="3" builtinId="5"/>
-    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
-    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
-    <cellStyle name="超链接" xfId="6" builtinId="8"/>
-    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
-    <cellStyle name="注释" xfId="8" builtinId="10"/>
-    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
-    <cellStyle name="标题" xfId="10" builtinId="15"/>
-    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
-    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
-    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
-    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
-    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
-    <cellStyle name="输入" xfId="16" builtinId="20"/>
-    <cellStyle name="输出" xfId="17" builtinId="21"/>
-    <cellStyle name="计算" xfId="18" builtinId="22"/>
-    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
-    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
-    <cellStyle name="汇总" xfId="21" builtinId="25"/>
-    <cellStyle name="好" xfId="22" builtinId="26"/>
-    <cellStyle name="差" xfId="23" builtinId="27"/>
-    <cellStyle name="适中" xfId="24" builtinId="28"/>
-    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
-    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
-    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
-    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
-    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
-    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
-      <color rgb="00FFFFFF"/>
-      <color rgb="00AB0580"/>
-      <color rgb="0000B050"/>
-      <color rgb="00FFB200"/>
-      <color rgb="004B58FF"/>
-      <color rgb="00FF2160"/>
+      <color rgb="FFFFFFFF"/>
+      <color rgb="FFAB0580"/>
+      <color rgb="FF00B050"/>
+      <color rgb="FFFFB200"/>
+      <color rgb="FF4B58FF"/>
+      <color rgb="FFFF2160"/>
     </mruColors>
   </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1908,42 +1290,43 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr filterMode="1"/>
   <dimension ref="A1:AE61"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="3.425" customWidth="1"/>
-    <col min="2" max="2" width="12.7083333333333" customWidth="1"/>
+    <col min="1" max="1" width="3.42578125" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" customWidth="1"/>
     <col min="3" max="3" width="35" customWidth="1"/>
-    <col min="4" max="4" width="10.425" customWidth="1"/>
-    <col min="5" max="5" width="13.425" customWidth="1"/>
-    <col min="6" max="6" width="10.5666666666667" customWidth="1"/>
-    <col min="7" max="7" width="9.70833333333333" style="2" customWidth="1"/>
-    <col min="8" max="8" width="7.14166666666667" customWidth="1"/>
+    <col min="4" max="4" width="10.42578125" customWidth="1"/>
+    <col min="5" max="5" width="13.42578125" customWidth="1"/>
+    <col min="6" max="6" width="10.5703125" customWidth="1"/>
+    <col min="7" max="7" width="9.7109375" style="2" customWidth="1"/>
+    <col min="8" max="8" width="7.140625" customWidth="1"/>
     <col min="9" max="9" width="14" style="2" customWidth="1"/>
-    <col min="10" max="10" width="10.2833333333333" customWidth="1"/>
-    <col min="11" max="11" width="13.7083333333333" customWidth="1"/>
-    <col min="12" max="12" width="9.70833333333333" style="2" customWidth="1"/>
-    <col min="13" max="13" width="9.70833333333333" customWidth="1"/>
-    <col min="14" max="14" width="12.1416666666667" customWidth="1"/>
-    <col min="15" max="15" width="17.7083333333333" style="2" customWidth="1"/>
+    <col min="10" max="10" width="10.28515625" customWidth="1"/>
+    <col min="11" max="11" width="13.7109375" customWidth="1"/>
+    <col min="12" max="12" width="9.7109375" style="2" customWidth="1"/>
+    <col min="13" max="13" width="9.7109375" customWidth="1"/>
+    <col min="14" max="14" width="12.140625" customWidth="1"/>
+    <col min="15" max="15" width="17.7109375" style="2" customWidth="1"/>
     <col min="16" max="16" width="11" customWidth="1"/>
-    <col min="17" max="17" width="12.2833333333333" customWidth="1"/>
-    <col min="18" max="18" width="17.1416666666667" style="2" customWidth="1"/>
-    <col min="21" max="21" width="17.7083333333333" style="2" customWidth="1"/>
-    <col min="22" max="22" width="10.7083333333333" customWidth="1"/>
+    <col min="17" max="17" width="12.28515625" customWidth="1"/>
+    <col min="18" max="18" width="17.140625" style="2" customWidth="1"/>
+    <col min="21" max="21" width="17.7109375" style="2" customWidth="1"/>
+    <col min="22" max="22" width="10.7109375" customWidth="1"/>
     <col min="23" max="23" width="11" customWidth="1"/>
-    <col min="24" max="24" width="17.7083333333333" style="2" customWidth="1"/>
-    <col min="25" max="25" width="12.425" customWidth="1"/>
-    <col min="26" max="26" width="12.425" style="2" customWidth="1"/>
-    <col min="27" max="27" width="12.2833333333333" customWidth="1"/>
+    <col min="24" max="24" width="17.7109375" style="2" customWidth="1"/>
+    <col min="25" max="25" width="12.42578125" customWidth="1"/>
+    <col min="26" max="26" width="12.42578125" style="2" customWidth="1"/>
+    <col min="27" max="27" width="12.28515625" customWidth="1"/>
     <col min="28" max="28" width="9" style="2"/>
-    <col min="29" max="29" width="4.28333333333333" customWidth="1"/>
+    <col min="29" max="29" width="4.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:31">
@@ -2038,7 +1421,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" hidden="1" spans="1:31">
+    <row r="2" spans="1:31" hidden="1">
       <c r="A2">
         <v>0</v>
       </c>
@@ -2090,7 +1473,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="3" hidden="1" spans="1:31">
+    <row r="3" spans="1:31" hidden="1">
       <c r="A3">
         <v>1</v>
       </c>
@@ -2196,7 +1579,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="5" hidden="1" spans="1:31">
+    <row r="5" spans="1:31" hidden="1">
       <c r="A5">
         <v>3</v>
       </c>
@@ -2316,7 +1699,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="7" hidden="1" spans="1:31">
+    <row r="7" spans="1:31" hidden="1">
       <c r="A7">
         <v>5</v>
       </c>
@@ -2379,7 +1762,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="8" hidden="1" spans="1:31">
+    <row r="8" spans="1:31" hidden="1">
       <c r="A8">
         <v>6</v>
       </c>
@@ -2449,7 +1832,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="9" hidden="1" spans="1:31">
+    <row r="9" spans="1:31" hidden="1">
       <c r="A9">
         <v>8</v>
       </c>
@@ -2509,7 +1892,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" hidden="1" spans="1:31">
+    <row r="10" spans="1:31" hidden="1">
       <c r="A10">
         <v>9</v>
       </c>
@@ -2623,7 +2006,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="12" hidden="1" spans="1:31">
+    <row r="12" spans="1:31" hidden="1">
       <c r="A12">
         <v>11</v>
       </c>
@@ -2686,7 +2069,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="13" hidden="1" spans="1:31">
+    <row r="13" spans="1:31" hidden="1">
       <c r="A13">
         <v>12</v>
       </c>
@@ -2746,7 +2129,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="14" hidden="1" spans="1:31">
+    <row r="14" spans="1:31" hidden="1">
       <c r="A14">
         <v>13</v>
       </c>
@@ -2798,7 +2181,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="15" hidden="1" spans="1:31">
+    <row r="15" spans="1:31" hidden="1">
       <c r="A15">
         <v>14</v>
       </c>
@@ -2850,7 +2233,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="16" hidden="1" spans="1:31">
+    <row r="16" spans="1:31" hidden="1">
       <c r="A16">
         <v>15</v>
       </c>
@@ -2899,7 +2282,7 @@
         <v>0.8</v>
       </c>
       <c r="R16" s="2">
-        <v>1.1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="U16"/>
       <c r="X16"/>
@@ -2910,7 +2293,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="17" hidden="1" spans="1:31">
+    <row r="17" spans="1:31" hidden="1">
       <c r="A17">
         <v>16</v>
       </c>
@@ -3029,7 +2412,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="19" hidden="1" spans="1:31">
+    <row r="19" spans="1:31" hidden="1">
       <c r="A19">
         <v>19</v>
       </c>
@@ -3206,7 +2589,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="22" hidden="1" spans="1:31">
+    <row r="22" spans="1:31" hidden="1">
       <c r="A22">
         <v>22</v>
       </c>
@@ -3266,7 +2649,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="23" hidden="1" spans="1:31">
+    <row r="23" spans="1:31" hidden="1">
       <c r="A23">
         <v>23</v>
       </c>
@@ -3386,7 +2769,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="25" hidden="1" spans="1:31">
+    <row r="25" spans="1:31" hidden="1">
       <c r="A25">
         <v>25</v>
       </c>
@@ -3438,7 +2821,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="26" hidden="1" spans="1:31">
+    <row r="26" spans="1:31" hidden="1">
       <c r="A26">
         <v>26</v>
       </c>
@@ -3615,7 +2998,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="29" hidden="1" spans="1:31">
+    <row r="29" spans="1:31" hidden="1">
       <c r="A29">
         <v>30</v>
       </c>
@@ -3683,7 +3066,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="30" hidden="1" spans="1:31">
+    <row r="30" spans="1:31" hidden="1">
       <c r="A30">
         <v>31</v>
       </c>
@@ -3743,7 +3126,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="31" hidden="1" spans="1:31">
+    <row r="31" spans="1:31" hidden="1">
       <c r="A31">
         <v>32</v>
       </c>
@@ -3803,7 +3186,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="32" hidden="1" spans="1:31">
+    <row r="32" spans="1:31" hidden="1">
       <c r="A32">
         <v>33</v>
       </c>
@@ -4040,7 +3423,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="37" hidden="1" spans="1:31">
+    <row r="37" spans="1:31" hidden="1">
       <c r="A37">
         <v>38</v>
       </c>
@@ -4099,7 +3482,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="38" hidden="1" spans="1:31">
+    <row r="38" spans="1:31" hidden="1">
       <c r="A38">
         <v>39</v>
       </c>
@@ -4158,7 +3541,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="39" hidden="1" spans="1:31">
+    <row r="39" spans="1:31" hidden="1">
       <c r="A39">
         <v>40</v>
       </c>
@@ -4217,7 +3600,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="40" hidden="1" spans="1:31">
+    <row r="40" spans="1:31" hidden="1">
       <c r="A40">
         <v>41</v>
       </c>
@@ -4276,7 +3659,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="41" hidden="1" spans="1:31">
+    <row r="41" spans="1:31" hidden="1">
       <c r="A41">
         <v>42</v>
       </c>
@@ -4335,7 +3718,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="42" hidden="1" spans="1:31">
+    <row r="42" spans="1:31" hidden="1">
       <c r="A42">
         <v>43</v>
       </c>
@@ -4394,7 +3777,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="43" hidden="1" spans="1:31">
+    <row r="43" spans="1:31" hidden="1">
       <c r="A43">
         <v>44</v>
       </c>
@@ -4514,7 +3897,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="45" hidden="1" spans="1:31">
+    <row r="45" spans="1:31" hidden="1">
       <c r="A45">
         <v>46</v>
       </c>
@@ -4581,7 +3964,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="46" hidden="1" spans="1:31">
+    <row r="46" spans="1:31" hidden="1">
       <c r="A46">
         <v>47</v>
       </c>
@@ -4648,7 +4031,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="47" hidden="1" spans="1:31">
+    <row r="47" spans="1:31" hidden="1">
       <c r="A47">
         <v>48</v>
       </c>
@@ -4699,7 +4082,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="48" hidden="1" spans="1:31">
+    <row r="48" spans="1:31" hidden="1">
       <c r="A48">
         <v>49</v>
       </c>
@@ -4811,7 +4194,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="50" hidden="1" spans="1:31">
+    <row r="50" spans="1:31" hidden="1">
       <c r="A50">
         <v>51</v>
       </c>
@@ -4857,7 +4240,7 @@
         <v>18</v>
       </c>
       <c r="Q50">
-        <v>1.1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="R50" s="2">
         <v>1.7</v>
@@ -4870,7 +4253,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="51" hidden="1" spans="1:31">
+    <row r="51" spans="1:31" hidden="1">
       <c r="A51">
         <v>52</v>
       </c>
@@ -4929,7 +4312,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="52" hidden="1" spans="1:31">
+    <row r="52" spans="1:31" hidden="1">
       <c r="A52">
         <v>53</v>
       </c>
@@ -5399,7 +4782,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="61" hidden="1" spans="1:11">
+    <row r="61" spans="1:31" hidden="1">
       <c r="A61">
         <v>62</v>
       </c>
@@ -5435,34 +4818,31 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:AE61" etc:filterBottomFollowUsedRange="0">
+  <autoFilter ref="A1:AE61" xr:uid="{00000000-0009-0000-0000-000000000000}">
     <filterColumn colId="30">
       <filters>
         <filter val="C"/>
       </filters>
     </filterColumn>
-    <extLst/>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
-  <headerFooter/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:I62"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="3.425" customWidth="1"/>
-    <col min="2" max="2" width="27.425" customWidth="1"/>
+    <col min="1" max="1" width="3.42578125" customWidth="1"/>
+    <col min="2" max="2" width="27.42578125" customWidth="1"/>
     <col min="3" max="3" width="35" customWidth="1"/>
     <col min="4" max="4" width="33" customWidth="1"/>
-    <col min="5" max="5" width="19.2833333333333" customWidth="1"/>
-    <col min="6" max="6" width="18.8583333333333" customWidth="1"/>
-    <col min="7" max="8" width="10.2833333333333" customWidth="1"/>
-    <col min="9" max="9" width="15.1416666666667" customWidth="1"/>
+    <col min="5" max="5" width="19.28515625" customWidth="1"/>
+    <col min="6" max="6" width="18.85546875" customWidth="1"/>
+    <col min="7" max="8" width="10.28515625" customWidth="1"/>
+    <col min="9" max="9" width="15.140625" customWidth="1"/>
     <col min="10" max="10" width="22" customWidth="1"/>
   </cols>
   <sheetData>
@@ -6786,26 +6166,24 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
-  <headerFooter/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:O22"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="9.425" customWidth="1"/>
-    <col min="2" max="2" width="27.425" customWidth="1"/>
-    <col min="3" max="3" width="14.425" customWidth="1"/>
-    <col min="4" max="5" width="16.1416666666667" customWidth="1"/>
-    <col min="6" max="6" width="12.425" customWidth="1"/>
-    <col min="7" max="7" width="14.425" customWidth="1"/>
+    <col min="1" max="1" width="9.42578125" customWidth="1"/>
+    <col min="2" max="2" width="27.42578125" customWidth="1"/>
+    <col min="3" max="3" width="14.42578125" customWidth="1"/>
+    <col min="4" max="5" width="16.140625" customWidth="1"/>
+    <col min="6" max="6" width="12.42578125" customWidth="1"/>
+    <col min="7" max="7" width="14.42578125" customWidth="1"/>
     <col min="8" max="8" width="10" customWidth="1"/>
     <col min="9" max="9" width="13" customWidth="1"/>
-    <col min="10" max="10" width="10.1416666666667" customWidth="1"/>
+    <col min="10" max="10" width="10.140625" customWidth="1"/>
     <col min="11" max="11" width="13" customWidth="1"/>
   </cols>
   <sheetData>
@@ -6856,7 +6234,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:15">
       <c r="A2">
         <v>0</v>
       </c>
@@ -6885,7 +6263,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:15">
       <c r="A3">
         <v>1</v>
       </c>
@@ -6908,7 +6286,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:15">
       <c r="A4">
         <v>2</v>
       </c>
@@ -6925,7 +6303,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
+    <row r="5" spans="1:15">
       <c r="A5">
         <v>3</v>
       </c>
@@ -6960,7 +6338,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:15">
       <c r="A6">
         <v>4</v>
       </c>
@@ -6983,7 +6361,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:15">
       <c r="A7">
         <v>5</v>
       </c>
@@ -7006,7 +6384,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="8" spans="1:7">
+    <row r="8" spans="1:15">
       <c r="A8">
         <v>6</v>
       </c>
@@ -7029,7 +6407,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:15">
       <c r="A9">
         <v>7</v>
       </c>
@@ -7052,7 +6430,7 @@
         <v>-0.5</v>
       </c>
     </row>
-    <row r="10" spans="1:7">
+    <row r="10" spans="1:15">
       <c r="A10">
         <v>8</v>
       </c>
@@ -7075,7 +6453,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:9">
+    <row r="11" spans="1:15">
       <c r="A11">
         <v>9</v>
       </c>
@@ -7104,7 +6482,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="12" spans="1:9">
+    <row r="12" spans="1:15">
       <c r="A12">
         <v>10</v>
       </c>
@@ -7133,7 +6511,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="13" spans="1:7">
+    <row r="13" spans="1:15">
       <c r="A13">
         <v>11</v>
       </c>
@@ -7156,7 +6534,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:7">
+    <row r="14" spans="1:15">
       <c r="A14">
         <v>12</v>
       </c>
@@ -7179,7 +6557,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:7">
+    <row r="15" spans="1:15">
       <c r="A15">
         <v>13</v>
       </c>
@@ -7202,7 +6580,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="1:7">
+    <row r="16" spans="1:15">
       <c r="A16">
         <v>14</v>
       </c>
@@ -7271,7 +6649,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:5">
+    <row r="19" spans="1:7">
       <c r="A19">
         <v>17</v>
       </c>
@@ -7288,7 +6666,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:5">
+    <row r="20" spans="1:7">
       <c r="A20">
         <v>18</v>
       </c>
@@ -7305,7 +6683,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:5">
+    <row r="21" spans="1:7">
       <c r="A21">
         <v>19</v>
       </c>
@@ -7347,24 +6725,22 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
-  <headerFooter/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:G11"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="4.85833333333333" customWidth="1"/>
-    <col min="2" max="2" width="22.7083333333333" customWidth="1"/>
-    <col min="3" max="3" width="28.5666666666667" customWidth="1"/>
-    <col min="4" max="4" width="15.5666666666667" customWidth="1"/>
-    <col min="5" max="5" width="16.1416666666667" customWidth="1"/>
+    <col min="1" max="1" width="4.85546875" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="3" max="3" width="28.5703125" customWidth="1"/>
+    <col min="4" max="4" width="15.5703125" customWidth="1"/>
+    <col min="5" max="5" width="16.140625" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="11.1416666666667" customWidth="1"/>
+    <col min="7" max="7" width="11.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -7390,7 +6766,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:7">
       <c r="A2">
         <v>0</v>
       </c>
@@ -7410,7 +6786,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" ht="12.95" customHeight="1" spans="1:6">
+    <row r="3" spans="1:7" ht="12.95" customHeight="1">
       <c r="A3">
         <v>1</v>
       </c>
@@ -7427,7 +6803,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="4" ht="12.95" customHeight="1" spans="1:6">
+    <row r="4" spans="1:7" ht="12.95" customHeight="1">
       <c r="A4">
         <v>2</v>
       </c>
@@ -7444,7 +6820,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:7">
       <c r="A5">
         <v>3</v>
       </c>
@@ -7464,7 +6840,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:7">
       <c r="A6">
         <v>4</v>
       </c>
@@ -7484,7 +6860,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:7">
       <c r="A7">
         <v>5</v>
       </c>
@@ -7504,7 +6880,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:7">
       <c r="A8">
         <v>6</v>
       </c>
@@ -7524,7 +6900,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:7">
       <c r="A9">
         <v>7</v>
       </c>
@@ -7544,7 +6920,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:7">
       <c r="A10">
         <v>8</v>
       </c>
@@ -7564,7 +6940,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:7">
       <c r="A11">
         <v>9</v>
       </c>
@@ -7586,7 +6962,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
-  <headerFooter/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added 2 card conditions
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Configurations/Cards.xlsx
+++ b/Assets/StreamingAssets/Configurations/Cards.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29029"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity\VTuberSim\Assets\StreamingAssets\Configurations\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{402544E3-79F5-492A-BE22-4EEB323B6A61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView windowWidth="24750" windowHeight="10480"/>
+    <workbookView xWindow="0" yWindow="540" windowWidth="38730" windowHeight="20850" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cards" sheetId="1" r:id="rId1"/>
@@ -24,8 +30,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -941,167 +945,17 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="20">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="34">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1120,188 +974,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="11">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -1327,332 +1001,44 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="49">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
-    <cellStyle name="货币" xfId="2" builtinId="4"/>
-    <cellStyle name="百分比" xfId="3" builtinId="5"/>
-    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
-    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
-    <cellStyle name="超链接" xfId="6" builtinId="8"/>
-    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
-    <cellStyle name="注释" xfId="8" builtinId="10"/>
-    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
-    <cellStyle name="标题" xfId="10" builtinId="15"/>
-    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
-    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
-    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
-    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
-    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
-    <cellStyle name="输入" xfId="16" builtinId="20"/>
-    <cellStyle name="输出" xfId="17" builtinId="21"/>
-    <cellStyle name="计算" xfId="18" builtinId="22"/>
-    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
-    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
-    <cellStyle name="汇总" xfId="21" builtinId="25"/>
-    <cellStyle name="好" xfId="22" builtinId="26"/>
-    <cellStyle name="差" xfId="23" builtinId="27"/>
-    <cellStyle name="适中" xfId="24" builtinId="28"/>
-    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
-    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
-    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
-    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
-    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
-    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
-      <color rgb="00FFFFFF"/>
-      <color rgb="00AB0580"/>
-      <color rgb="0000B050"/>
-      <color rgb="00FFB200"/>
-      <color rgb="004B58FF"/>
-      <color rgb="00FF2160"/>
+      <color rgb="FFFFFFFF"/>
+      <color rgb="FFAB0580"/>
+      <color rgb="FF00B050"/>
+      <color rgb="FFFFB200"/>
+      <color rgb="FF4B58FF"/>
+      <color rgb="FFFF2160"/>
     </mruColors>
   </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1910,48 +1296,48 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AG61"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="3.425" customWidth="1"/>
-    <col min="2" max="2" width="12.7083333333333" customWidth="1"/>
+    <col min="1" max="1" width="3.42578125" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" customWidth="1"/>
     <col min="3" max="3" width="35" customWidth="1"/>
-    <col min="4" max="4" width="10.425" style="2" customWidth="1"/>
-    <col min="5" max="5" width="4.85" customWidth="1"/>
-    <col min="6" max="6" width="7.89166666666667" customWidth="1"/>
-    <col min="7" max="7" width="5.06666666666667" customWidth="1"/>
-    <col min="8" max="8" width="5.50833333333333" style="3" customWidth="1"/>
-    <col min="9" max="9" width="10.5666666666667" customWidth="1"/>
-    <col min="10" max="10" width="9.70833333333333" style="4" customWidth="1"/>
-    <col min="11" max="11" width="7.14166666666667" customWidth="1"/>
-    <col min="12" max="12" width="14" style="4" customWidth="1"/>
-    <col min="13" max="13" width="10.2833333333333" customWidth="1"/>
-    <col min="14" max="14" width="13.7083333333333" customWidth="1"/>
-    <col min="15" max="15" width="9.70833333333333" style="4" customWidth="1"/>
-    <col min="16" max="16" width="9.70833333333333" customWidth="1"/>
-    <col min="17" max="17" width="12.1416666666667" customWidth="1"/>
-    <col min="18" max="18" width="17.7083333333333" style="4" customWidth="1"/>
+    <col min="4" max="4" width="10.42578125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="4.85546875" customWidth="1"/>
+    <col min="6" max="6" width="7.85546875" customWidth="1"/>
+    <col min="7" max="7" width="5" customWidth="1"/>
+    <col min="8" max="8" width="5.5703125" style="3" customWidth="1"/>
+    <col min="9" max="9" width="10.5703125" customWidth="1"/>
+    <col min="10" max="10" width="9.7109375" style="3" customWidth="1"/>
+    <col min="11" max="11" width="7.140625" customWidth="1"/>
+    <col min="12" max="12" width="14" style="3" customWidth="1"/>
+    <col min="13" max="13" width="10.28515625" customWidth="1"/>
+    <col min="14" max="14" width="13.7109375" customWidth="1"/>
+    <col min="15" max="15" width="9.7109375" style="3" customWidth="1"/>
+    <col min="16" max="16" width="9.7109375" customWidth="1"/>
+    <col min="17" max="17" width="12.140625" customWidth="1"/>
+    <col min="18" max="18" width="17.7109375" style="3" customWidth="1"/>
     <col min="19" max="19" width="11" customWidth="1"/>
-    <col min="20" max="20" width="12.2833333333333" customWidth="1"/>
-    <col min="21" max="21" width="17.1416666666667" style="4" customWidth="1"/>
-    <col min="24" max="24" width="17.7083333333333" style="4" customWidth="1"/>
-    <col min="25" max="25" width="10.7083333333333" customWidth="1"/>
+    <col min="20" max="20" width="12.28515625" customWidth="1"/>
+    <col min="21" max="21" width="17.140625" style="3" customWidth="1"/>
+    <col min="24" max="24" width="17.7109375" style="3" customWidth="1"/>
+    <col min="25" max="25" width="10.7109375" customWidth="1"/>
     <col min="26" max="26" width="11" customWidth="1"/>
-    <col min="27" max="27" width="17.7083333333333" style="4" customWidth="1"/>
-    <col min="28" max="28" width="12.425" customWidth="1"/>
-    <col min="29" max="29" width="12.425" style="4" customWidth="1"/>
-    <col min="30" max="30" width="12.2833333333333" customWidth="1"/>
-    <col min="31" max="31" width="9" style="4"/>
-    <col min="32" max="32" width="4.28333333333333" customWidth="1"/>
+    <col min="27" max="27" width="17.7109375" style="3" customWidth="1"/>
+    <col min="28" max="28" width="12.42578125" customWidth="1"/>
+    <col min="29" max="29" width="12.42578125" style="3" customWidth="1"/>
+    <col min="30" max="30" width="12.28515625" customWidth="1"/>
+    <col min="31" max="31" width="9" style="3"/>
+    <col min="32" max="32" width="4.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32">
+    <row r="1" spans="1:33">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1979,13 +1365,13 @@
       <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="J1" s="3" t="s">
         <v>9</v>
       </c>
       <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="L1" s="3" t="s">
         <v>11</v>
       </c>
       <c r="M1" t="s">
@@ -1994,62 +1380,62 @@
       <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="4" t="s">
+      <c r="O1" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="6" t="s">
+      <c r="P1" s="2" t="s">
         <v>15</v>
       </c>
       <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="4" t="s">
+      <c r="R1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="6" t="s">
+      <c r="S1" s="2" t="s">
         <v>18</v>
       </c>
       <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="4" t="s">
+      <c r="U1" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="6" t="s">
+      <c r="V1" s="2" t="s">
         <v>21</v>
       </c>
       <c r="W1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="4" t="s">
+      <c r="X1" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="6" t="s">
+      <c r="Y1" s="2" t="s">
         <v>24</v>
       </c>
       <c r="Z1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="4" t="s">
+      <c r="AA1" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="6" t="s">
+      <c r="AB1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="4" t="s">
+      <c r="AC1" s="3" t="s">
         <v>28</v>
       </c>
       <c r="AD1" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" s="4" t="s">
+      <c r="AE1" s="3" t="s">
         <v>30</v>
       </c>
       <c r="AF1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:32">
+    <row r="2" spans="1:33">
       <c r="A2">
         <v>0</v>
       </c>
@@ -2072,10 +1458,10 @@
         <v>37</v>
       </c>
       <c r="J2"/>
-      <c r="K2" s="6">
+      <c r="K2" s="2">
         <v>4</v>
       </c>
-      <c r="L2" s="4">
+      <c r="L2" s="3">
         <v>3</v>
       </c>
       <c r="M2">
@@ -2085,13 +1471,13 @@
         <v>0</v>
       </c>
       <c r="O2"/>
-      <c r="P2" s="6">
+      <c r="P2" s="2">
         <v>11</v>
       </c>
       <c r="Q2">
         <v>7</v>
       </c>
-      <c r="R2" s="4">
+      <c r="R2" s="3">
         <v>7</v>
       </c>
       <c r="U2"/>
@@ -2099,9 +1485,9 @@
       <c r="AA2"/>
       <c r="AC2"/>
       <c r="AE2"/>
-      <c r="AF2" s="7"/>
-    </row>
-    <row r="3" spans="1:32">
+      <c r="AF2" s="5"/>
+    </row>
+    <row r="3" spans="1:33">
       <c r="A3">
         <v>1</v>
       </c>
@@ -2124,10 +1510,10 @@
         <v>37</v>
       </c>
       <c r="J3"/>
-      <c r="K3" s="6">
-        <v>0</v>
-      </c>
-      <c r="L3" s="4">
+      <c r="K3" s="2">
+        <v>0</v>
+      </c>
+      <c r="L3" s="3">
         <v>0</v>
       </c>
       <c r="M3">
@@ -2137,13 +1523,13 @@
         <v>0</v>
       </c>
       <c r="O3"/>
-      <c r="P3" s="6">
+      <c r="P3" s="2">
         <v>2</v>
       </c>
       <c r="Q3">
         <v>4</v>
       </c>
-      <c r="R3" s="4">
+      <c r="R3" s="3">
         <v>4</v>
       </c>
       <c r="U3"/>
@@ -2151,9 +1537,9 @@
       <c r="AA3"/>
       <c r="AC3"/>
       <c r="AE3"/>
-      <c r="AF3" s="7"/>
-    </row>
-    <row r="4" spans="1:32">
+      <c r="AF3" s="5"/>
+    </row>
+    <row r="4" spans="1:33">
       <c r="A4">
         <v>2</v>
       </c>
@@ -2178,7 +1564,7 @@
       <c r="K4">
         <v>5</v>
       </c>
-      <c r="L4" s="4">
+      <c r="L4" s="3">
         <v>4</v>
       </c>
       <c r="M4">
@@ -2187,13 +1573,13 @@
       <c r="N4">
         <v>0</v>
       </c>
-      <c r="P4" s="6">
+      <c r="P4" s="2">
         <v>11</v>
       </c>
       <c r="Q4">
         <v>15</v>
       </c>
-      <c r="R4" s="4">
+      <c r="R4" s="3">
         <v>18</v>
       </c>
       <c r="S4">
@@ -2202,12 +1588,12 @@
       <c r="T4">
         <v>9</v>
       </c>
-      <c r="U4" s="4">
+      <c r="U4" s="3">
         <v>12</v>
       </c>
-      <c r="AF4" s="7"/>
-    </row>
-    <row r="5" spans="1:32">
+      <c r="AF4" s="5"/>
+    </row>
+    <row r="5" spans="1:33">
       <c r="A5">
         <v>3</v>
       </c>
@@ -2230,10 +1616,10 @@
         <v>37</v>
       </c>
       <c r="J5"/>
-      <c r="K5" s="6">
-        <v>3</v>
-      </c>
-      <c r="L5" s="4">
+      <c r="K5" s="2">
+        <v>3</v>
+      </c>
+      <c r="L5" s="3">
         <v>3</v>
       </c>
       <c r="M5">
@@ -2243,31 +1629,31 @@
         <v>0</v>
       </c>
       <c r="O5"/>
-      <c r="P5" s="6">
+      <c r="P5" s="2">
         <v>11</v>
       </c>
       <c r="Q5">
         <v>5</v>
       </c>
-      <c r="R5" s="4">
+      <c r="R5" s="3">
         <v>5</v>
       </c>
-      <c r="S5" s="6">
+      <c r="S5" s="2">
         <v>2</v>
       </c>
       <c r="T5">
         <v>2</v>
       </c>
-      <c r="U5" s="4">
+      <c r="U5" s="3">
         <v>2</v>
       </c>
       <c r="X5"/>
       <c r="AA5"/>
       <c r="AC5"/>
       <c r="AE5"/>
-      <c r="AF5" s="7"/>
-    </row>
-    <row r="6" spans="1:32">
+      <c r="AF5" s="5"/>
+    </row>
+    <row r="6" spans="1:33">
       <c r="A6">
         <v>4</v>
       </c>
@@ -2289,13 +1675,13 @@
       <c r="I6" t="s">
         <v>49</v>
       </c>
-      <c r="J6" s="4">
+      <c r="J6" s="3">
         <v>3</v>
       </c>
       <c r="K6">
         <v>1</v>
       </c>
-      <c r="L6" s="4">
+      <c r="L6" s="3">
         <v>1</v>
       </c>
       <c r="M6">
@@ -2304,7 +1690,7 @@
       <c r="N6">
         <v>1</v>
       </c>
-      <c r="P6" s="6">
+      <c r="P6" s="2">
         <v>0</v>
       </c>
       <c r="S6">
@@ -2313,7 +1699,7 @@
       <c r="T6">
         <v>2</v>
       </c>
-      <c r="U6" s="4">
+      <c r="U6" s="3">
         <v>7</v>
       </c>
       <c r="V6">
@@ -2322,12 +1708,12 @@
       <c r="W6">
         <v>1</v>
       </c>
-      <c r="X6" s="4">
-        <v>1</v>
-      </c>
-      <c r="AF6" s="7"/>
-    </row>
-    <row r="7" spans="1:32">
+      <c r="X6" s="3">
+        <v>1</v>
+      </c>
+      <c r="AF6" s="5"/>
+    </row>
+    <row r="7" spans="1:33">
       <c r="A7">
         <v>5</v>
       </c>
@@ -2350,10 +1736,10 @@
         <v>37</v>
       </c>
       <c r="J7"/>
-      <c r="K7" s="6">
+      <c r="K7" s="2">
         <v>5</v>
       </c>
-      <c r="L7" s="4">
+      <c r="L7" s="3">
         <v>4</v>
       </c>
       <c r="M7">
@@ -2363,34 +1749,34 @@
         <v>1</v>
       </c>
       <c r="O7"/>
-      <c r="P7" s="6">
+      <c r="P7" s="2">
         <v>4</v>
       </c>
       <c r="R7"/>
-      <c r="S7" s="6">
+      <c r="S7" s="2">
         <v>21</v>
       </c>
       <c r="T7">
         <v>2</v>
       </c>
-      <c r="U7" s="4">
-        <v>2</v>
-      </c>
-      <c r="V7" s="6">
+      <c r="U7" s="3">
+        <v>2</v>
+      </c>
+      <c r="V7" s="2">
         <v>14</v>
       </c>
       <c r="W7">
         <v>1</v>
       </c>
-      <c r="X7" s="4">
+      <c r="X7" s="3">
         <v>1</v>
       </c>
       <c r="AA7"/>
       <c r="AC7"/>
       <c r="AE7"/>
-      <c r="AF7" s="7"/>
-    </row>
-    <row r="8" spans="1:32">
+      <c r="AF7" s="5"/>
+    </row>
+    <row r="8" spans="1:33">
       <c r="A8">
         <v>6</v>
       </c>
@@ -2415,10 +1801,10 @@
       <c r="J8">
         <v>0</v>
       </c>
-      <c r="K8" s="6">
-        <v>1</v>
-      </c>
-      <c r="L8" s="4">
+      <c r="K8" s="2">
+        <v>1</v>
+      </c>
+      <c r="L8" s="3">
         <v>1</v>
       </c>
       <c r="M8">
@@ -2428,39 +1814,39 @@
         <v>1</v>
       </c>
       <c r="O8"/>
-      <c r="P8" s="6">
+      <c r="P8" s="2">
         <v>2</v>
       </c>
       <c r="Q8">
         <v>7</v>
       </c>
-      <c r="R8" s="4">
+      <c r="R8" s="3">
         <v>7</v>
       </c>
-      <c r="S8" s="6">
+      <c r="S8" s="2">
         <v>3</v>
       </c>
       <c r="T8">
         <v>1</v>
       </c>
-      <c r="U8" s="4">
-        <v>1</v>
-      </c>
-      <c r="V8" s="6">
+      <c r="U8" s="3">
+        <v>1</v>
+      </c>
+      <c r="V8" s="2">
         <v>14</v>
       </c>
       <c r="W8">
         <v>1</v>
       </c>
-      <c r="X8" s="4">
+      <c r="X8" s="3">
         <v>1</v>
       </c>
       <c r="AA8"/>
       <c r="AC8"/>
       <c r="AE8"/>
-      <c r="AF8" s="7"/>
-    </row>
-    <row r="9" spans="1:32">
+      <c r="AF8" s="5"/>
+    </row>
+    <row r="9" spans="1:33">
       <c r="A9">
         <v>8</v>
       </c>
@@ -2483,10 +1869,10 @@
         <v>37</v>
       </c>
       <c r="J9"/>
-      <c r="K9" s="6">
-        <v>2</v>
-      </c>
-      <c r="L9" s="4">
+      <c r="K9" s="2">
+        <v>2</v>
+      </c>
+      <c r="L9" s="3">
         <v>2</v>
       </c>
       <c r="M9">
@@ -2496,31 +1882,31 @@
         <v>0</v>
       </c>
       <c r="O9"/>
-      <c r="P9" s="6">
+      <c r="P9" s="2">
         <v>6</v>
       </c>
       <c r="Q9">
         <v>3</v>
       </c>
-      <c r="R9" s="4">
+      <c r="R9" s="3">
         <v>4</v>
       </c>
-      <c r="S9" s="6">
+      <c r="S9" s="2">
         <v>2</v>
       </c>
       <c r="T9">
         <v>3</v>
       </c>
-      <c r="U9" s="4">
+      <c r="U9" s="3">
         <v>4</v>
       </c>
       <c r="X9"/>
       <c r="AA9"/>
       <c r="AC9"/>
       <c r="AE9"/>
-      <c r="AF9" s="7"/>
-    </row>
-    <row r="10" spans="1:32">
+      <c r="AF9" s="5"/>
+    </row>
+    <row r="10" spans="1:33">
       <c r="A10">
         <v>9</v>
       </c>
@@ -2543,10 +1929,10 @@
         <v>37</v>
       </c>
       <c r="J10"/>
-      <c r="K10" s="6">
-        <v>2</v>
-      </c>
-      <c r="L10" s="4">
+      <c r="K10" s="2">
+        <v>2</v>
+      </c>
+      <c r="L10" s="3">
         <v>2</v>
       </c>
       <c r="M10">
@@ -2556,31 +1942,31 @@
         <v>0</v>
       </c>
       <c r="O10"/>
-      <c r="P10" s="6">
+      <c r="P10" s="2">
         <v>7</v>
       </c>
       <c r="Q10">
         <v>2</v>
       </c>
-      <c r="R10" s="4">
-        <v>3</v>
-      </c>
-      <c r="S10" s="6">
+      <c r="R10" s="3">
+        <v>3</v>
+      </c>
+      <c r="S10" s="2">
         <v>2</v>
       </c>
       <c r="T10">
         <v>2</v>
       </c>
-      <c r="U10" s="4">
+      <c r="U10" s="3">
         <v>3</v>
       </c>
       <c r="X10"/>
       <c r="AA10"/>
       <c r="AC10"/>
       <c r="AE10"/>
-      <c r="AF10" s="7"/>
-    </row>
-    <row r="11" spans="1:32">
+      <c r="AF10" s="5"/>
+    </row>
+    <row r="11" spans="1:33">
       <c r="A11">
         <v>10</v>
       </c>
@@ -2605,7 +1991,7 @@
       <c r="K11">
         <v>2</v>
       </c>
-      <c r="L11" s="4">
+      <c r="L11" s="3">
         <v>2</v>
       </c>
       <c r="M11">
@@ -2614,25 +2000,25 @@
       <c r="N11">
         <v>0</v>
       </c>
-      <c r="P11" s="6">
+      <c r="P11" s="2">
         <v>15</v>
       </c>
       <c r="Q11">
         <v>2</v>
       </c>
-      <c r="R11" s="4">
-        <v>3</v>
-      </c>
-      <c r="S11" s="6">
+      <c r="R11" s="3">
+        <v>3</v>
+      </c>
+      <c r="S11" s="2">
         <v>2</v>
       </c>
       <c r="T11">
         <v>2</v>
       </c>
-      <c r="U11" s="4">
-        <v>3</v>
-      </c>
-      <c r="AF11" s="7"/>
+      <c r="U11" s="3">
+        <v>3</v>
+      </c>
+      <c r="AF11" s="5"/>
     </row>
     <row r="12" spans="1:33">
       <c r="A12">
@@ -2657,10 +2043,10 @@
         <v>37</v>
       </c>
       <c r="J12"/>
-      <c r="K12" s="6">
+      <c r="K12" s="2">
         <v>6</v>
       </c>
-      <c r="L12" s="4">
+      <c r="L12" s="3">
         <v>6</v>
       </c>
       <c r="M12">
@@ -2670,34 +2056,34 @@
         <v>0</v>
       </c>
       <c r="O12"/>
-      <c r="P12" s="6">
+      <c r="P12" s="2">
         <v>11</v>
       </c>
       <c r="Q12">
         <v>9</v>
       </c>
-      <c r="R12" s="4">
+      <c r="R12" s="3">
         <v>13</v>
       </c>
-      <c r="S12" s="6">
+      <c r="S12" s="2">
         <v>11</v>
       </c>
       <c r="T12">
         <v>9</v>
       </c>
-      <c r="U12" s="4">
+      <c r="U12" s="3">
         <v>13</v>
       </c>
       <c r="X12"/>
       <c r="AA12"/>
       <c r="AC12"/>
       <c r="AE12"/>
-      <c r="AF12" s="7"/>
+      <c r="AF12" s="5"/>
       <c r="AG12" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="13" spans="1:32">
+    <row r="13" spans="1:33">
       <c r="A13">
         <v>12</v>
       </c>
@@ -2720,10 +2106,10 @@
         <v>37</v>
       </c>
       <c r="J13"/>
-      <c r="K13" s="6">
+      <c r="K13" s="2">
         <v>5</v>
       </c>
-      <c r="L13" s="4">
+      <c r="L13" s="3">
         <v>5</v>
       </c>
       <c r="M13">
@@ -2733,31 +2119,31 @@
         <v>0</v>
       </c>
       <c r="O13"/>
-      <c r="P13" s="6">
+      <c r="P13" s="2">
         <v>11</v>
       </c>
       <c r="Q13">
         <v>11</v>
       </c>
-      <c r="R13" s="4">
+      <c r="R13" s="3">
         <v>15</v>
       </c>
-      <c r="S13" s="6">
+      <c r="S13" s="2">
         <v>2</v>
       </c>
       <c r="T13">
         <v>7</v>
       </c>
-      <c r="U13" s="4">
+      <c r="U13" s="3">
         <v>9</v>
       </c>
       <c r="X13"/>
       <c r="AA13"/>
       <c r="AC13"/>
       <c r="AE13"/>
-      <c r="AF13" s="7"/>
-    </row>
-    <row r="14" spans="1:32">
+      <c r="AF13" s="5"/>
+    </row>
+    <row r="14" spans="1:33">
       <c r="A14">
         <v>13</v>
       </c>
@@ -2780,10 +2166,10 @@
         <v>37</v>
       </c>
       <c r="J14"/>
-      <c r="K14" s="6">
+      <c r="K14" s="2">
         <v>5</v>
       </c>
-      <c r="L14" s="4">
+      <c r="L14" s="3">
         <v>4</v>
       </c>
       <c r="M14">
@@ -2793,13 +2179,13 @@
         <v>0</v>
       </c>
       <c r="O14"/>
-      <c r="P14" s="6">
+      <c r="P14" s="2">
         <v>6</v>
       </c>
       <c r="Q14">
         <v>6</v>
       </c>
-      <c r="R14" s="4">
+      <c r="R14" s="3">
         <v>8</v>
       </c>
       <c r="U14"/>
@@ -2807,9 +2193,9 @@
       <c r="AA14"/>
       <c r="AC14"/>
       <c r="AE14"/>
-      <c r="AF14" s="7"/>
-    </row>
-    <row r="15" spans="1:32">
+      <c r="AF14" s="5"/>
+    </row>
+    <row r="15" spans="1:33">
       <c r="A15">
         <v>14</v>
       </c>
@@ -2832,10 +2218,10 @@
         <v>37</v>
       </c>
       <c r="J15"/>
-      <c r="K15" s="6">
+      <c r="K15" s="2">
         <v>4</v>
       </c>
-      <c r="L15" s="4">
+      <c r="L15" s="3">
         <v>4</v>
       </c>
       <c r="M15">
@@ -2845,13 +2231,13 @@
         <v>0</v>
       </c>
       <c r="O15"/>
-      <c r="P15" s="6">
+      <c r="P15" s="2">
         <v>18</v>
       </c>
       <c r="Q15">
         <v>1.4</v>
       </c>
-      <c r="R15" s="4">
+      <c r="R15" s="3">
         <v>1.8</v>
       </c>
       <c r="U15"/>
@@ -2859,9 +2245,9 @@
       <c r="AA15"/>
       <c r="AC15"/>
       <c r="AE15"/>
-      <c r="AF15" s="7"/>
-    </row>
-    <row r="16" spans="1:32">
+      <c r="AF15" s="5"/>
+    </row>
+    <row r="16" spans="1:33">
       <c r="A16">
         <v>15</v>
       </c>
@@ -2884,10 +2270,10 @@
         <v>37</v>
       </c>
       <c r="J16"/>
-      <c r="K16" s="6">
+      <c r="K16" s="2">
         <v>6</v>
       </c>
-      <c r="L16" s="4">
+      <c r="L16" s="3">
         <v>5</v>
       </c>
       <c r="M16">
@@ -2897,29 +2283,29 @@
         <v>0</v>
       </c>
       <c r="O16"/>
-      <c r="P16" s="6">
+      <c r="P16" s="2">
         <v>6</v>
       </c>
       <c r="Q16">
         <v>4</v>
       </c>
-      <c r="R16" s="4">
+      <c r="R16" s="3">
         <v>5</v>
       </c>
-      <c r="S16" s="6">
+      <c r="S16" s="2">
         <v>18</v>
       </c>
       <c r="T16">
         <v>0.8</v>
       </c>
-      <c r="U16" s="4">
-        <v>1.1</v>
+      <c r="U16" s="3">
+        <v>1.1000000000000001</v>
       </c>
       <c r="X16"/>
       <c r="AA16"/>
       <c r="AC16"/>
       <c r="AE16"/>
-      <c r="AF16" s="7"/>
+      <c r="AF16" s="5"/>
     </row>
     <row r="17" spans="1:32">
       <c r="A17">
@@ -2944,10 +2330,10 @@
         <v>37</v>
       </c>
       <c r="J17"/>
-      <c r="K17" s="6">
-        <v>3</v>
-      </c>
-      <c r="L17" s="4">
+      <c r="K17" s="2">
+        <v>3</v>
+      </c>
+      <c r="L17" s="3">
         <v>3</v>
       </c>
       <c r="M17">
@@ -2957,37 +2343,37 @@
         <v>1</v>
       </c>
       <c r="O17"/>
-      <c r="P17" s="6">
+      <c r="P17" s="2">
         <v>19</v>
       </c>
       <c r="Q17">
         <v>1</v>
       </c>
-      <c r="R17" s="4">
-        <v>1</v>
-      </c>
-      <c r="S17" s="6">
+      <c r="R17" s="3">
+        <v>1</v>
+      </c>
+      <c r="S17" s="2">
         <v>2</v>
       </c>
       <c r="T17">
         <v>4</v>
       </c>
-      <c r="U17" s="4">
+      <c r="U17" s="3">
         <v>6</v>
       </c>
-      <c r="V17" s="6">
+      <c r="V17" s="2">
         <v>21</v>
       </c>
       <c r="W17">
         <v>2</v>
       </c>
-      <c r="X17" s="4">
+      <c r="X17" s="3">
         <v>3</v>
       </c>
       <c r="AA17"/>
       <c r="AC17"/>
       <c r="AE17"/>
-      <c r="AF17" s="8"/>
+      <c r="AF17" s="6"/>
     </row>
     <row r="18" spans="1:32">
       <c r="A18">
@@ -3014,7 +2400,7 @@
       <c r="K18">
         <v>4</v>
       </c>
-      <c r="L18" s="4">
+      <c r="L18" s="3">
         <v>3</v>
       </c>
       <c r="M18">
@@ -3023,22 +2409,22 @@
       <c r="N18">
         <v>0</v>
       </c>
-      <c r="P18" s="6">
+      <c r="P18" s="2">
         <v>15</v>
       </c>
       <c r="Q18">
         <v>5</v>
       </c>
-      <c r="R18" s="4">
+      <c r="R18" s="3">
         <v>7</v>
       </c>
       <c r="AB18">
         <v>61</v>
       </c>
-      <c r="AC18" s="4">
+      <c r="AC18" s="3">
         <v>1.5</v>
       </c>
-      <c r="AF18" s="7"/>
+      <c r="AF18" s="5"/>
     </row>
     <row r="19" spans="1:32">
       <c r="A19">
@@ -3063,10 +2449,10 @@
         <v>37</v>
       </c>
       <c r="J19"/>
-      <c r="K19" s="6">
+      <c r="K19" s="2">
         <v>5</v>
       </c>
-      <c r="L19" s="4">
+      <c r="L19" s="3">
         <v>4</v>
       </c>
       <c r="M19">
@@ -3076,29 +2462,29 @@
         <v>1</v>
       </c>
       <c r="O19"/>
-      <c r="P19" s="6">
+      <c r="P19" s="2">
         <v>23</v>
       </c>
       <c r="Q19">
         <v>1</v>
       </c>
-      <c r="R19" s="4">
-        <v>1</v>
-      </c>
-      <c r="S19" s="6">
+      <c r="R19" s="3">
+        <v>1</v>
+      </c>
+      <c r="S19" s="2">
         <v>7</v>
       </c>
       <c r="T19">
         <v>1</v>
       </c>
-      <c r="U19" s="4">
+      <c r="U19" s="3">
         <v>2</v>
       </c>
       <c r="X19"/>
       <c r="AA19"/>
       <c r="AC19"/>
       <c r="AE19"/>
-      <c r="AF19" s="7"/>
+      <c r="AF19" s="5"/>
     </row>
     <row r="20" spans="1:32">
       <c r="A20">
@@ -3125,7 +2511,7 @@
       <c r="K20">
         <v>6</v>
       </c>
-      <c r="L20" s="4">
+      <c r="L20" s="3">
         <v>6</v>
       </c>
       <c r="M20">
@@ -3134,25 +2520,25 @@
       <c r="N20">
         <v>0</v>
       </c>
-      <c r="O20" s="4">
-        <v>0</v>
-      </c>
-      <c r="P20" s="6">
+      <c r="O20" s="3">
+        <v>0</v>
+      </c>
+      <c r="P20" s="2">
         <v>11</v>
       </c>
       <c r="Q20">
         <v>24</v>
       </c>
-      <c r="R20" s="4">
+      <c r="R20" s="3">
         <v>30</v>
       </c>
       <c r="AB20">
         <v>62</v>
       </c>
-      <c r="AC20" s="4">
+      <c r="AC20" s="3">
         <v>7</v>
       </c>
-      <c r="AF20" s="8"/>
+      <c r="AF20" s="6"/>
     </row>
     <row r="21" spans="1:32">
       <c r="A21">
@@ -3179,7 +2565,7 @@
       <c r="K21">
         <v>5</v>
       </c>
-      <c r="L21" s="4">
+      <c r="L21" s="3">
         <v>4</v>
       </c>
       <c r="M21">
@@ -3188,22 +2574,22 @@
       <c r="N21">
         <v>1</v>
       </c>
-      <c r="P21" s="6">
+      <c r="P21" s="2">
         <v>26</v>
       </c>
       <c r="Q21">
         <v>2</v>
       </c>
-      <c r="R21" s="4">
-        <v>2</v>
-      </c>
-      <c r="S21" s="6">
+      <c r="R21" s="3">
+        <v>2</v>
+      </c>
+      <c r="S21" s="2">
         <v>11</v>
       </c>
       <c r="T21">
         <v>30</v>
       </c>
-      <c r="U21" s="4">
+      <c r="U21" s="3">
         <v>42</v>
       </c>
       <c r="V21">
@@ -3212,10 +2598,10 @@
       <c r="W21">
         <v>5</v>
       </c>
-      <c r="X21" s="4">
+      <c r="X21" s="3">
         <v>7</v>
       </c>
-      <c r="AF21" s="7"/>
+      <c r="AF21" s="5"/>
     </row>
     <row r="22" spans="1:32">
       <c r="A22">
@@ -3240,10 +2626,10 @@
         <v>37</v>
       </c>
       <c r="J22"/>
-      <c r="K22" s="6">
+      <c r="K22" s="2">
         <v>4</v>
       </c>
-      <c r="L22" s="4">
+      <c r="L22" s="3">
         <v>4</v>
       </c>
       <c r="M22">
@@ -3253,29 +2639,29 @@
         <v>1</v>
       </c>
       <c r="O22"/>
-      <c r="P22" s="6">
+      <c r="P22" s="2">
         <v>6</v>
       </c>
       <c r="Q22">
         <v>2</v>
       </c>
-      <c r="R22" s="4">
+      <c r="R22" s="3">
         <v>4</v>
       </c>
-      <c r="S22" s="6">
+      <c r="S22" s="2">
         <v>28</v>
       </c>
       <c r="T22">
         <v>1</v>
       </c>
-      <c r="U22" s="4">
+      <c r="U22" s="3">
         <v>1</v>
       </c>
       <c r="X22"/>
       <c r="AA22"/>
       <c r="AC22"/>
       <c r="AE22"/>
-      <c r="AF22" s="7"/>
+      <c r="AF22" s="5"/>
     </row>
     <row r="23" spans="1:32">
       <c r="A23">
@@ -3300,10 +2686,10 @@
         <v>37</v>
       </c>
       <c r="J23"/>
-      <c r="K23" s="6">
-        <v>1</v>
-      </c>
-      <c r="L23" s="4">
+      <c r="K23" s="2">
+        <v>1</v>
+      </c>
+      <c r="L23" s="3">
         <v>1</v>
       </c>
       <c r="M23">
@@ -3313,29 +2699,29 @@
         <v>0</v>
       </c>
       <c r="O23"/>
-      <c r="P23" s="6">
+      <c r="P23" s="2">
         <v>6</v>
       </c>
       <c r="Q23">
         <v>5</v>
       </c>
-      <c r="R23" s="4">
+      <c r="R23" s="3">
         <v>7</v>
       </c>
-      <c r="S23" s="6">
+      <c r="S23" s="2">
         <v>2</v>
       </c>
       <c r="T23">
         <v>1</v>
       </c>
-      <c r="U23" s="4">
+      <c r="U23" s="3">
         <v>1</v>
       </c>
       <c r="X23"/>
       <c r="AA23"/>
       <c r="AC23"/>
       <c r="AE23"/>
-      <c r="AF23" s="7"/>
+      <c r="AF23" s="5"/>
     </row>
     <row r="24" spans="1:32">
       <c r="A24">
@@ -3362,7 +2748,7 @@
       <c r="K24">
         <v>4</v>
       </c>
-      <c r="L24" s="4">
+      <c r="L24" s="3">
         <v>4</v>
       </c>
       <c r="M24">
@@ -3371,31 +2757,31 @@
       <c r="N24">
         <v>0</v>
       </c>
-      <c r="P24" s="6">
+      <c r="P24" s="2">
         <v>15</v>
       </c>
       <c r="Q24">
         <v>3</v>
       </c>
-      <c r="R24" s="4">
+      <c r="R24" s="3">
         <v>4</v>
       </c>
-      <c r="S24" s="6">
+      <c r="S24" s="2">
         <v>11</v>
       </c>
       <c r="T24">
         <v>8</v>
       </c>
-      <c r="U24" s="4">
+      <c r="U24" s="3">
         <v>11</v>
       </c>
       <c r="AB24">
         <v>63</v>
       </c>
-      <c r="AC24" s="4">
-        <v>3</v>
-      </c>
-      <c r="AF24" s="7"/>
+      <c r="AC24" s="3">
+        <v>3</v>
+      </c>
+      <c r="AF24" s="5"/>
     </row>
     <row r="25" spans="1:32">
       <c r="A25">
@@ -3420,10 +2806,10 @@
         <v>37</v>
       </c>
       <c r="J25"/>
-      <c r="K25" s="6">
-        <v>3</v>
-      </c>
-      <c r="L25" s="4">
+      <c r="K25" s="2">
+        <v>3</v>
+      </c>
+      <c r="L25" s="3">
         <v>2</v>
       </c>
       <c r="M25">
@@ -3433,13 +2819,13 @@
         <v>0</v>
       </c>
       <c r="O25"/>
-      <c r="P25" s="6">
+      <c r="P25" s="2">
         <v>7</v>
       </c>
       <c r="Q25">
         <v>3</v>
       </c>
-      <c r="R25" s="4">
+      <c r="R25" s="3">
         <v>5</v>
       </c>
       <c r="U25"/>
@@ -3447,7 +2833,7 @@
       <c r="AA25"/>
       <c r="AC25"/>
       <c r="AE25"/>
-      <c r="AF25" s="7"/>
+      <c r="AF25" s="5"/>
     </row>
     <row r="26" spans="1:32">
       <c r="A26">
@@ -3472,10 +2858,10 @@
         <v>37</v>
       </c>
       <c r="J26"/>
-      <c r="K26" s="6">
-        <v>3</v>
-      </c>
-      <c r="L26" s="4">
+      <c r="K26" s="2">
+        <v>3</v>
+      </c>
+      <c r="L26" s="3">
         <v>2</v>
       </c>
       <c r="M26">
@@ -3485,29 +2871,29 @@
         <v>0</v>
       </c>
       <c r="O26"/>
-      <c r="P26" s="6">
+      <c r="P26" s="2">
         <v>7</v>
       </c>
       <c r="Q26">
         <v>3</v>
       </c>
-      <c r="R26" s="4">
+      <c r="R26" s="3">
         <v>4</v>
       </c>
-      <c r="S26" s="6">
+      <c r="S26" s="2">
         <v>2</v>
       </c>
       <c r="T26">
         <v>4</v>
       </c>
-      <c r="U26" s="4">
+      <c r="U26" s="3">
         <v>6</v>
       </c>
       <c r="X26"/>
       <c r="AA26"/>
       <c r="AC26"/>
       <c r="AE26"/>
-      <c r="AF26" s="7"/>
+      <c r="AF26" s="5"/>
     </row>
     <row r="27" spans="1:32">
       <c r="A27">
@@ -3534,7 +2920,7 @@
       <c r="K27">
         <v>8</v>
       </c>
-      <c r="L27" s="4">
+      <c r="L27" s="3">
         <v>6</v>
       </c>
       <c r="M27">
@@ -3543,25 +2929,25 @@
       <c r="N27">
         <v>1</v>
       </c>
-      <c r="O27" s="4">
-        <v>0</v>
-      </c>
-      <c r="P27" s="6">
+      <c r="O27" s="3">
+        <v>0</v>
+      </c>
+      <c r="P27" s="2">
         <v>11</v>
       </c>
       <c r="Q27">
         <v>12</v>
       </c>
-      <c r="R27" s="4">
+      <c r="R27" s="3">
         <v>18</v>
       </c>
-      <c r="S27" s="6">
+      <c r="S27" s="2">
         <v>56</v>
       </c>
       <c r="T27">
         <v>24</v>
       </c>
-      <c r="U27" s="4">
+      <c r="U27" s="3">
         <v>30</v>
       </c>
       <c r="V27">
@@ -3570,10 +2956,10 @@
       <c r="W27">
         <v>36</v>
       </c>
-      <c r="X27" s="4">
+      <c r="X27" s="3">
         <v>44</v>
       </c>
-      <c r="AF27" s="8"/>
+      <c r="AF27" s="6"/>
     </row>
     <row r="28" spans="1:32">
       <c r="A28">
@@ -3600,7 +2986,7 @@
       <c r="K28">
         <v>1</v>
       </c>
-      <c r="L28" s="4">
+      <c r="L28" s="3">
         <v>0</v>
       </c>
       <c r="M28">
@@ -3609,22 +2995,22 @@
       <c r="N28">
         <v>0</v>
       </c>
-      <c r="P28" s="6">
+      <c r="P28" s="2">
         <v>2</v>
       </c>
       <c r="Q28">
         <v>6</v>
       </c>
-      <c r="R28" s="4">
+      <c r="R28" s="3">
         <v>8</v>
       </c>
       <c r="AB28">
         <v>21</v>
       </c>
-      <c r="AC28" s="4">
+      <c r="AC28" s="3">
         <v>12</v>
       </c>
-      <c r="AF28" s="7"/>
+      <c r="AF28" s="5"/>
     </row>
     <row r="29" spans="1:32">
       <c r="A29">
@@ -3649,10 +3035,10 @@
         <v>37</v>
       </c>
       <c r="J29"/>
-      <c r="K29" s="6">
+      <c r="K29" s="2">
         <v>5</v>
       </c>
-      <c r="L29" s="4">
+      <c r="L29" s="3">
         <v>5</v>
       </c>
       <c r="M29">
@@ -3662,37 +3048,37 @@
         <v>1</v>
       </c>
       <c r="O29"/>
-      <c r="P29" s="6">
+      <c r="P29" s="2">
         <v>32</v>
       </c>
       <c r="Q29">
         <v>30</v>
       </c>
-      <c r="R29" s="4">
+      <c r="R29" s="3">
         <v>30</v>
       </c>
-      <c r="S29" s="6">
+      <c r="S29" s="2">
         <v>2</v>
       </c>
       <c r="T29">
         <v>3</v>
       </c>
-      <c r="U29" s="4">
+      <c r="U29" s="3">
         <v>5</v>
       </c>
-      <c r="V29" s="6">
+      <c r="V29" s="2">
         <v>21</v>
       </c>
       <c r="W29">
         <v>2</v>
       </c>
-      <c r="X29" s="4">
+      <c r="X29" s="3">
         <v>3</v>
       </c>
       <c r="AA29"/>
       <c r="AC29"/>
       <c r="AE29"/>
-      <c r="AF29" s="7"/>
+      <c r="AF29" s="5"/>
     </row>
     <row r="30" spans="1:32">
       <c r="A30">
@@ -3717,10 +3103,10 @@
         <v>37</v>
       </c>
       <c r="J30"/>
-      <c r="K30" s="6">
+      <c r="K30" s="2">
         <v>4</v>
       </c>
-      <c r="L30" s="4">
+      <c r="L30" s="3">
         <v>4</v>
       </c>
       <c r="M30">
@@ -3730,29 +3116,29 @@
         <v>1</v>
       </c>
       <c r="O30"/>
-      <c r="P30" s="6">
+      <c r="P30" s="2">
         <v>33</v>
       </c>
       <c r="Q30">
         <v>50</v>
       </c>
-      <c r="R30" s="4">
+      <c r="R30" s="3">
         <v>70</v>
       </c>
-      <c r="S30" s="6">
+      <c r="S30" s="2">
         <v>2</v>
       </c>
       <c r="T30">
         <v>2</v>
       </c>
-      <c r="U30" s="4">
+      <c r="U30" s="3">
         <v>4</v>
       </c>
       <c r="X30"/>
       <c r="AA30"/>
       <c r="AC30"/>
       <c r="AE30"/>
-      <c r="AF30" s="8"/>
+      <c r="AF30" s="6"/>
     </row>
     <row r="31" spans="1:32">
       <c r="A31">
@@ -3777,10 +3163,10 @@
         <v>37</v>
       </c>
       <c r="J31"/>
-      <c r="K31" s="6">
+      <c r="K31" s="2">
         <v>4</v>
       </c>
-      <c r="L31" s="4">
+      <c r="L31" s="3">
         <v>3</v>
       </c>
       <c r="M31">
@@ -3790,31 +3176,31 @@
         <v>1</v>
       </c>
       <c r="O31"/>
-      <c r="P31" s="6">
+      <c r="P31" s="2">
         <v>33</v>
       </c>
       <c r="Q31">
         <v>20</v>
       </c>
-      <c r="R31" s="4">
+      <c r="R31" s="3">
         <v>30</v>
       </c>
-      <c r="S31" s="6">
+      <c r="S31" s="2">
         <v>35</v>
       </c>
       <c r="T31">
         <v>1</v>
       </c>
-      <c r="U31" s="4">
+      <c r="U31" s="3">
         <v>1</v>
       </c>
       <c r="X31"/>
       <c r="AA31"/>
       <c r="AC31"/>
       <c r="AE31"/>
-      <c r="AF31" s="8"/>
-    </row>
-    <row r="32" spans="1:31">
+      <c r="AF31" s="6"/>
+    </row>
+    <row r="32" spans="1:32">
       <c r="A32">
         <v>33</v>
       </c>
@@ -3837,10 +3223,10 @@
         <v>37</v>
       </c>
       <c r="J32"/>
-      <c r="K32" s="6">
+      <c r="K32" s="2">
         <v>7</v>
       </c>
-      <c r="L32" s="4">
+      <c r="L32" s="3">
         <v>6</v>
       </c>
       <c r="M32">
@@ -3857,7 +3243,7 @@
       <c r="AC32"/>
       <c r="AE32"/>
     </row>
-    <row r="33" spans="1:29">
+    <row r="33" spans="1:31">
       <c r="A33">
         <v>34</v>
       </c>
@@ -3882,7 +3268,7 @@
       <c r="K33">
         <v>8</v>
       </c>
-      <c r="L33" s="4">
+      <c r="L33" s="3">
         <v>7</v>
       </c>
       <c r="M33">
@@ -3891,23 +3277,23 @@
       <c r="N33">
         <v>1</v>
       </c>
-      <c r="P33" s="6">
+      <c r="P33" s="2">
         <v>11</v>
       </c>
       <c r="Q33">
         <v>38</v>
       </c>
-      <c r="R33" s="4">
+      <c r="R33" s="3">
         <v>52</v>
       </c>
       <c r="AB33">
         <v>64</v>
       </c>
-      <c r="AC33" s="4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34" spans="1:18">
+      <c r="AC33" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:31">
       <c r="A34">
         <v>35</v>
       </c>
@@ -3932,7 +3318,7 @@
       <c r="K34">
         <v>3</v>
       </c>
-      <c r="L34" s="4">
+      <c r="L34" s="3">
         <v>3</v>
       </c>
       <c r="M34">
@@ -3941,20 +3327,20 @@
       <c r="N34">
         <v>0</v>
       </c>
-      <c r="O34" s="4">
-        <v>0</v>
-      </c>
-      <c r="P34" s="6">
+      <c r="O34" s="3">
+        <v>0</v>
+      </c>
+      <c r="P34" s="2">
         <v>15</v>
       </c>
       <c r="Q34">
         <v>3</v>
       </c>
-      <c r="R34" s="4">
+      <c r="R34" s="3">
         <v>4</v>
       </c>
     </row>
-    <row r="35" spans="1:18">
+    <row r="35" spans="1:31">
       <c r="A35">
         <v>36</v>
       </c>
@@ -3979,7 +3365,7 @@
       <c r="K35">
         <v>3</v>
       </c>
-      <c r="L35" s="4">
+      <c r="L35" s="3">
         <v>3</v>
       </c>
       <c r="M35">
@@ -3988,21 +3374,21 @@
       <c r="N35">
         <v>0</v>
       </c>
-      <c r="P35" s="6">
+      <c r="P35" s="2">
         <v>11</v>
       </c>
       <c r="Q35">
         <v>18</v>
       </c>
-      <c r="R35" s="4">
+      <c r="R35" s="3">
         <v>22</v>
       </c>
     </row>
-    <row r="36" spans="1:21">
+    <row r="36" spans="1:31">
       <c r="A36">
         <v>37</v>
       </c>
-      <c r="B36" s="5">
+      <c r="B36" s="4">
         <v>144</v>
       </c>
       <c r="C36" t="s">
@@ -4023,7 +3409,7 @@
       <c r="K36">
         <v>3</v>
       </c>
-      <c r="L36" s="4">
+      <c r="L36" s="3">
         <v>3</v>
       </c>
       <c r="M36">
@@ -4032,22 +3418,22 @@
       <c r="N36">
         <v>0</v>
       </c>
-      <c r="P36" s="6">
+      <c r="P36" s="2">
         <v>15</v>
       </c>
       <c r="Q36">
         <v>3</v>
       </c>
-      <c r="R36" s="4">
+      <c r="R36" s="3">
         <v>4</v>
       </c>
-      <c r="S36" s="6">
+      <c r="S36" s="2">
         <v>2</v>
       </c>
       <c r="T36">
         <v>6</v>
       </c>
-      <c r="U36" s="4">
+      <c r="U36" s="3">
         <v>8</v>
       </c>
     </row>
@@ -4074,10 +3460,10 @@
         <v>37</v>
       </c>
       <c r="J37"/>
-      <c r="K37" s="6">
-        <v>3</v>
-      </c>
-      <c r="L37" s="4">
+      <c r="K37" s="2">
+        <v>3</v>
+      </c>
+      <c r="L37" s="3">
         <v>3</v>
       </c>
       <c r="M37">
@@ -4087,22 +3473,22 @@
         <v>0</v>
       </c>
       <c r="O37"/>
-      <c r="P37" s="6">
+      <c r="P37" s="2">
         <v>7</v>
       </c>
       <c r="Q37">
         <v>3</v>
       </c>
-      <c r="R37" s="4">
+      <c r="R37" s="3">
         <v>4</v>
       </c>
-      <c r="S37" s="6">
+      <c r="S37" s="2">
         <v>2</v>
       </c>
       <c r="T37">
         <v>6</v>
       </c>
-      <c r="U37" s="4">
+      <c r="U37" s="3">
         <v>8</v>
       </c>
       <c r="X37"/>
@@ -4133,10 +3519,10 @@
         <v>37</v>
       </c>
       <c r="J38"/>
-      <c r="K38" s="6">
-        <v>1</v>
-      </c>
-      <c r="L38" s="4">
+      <c r="K38" s="2">
+        <v>1</v>
+      </c>
+      <c r="L38" s="3">
         <v>1</v>
       </c>
       <c r="M38">
@@ -4146,22 +3532,22 @@
         <v>1</v>
       </c>
       <c r="O38"/>
-      <c r="P38" s="6">
+      <c r="P38" s="2">
         <v>21</v>
       </c>
       <c r="Q38">
         <v>4</v>
       </c>
-      <c r="R38" s="4">
+      <c r="R38" s="3">
         <v>5</v>
       </c>
-      <c r="S38" s="6">
+      <c r="S38" s="2">
         <v>2</v>
       </c>
       <c r="T38">
         <v>3</v>
       </c>
-      <c r="U38" s="4">
+      <c r="U38" s="3">
         <v>5</v>
       </c>
       <c r="X38"/>
@@ -4192,10 +3578,10 @@
         <v>37</v>
       </c>
       <c r="J39"/>
-      <c r="K39" s="6">
-        <v>1</v>
-      </c>
-      <c r="L39" s="4">
+      <c r="K39" s="2">
+        <v>1</v>
+      </c>
+      <c r="L39" s="3">
         <v>1</v>
       </c>
       <c r="M39">
@@ -4205,22 +3591,22 @@
         <v>1</v>
       </c>
       <c r="O39"/>
-      <c r="P39" s="6">
+      <c r="P39" s="2">
         <v>5</v>
       </c>
       <c r="Q39">
         <v>1</v>
       </c>
-      <c r="R39" s="4">
-        <v>2</v>
-      </c>
-      <c r="S39" s="6">
+      <c r="R39" s="3">
+        <v>2</v>
+      </c>
+      <c r="S39" s="2">
         <v>2</v>
       </c>
       <c r="T39">
         <v>6</v>
       </c>
-      <c r="U39" s="4">
+      <c r="U39" s="3">
         <v>7</v>
       </c>
       <c r="X39"/>
@@ -4251,10 +3637,10 @@
         <v>37</v>
       </c>
       <c r="J40"/>
-      <c r="K40" s="6">
+      <c r="K40" s="2">
         <v>4</v>
       </c>
-      <c r="L40" s="4">
+      <c r="L40" s="3">
         <v>3</v>
       </c>
       <c r="M40">
@@ -4264,22 +3650,22 @@
         <v>1</v>
       </c>
       <c r="O40"/>
-      <c r="P40" s="6">
+      <c r="P40" s="2">
         <v>7</v>
       </c>
       <c r="Q40">
         <v>4</v>
       </c>
-      <c r="R40" s="4">
+      <c r="R40" s="3">
         <v>5</v>
       </c>
-      <c r="S40" s="6">
+      <c r="S40" s="2">
         <v>38</v>
       </c>
       <c r="T40">
         <v>4</v>
       </c>
-      <c r="U40" s="4">
+      <c r="U40" s="3">
         <v>5</v>
       </c>
       <c r="X40"/>
@@ -4310,10 +3696,10 @@
         <v>37</v>
       </c>
       <c r="J41"/>
-      <c r="K41" s="6">
-        <v>2</v>
-      </c>
-      <c r="L41" s="4">
+      <c r="K41" s="2">
+        <v>2</v>
+      </c>
+      <c r="L41" s="3">
         <v>2</v>
       </c>
       <c r="M41">
@@ -4323,22 +3709,22 @@
         <v>0</v>
       </c>
       <c r="O41"/>
-      <c r="P41" s="6">
+      <c r="P41" s="2">
         <v>6</v>
       </c>
       <c r="Q41">
         <v>3</v>
       </c>
-      <c r="R41" s="4">
-        <v>3</v>
-      </c>
-      <c r="S41" s="6">
+      <c r="R41" s="3">
+        <v>3</v>
+      </c>
+      <c r="S41" s="2">
         <v>39</v>
       </c>
       <c r="T41">
         <v>2</v>
       </c>
-      <c r="U41" s="4">
+      <c r="U41" s="3">
         <v>3</v>
       </c>
       <c r="X41"/>
@@ -4369,10 +3755,10 @@
         <v>37</v>
       </c>
       <c r="J42"/>
-      <c r="K42" s="6">
+      <c r="K42" s="2">
         <v>4</v>
       </c>
-      <c r="L42" s="4">
+      <c r="L42" s="3">
         <v>3</v>
       </c>
       <c r="M42">
@@ -4382,22 +3768,22 @@
         <v>1</v>
       </c>
       <c r="O42"/>
-      <c r="P42" s="6">
+      <c r="P42" s="2">
         <v>7</v>
       </c>
       <c r="Q42">
         <v>1</v>
       </c>
-      <c r="R42" s="4">
-        <v>3</v>
-      </c>
-      <c r="S42" s="6">
+      <c r="R42" s="3">
+        <v>3</v>
+      </c>
+      <c r="S42" s="2">
         <v>41</v>
       </c>
       <c r="T42">
         <v>1</v>
       </c>
-      <c r="U42" s="4">
+      <c r="U42" s="3">
         <v>1</v>
       </c>
       <c r="X42"/>
@@ -4428,10 +3814,10 @@
         <v>37</v>
       </c>
       <c r="J43"/>
-      <c r="K43" s="6">
+      <c r="K43" s="2">
         <v>7</v>
       </c>
-      <c r="L43" s="4">
+      <c r="L43" s="3">
         <v>4</v>
       </c>
       <c r="M43">
@@ -4441,38 +3827,38 @@
         <v>1</v>
       </c>
       <c r="O43"/>
-      <c r="P43" s="6">
+      <c r="P43" s="2">
         <v>6</v>
       </c>
       <c r="Q43">
         <v>5</v>
       </c>
-      <c r="R43" s="4">
+      <c r="R43" s="3">
         <v>5</v>
       </c>
-      <c r="S43" s="6">
+      <c r="S43" s="2">
         <v>14</v>
       </c>
       <c r="T43">
         <v>1</v>
       </c>
-      <c r="U43" s="4">
-        <v>1</v>
-      </c>
-      <c r="V43" s="6">
+      <c r="U43" s="3">
+        <v>1</v>
+      </c>
+      <c r="V43" s="2">
         <v>18</v>
       </c>
       <c r="W43">
         <v>0.9</v>
       </c>
-      <c r="X43" s="4">
+      <c r="X43" s="3">
         <v>1.2</v>
       </c>
       <c r="AA43"/>
       <c r="AC43"/>
       <c r="AE43"/>
     </row>
-    <row r="44" spans="1:21">
+    <row r="44" spans="1:31">
       <c r="A44">
         <v>45</v>
       </c>
@@ -4497,7 +3883,7 @@
       <c r="K44">
         <v>6</v>
       </c>
-      <c r="L44" s="4">
+      <c r="L44" s="3">
         <v>4</v>
       </c>
       <c r="M44">
@@ -4506,22 +3892,22 @@
       <c r="N44">
         <v>1</v>
       </c>
-      <c r="P44" s="6">
+      <c r="P44" s="2">
         <v>15</v>
       </c>
       <c r="Q44">
         <v>2</v>
       </c>
-      <c r="R44" s="4">
-        <v>2</v>
-      </c>
-      <c r="S44" s="6">
+      <c r="R44" s="3">
+        <v>2</v>
+      </c>
+      <c r="S44" s="2">
         <v>42</v>
       </c>
       <c r="T44">
         <v>8</v>
       </c>
-      <c r="U44" s="4">
+      <c r="U44" s="3">
         <v>12</v>
       </c>
     </row>
@@ -4548,10 +3934,10 @@
         <v>37</v>
       </c>
       <c r="J45"/>
-      <c r="K45" s="6">
+      <c r="K45" s="2">
         <v>5</v>
       </c>
-      <c r="L45" s="4">
+      <c r="L45" s="3">
         <v>4</v>
       </c>
       <c r="M45">
@@ -4561,31 +3947,31 @@
         <v>1</v>
       </c>
       <c r="O45"/>
-      <c r="P45" s="6">
+      <c r="P45" s="2">
         <v>7</v>
       </c>
       <c r="Q45">
         <v>7</v>
       </c>
-      <c r="R45" s="4">
+      <c r="R45" s="3">
         <v>9</v>
       </c>
-      <c r="S45" s="6">
+      <c r="S45" s="2">
         <v>26</v>
       </c>
       <c r="T45">
         <v>2</v>
       </c>
-      <c r="U45" s="4">
-        <v>2</v>
-      </c>
-      <c r="V45" s="6">
+      <c r="U45" s="3">
+        <v>2</v>
+      </c>
+      <c r="V45" s="2">
         <v>2</v>
       </c>
       <c r="W45">
         <v>7</v>
       </c>
-      <c r="X45" s="4">
+      <c r="X45" s="3">
         <v>8</v>
       </c>
       <c r="AA45"/>
@@ -4615,10 +4001,10 @@
         <v>37</v>
       </c>
       <c r="J46"/>
-      <c r="K46" s="6">
+      <c r="K46" s="2">
         <v>10</v>
       </c>
-      <c r="L46" s="4">
+      <c r="L46" s="3">
         <v>6</v>
       </c>
       <c r="M46">
@@ -4628,31 +4014,31 @@
         <v>1</v>
       </c>
       <c r="O46"/>
-      <c r="P46" s="6">
+      <c r="P46" s="2">
         <v>32</v>
       </c>
       <c r="Q46">
         <v>40</v>
       </c>
-      <c r="R46" s="4">
+      <c r="R46" s="3">
         <v>40</v>
       </c>
-      <c r="S46" s="6">
+      <c r="S46" s="2">
         <v>33</v>
       </c>
       <c r="T46">
         <v>30</v>
       </c>
-      <c r="U46" s="4">
+      <c r="U46" s="3">
         <v>30</v>
       </c>
-      <c r="V46" s="6">
+      <c r="V46" s="2">
         <v>19</v>
       </c>
       <c r="W46">
         <v>1</v>
       </c>
-      <c r="X46" s="4">
+      <c r="X46" s="3">
         <v>1</v>
       </c>
       <c r="AA46"/>
@@ -4682,10 +4068,10 @@
         <v>37</v>
       </c>
       <c r="J47"/>
-      <c r="K47" s="6">
-        <v>2</v>
-      </c>
-      <c r="L47" s="4">
+      <c r="K47" s="2">
+        <v>2</v>
+      </c>
+      <c r="L47" s="3">
         <v>1</v>
       </c>
       <c r="M47">
@@ -4695,13 +4081,13 @@
         <v>0</v>
       </c>
       <c r="O47"/>
-      <c r="P47" s="6">
+      <c r="P47" s="2">
         <v>11</v>
       </c>
       <c r="Q47">
         <v>10</v>
       </c>
-      <c r="R47" s="4">
+      <c r="R47" s="3">
         <v>14</v>
       </c>
       <c r="U47"/>
@@ -4733,10 +4119,10 @@
         <v>37</v>
       </c>
       <c r="J48"/>
-      <c r="K48" s="6">
+      <c r="K48" s="2">
         <v>4</v>
       </c>
-      <c r="L48" s="4">
+      <c r="L48" s="3">
         <v>3</v>
       </c>
       <c r="M48">
@@ -4746,22 +4132,22 @@
         <v>0</v>
       </c>
       <c r="O48"/>
-      <c r="P48" s="6">
+      <c r="P48" s="2">
         <v>11</v>
       </c>
       <c r="Q48">
         <v>8</v>
       </c>
-      <c r="R48" s="4">
+      <c r="R48" s="3">
         <v>11</v>
       </c>
-      <c r="S48" s="6">
+      <c r="S48" s="2">
         <v>6</v>
       </c>
       <c r="T48">
         <v>3</v>
       </c>
-      <c r="U48" s="4">
+      <c r="U48" s="3">
         <v>3</v>
       </c>
       <c r="X48"/>
@@ -4769,7 +4155,7 @@
       <c r="AC48"/>
       <c r="AE48"/>
     </row>
-    <row r="49" spans="1:21">
+    <row r="49" spans="1:31">
       <c r="A49">
         <v>50</v>
       </c>
@@ -4794,7 +4180,7 @@
       <c r="K49">
         <v>4</v>
       </c>
-      <c r="L49" s="4">
+      <c r="L49" s="3">
         <v>3</v>
       </c>
       <c r="M49">
@@ -4803,22 +4189,22 @@
       <c r="N49">
         <v>0</v>
       </c>
-      <c r="P49" s="6">
+      <c r="P49" s="2">
         <v>11</v>
       </c>
       <c r="Q49">
         <v>7</v>
       </c>
-      <c r="R49" s="4">
+      <c r="R49" s="3">
         <v>11</v>
       </c>
-      <c r="S49" s="6">
+      <c r="S49" s="2">
         <v>45</v>
       </c>
       <c r="T49">
         <v>2</v>
       </c>
-      <c r="U49" s="4">
+      <c r="U49" s="3">
         <v>3</v>
       </c>
     </row>
@@ -4845,10 +4231,10 @@
         <v>37</v>
       </c>
       <c r="J50"/>
-      <c r="K50" s="6">
+      <c r="K50" s="2">
         <v>5</v>
       </c>
-      <c r="L50" s="4">
+      <c r="L50" s="3">
         <v>4</v>
       </c>
       <c r="M50">
@@ -4858,22 +4244,22 @@
         <v>1</v>
       </c>
       <c r="O50"/>
-      <c r="P50" s="6">
+      <c r="P50" s="2">
         <v>6</v>
       </c>
       <c r="Q50">
         <v>5</v>
       </c>
-      <c r="R50" s="4">
+      <c r="R50" s="3">
         <v>7</v>
       </c>
-      <c r="S50" s="6">
+      <c r="S50" s="2">
         <v>18</v>
       </c>
       <c r="T50">
-        <v>1.1</v>
-      </c>
-      <c r="U50" s="4">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="U50" s="3">
         <v>1.7</v>
       </c>
       <c r="X50"/>
@@ -4904,10 +4290,10 @@
         <v>37</v>
       </c>
       <c r="J51"/>
-      <c r="K51" s="6">
+      <c r="K51" s="2">
         <v>9</v>
       </c>
-      <c r="L51" s="4">
+      <c r="L51" s="3">
         <v>6</v>
       </c>
       <c r="M51">
@@ -4917,22 +4303,22 @@
         <v>1</v>
       </c>
       <c r="O51"/>
-      <c r="P51" s="6">
+      <c r="P51" s="2">
         <v>6</v>
       </c>
       <c r="Q51">
         <v>1</v>
       </c>
-      <c r="R51" s="4">
-        <v>3</v>
-      </c>
-      <c r="S51" s="6">
+      <c r="R51" s="3">
+        <v>3</v>
+      </c>
+      <c r="S51" s="2">
         <v>49</v>
       </c>
       <c r="T51">
         <v>1</v>
       </c>
-      <c r="U51" s="4">
+      <c r="U51" s="3">
         <v>1</v>
       </c>
       <c r="X51"/>
@@ -4963,10 +4349,10 @@
         <v>37</v>
       </c>
       <c r="J52"/>
-      <c r="K52" s="6">
-        <v>1</v>
-      </c>
-      <c r="L52" s="4">
+      <c r="K52" s="2">
+        <v>1</v>
+      </c>
+      <c r="L52" s="3">
         <v>0</v>
       </c>
       <c r="M52">
@@ -4976,22 +4362,22 @@
         <v>1</v>
       </c>
       <c r="O52"/>
-      <c r="P52" s="6">
+      <c r="P52" s="2">
         <v>9</v>
       </c>
       <c r="Q52">
         <v>2</v>
       </c>
-      <c r="R52" s="4">
-        <v>2</v>
-      </c>
-      <c r="S52" s="6">
+      <c r="R52" s="3">
+        <v>2</v>
+      </c>
+      <c r="S52" s="2">
         <v>21</v>
       </c>
       <c r="T52">
         <v>2</v>
       </c>
-      <c r="U52" s="4">
+      <c r="U52" s="3">
         <v>2</v>
       </c>
       <c r="X52"/>
@@ -4999,7 +4385,7 @@
       <c r="AC52"/>
       <c r="AE52"/>
     </row>
-    <row r="53" spans="1:21">
+    <row r="53" spans="1:31">
       <c r="A53">
         <v>54</v>
       </c>
@@ -5024,7 +4410,7 @@
       <c r="K53">
         <v>5</v>
       </c>
-      <c r="L53" s="4">
+      <c r="L53" s="3">
         <v>5</v>
       </c>
       <c r="M53">
@@ -5033,7 +4419,7 @@
       <c r="N53">
         <v>1</v>
       </c>
-      <c r="O53" s="4">
+      <c r="O53" s="3">
         <v>6</v>
       </c>
       <c r="P53">
@@ -5042,7 +4428,7 @@
       <c r="Q53">
         <v>3</v>
       </c>
-      <c r="R53" s="4">
+      <c r="R53" s="3">
         <v>4</v>
       </c>
       <c r="S53">
@@ -5051,11 +4437,11 @@
       <c r="T53">
         <v>-0.5</v>
       </c>
-      <c r="U53" s="4">
+      <c r="U53" s="3">
         <v>-0.5</v>
       </c>
     </row>
-    <row r="54" spans="1:24">
+    <row r="54" spans="1:31">
       <c r="A54">
         <v>55</v>
       </c>
@@ -5077,13 +4463,13 @@
       <c r="I54" t="s">
         <v>49</v>
       </c>
-      <c r="J54" s="4">
+      <c r="J54" s="3">
         <v>14</v>
       </c>
       <c r="K54">
         <v>2</v>
       </c>
-      <c r="L54" s="4">
+      <c r="L54" s="3">
         <v>1</v>
       </c>
       <c r="M54">
@@ -5098,7 +4484,7 @@
       <c r="Q54">
         <v>3</v>
       </c>
-      <c r="R54" s="4">
+      <c r="R54" s="3">
         <v>4</v>
       </c>
       <c r="S54">
@@ -5107,7 +4493,7 @@
       <c r="T54">
         <v>1</v>
       </c>
-      <c r="U54" s="4">
+      <c r="U54" s="3">
         <v>1</v>
       </c>
       <c r="V54">
@@ -5116,11 +4502,11 @@
       <c r="W54">
         <v>3</v>
       </c>
-      <c r="X54" s="4">
+      <c r="X54" s="3">
         <v>5</v>
       </c>
     </row>
-    <row r="55" spans="1:30">
+    <row r="55" spans="1:31">
       <c r="A55">
         <v>56</v>
       </c>
@@ -5145,7 +4531,7 @@
       <c r="K55">
         <v>4</v>
       </c>
-      <c r="L55" s="4">
+      <c r="L55" s="3">
         <v>3</v>
       </c>
       <c r="M55">
@@ -5160,7 +4546,7 @@
       <c r="Q55">
         <v>1</v>
       </c>
-      <c r="R55" s="4">
+      <c r="R55" s="3">
         <v>3</v>
       </c>
       <c r="S55">
@@ -5169,12 +4555,12 @@
       <c r="T55">
         <v>1</v>
       </c>
-      <c r="U55" s="4">
-        <v>1</v>
-      </c>
-      <c r="AD55" s="4"/>
-    </row>
-    <row r="56" spans="1:30">
+      <c r="U55" s="3">
+        <v>1</v>
+      </c>
+      <c r="AD55" s="3"/>
+    </row>
+    <row r="56" spans="1:31">
       <c r="A56">
         <v>57</v>
       </c>
@@ -5196,13 +4582,13 @@
       <c r="I56" t="s">
         <v>49</v>
       </c>
-      <c r="J56" s="4">
+      <c r="J56" s="3">
         <v>3</v>
       </c>
       <c r="K56">
         <v>2</v>
       </c>
-      <c r="L56" s="4">
+      <c r="L56" s="3">
         <v>1</v>
       </c>
       <c r="M56">
@@ -5217,7 +4603,7 @@
       <c r="Q56">
         <v>3</v>
       </c>
-      <c r="R56" s="4">
+      <c r="R56" s="3">
         <v>4</v>
       </c>
       <c r="S56">
@@ -5226,7 +4612,7 @@
       <c r="T56">
         <v>12</v>
       </c>
-      <c r="U56" s="4">
+      <c r="U56" s="3">
         <v>18</v>
       </c>
       <c r="V56">
@@ -5235,12 +4621,12 @@
       <c r="W56">
         <v>1</v>
       </c>
-      <c r="X56" s="4">
-        <v>1</v>
-      </c>
-      <c r="AD56" s="4"/>
-    </row>
-    <row r="57" spans="1:21">
+      <c r="X56" s="3">
+        <v>1</v>
+      </c>
+      <c r="AD56" s="3"/>
+    </row>
+    <row r="57" spans="1:31">
       <c r="A57">
         <v>58</v>
       </c>
@@ -5262,13 +4648,13 @@
       <c r="I57" t="s">
         <v>49</v>
       </c>
-      <c r="J57" s="4">
+      <c r="J57" s="3">
         <v>3</v>
       </c>
       <c r="K57">
         <v>2</v>
       </c>
-      <c r="L57" s="4">
+      <c r="L57" s="3">
         <v>1</v>
       </c>
       <c r="M57">
@@ -5283,7 +4669,7 @@
       <c r="Q57">
         <v>5</v>
       </c>
-      <c r="R57" s="4">
+      <c r="R57" s="3">
         <v>6</v>
       </c>
       <c r="S57">
@@ -5292,11 +4678,11 @@
       <c r="T57">
         <v>5</v>
       </c>
-      <c r="U57" s="4">
+      <c r="U57" s="3">
         <v>6</v>
       </c>
     </row>
-    <row r="58" spans="1:14">
+    <row r="58" spans="1:31">
       <c r="A58">
         <v>59</v>
       </c>
@@ -5321,7 +4707,7 @@
       <c r="K58">
         <v>3</v>
       </c>
-      <c r="L58" s="4">
+      <c r="L58" s="3">
         <v>2</v>
       </c>
       <c r="M58">
@@ -5331,7 +4717,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:18">
+    <row r="59" spans="1:31">
       <c r="A59">
         <v>60</v>
       </c>
@@ -5356,7 +4742,7 @@
       <c r="K59">
         <v>4</v>
       </c>
-      <c r="L59" s="4">
+      <c r="L59" s="3">
         <v>3</v>
       </c>
       <c r="M59">
@@ -5371,11 +4757,11 @@
       <c r="Q59">
         <v>7</v>
       </c>
-      <c r="R59" s="4">
+      <c r="R59" s="3">
         <v>9</v>
       </c>
     </row>
-    <row r="60" spans="1:14">
+    <row r="60" spans="1:31">
       <c r="A60">
         <v>61</v>
       </c>
@@ -5400,7 +4786,7 @@
       <c r="K60">
         <v>2</v>
       </c>
-      <c r="L60" s="4">
+      <c r="L60" s="3">
         <v>2</v>
       </c>
       <c r="M60">
@@ -5410,7 +4796,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:14">
+    <row r="61" spans="1:31">
       <c r="A61">
         <v>62</v>
       </c>
@@ -5429,13 +4815,13 @@
       <c r="I61" t="s">
         <v>49</v>
       </c>
-      <c r="J61" s="4">
+      <c r="J61" s="3">
         <v>14</v>
       </c>
       <c r="K61">
         <v>3</v>
       </c>
-      <c r="L61" s="4">
+      <c r="L61" s="3">
         <v>2</v>
       </c>
       <c r="M61">
@@ -5447,25 +4833,23 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
-  <headerFooter/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:I62"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="3.425" customWidth="1"/>
-    <col min="2" max="2" width="27.425" customWidth="1"/>
+    <col min="1" max="1" width="3.42578125" customWidth="1"/>
+    <col min="2" max="2" width="27.42578125" customWidth="1"/>
     <col min="3" max="3" width="35" customWidth="1"/>
     <col min="4" max="4" width="33" customWidth="1"/>
-    <col min="5" max="5" width="19.2833333333333" customWidth="1"/>
-    <col min="6" max="6" width="18.8583333333333" customWidth="1"/>
-    <col min="7" max="8" width="10.2833333333333" customWidth="1"/>
-    <col min="9" max="9" width="15.1416666666667" customWidth="1"/>
+    <col min="5" max="5" width="19.28515625" customWidth="1"/>
+    <col min="6" max="6" width="18.85546875" customWidth="1"/>
+    <col min="7" max="8" width="10.28515625" customWidth="1"/>
+    <col min="9" max="9" width="15.140625" customWidth="1"/>
     <col min="10" max="10" width="22" customWidth="1"/>
   </cols>
   <sheetData>
@@ -6789,26 +6173,24 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
-  <headerFooter/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:O22"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="9.425" customWidth="1"/>
-    <col min="2" max="2" width="27.425" customWidth="1"/>
-    <col min="3" max="3" width="14.425" customWidth="1"/>
-    <col min="4" max="5" width="16.1416666666667" customWidth="1"/>
-    <col min="6" max="6" width="12.425" customWidth="1"/>
-    <col min="7" max="7" width="14.425" customWidth="1"/>
+    <col min="1" max="1" width="9.42578125" customWidth="1"/>
+    <col min="2" max="2" width="27.42578125" customWidth="1"/>
+    <col min="3" max="3" width="14.42578125" customWidth="1"/>
+    <col min="4" max="5" width="16.140625" customWidth="1"/>
+    <col min="6" max="6" width="12.42578125" customWidth="1"/>
+    <col min="7" max="7" width="14.42578125" customWidth="1"/>
     <col min="8" max="8" width="10" customWidth="1"/>
     <col min="9" max="9" width="13" customWidth="1"/>
-    <col min="10" max="10" width="10.1416666666667" customWidth="1"/>
+    <col min="10" max="10" width="10.140625" customWidth="1"/>
     <col min="11" max="11" width="13" customWidth="1"/>
   </cols>
   <sheetData>
@@ -6859,7 +6241,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:15">
       <c r="A2">
         <v>0</v>
       </c>
@@ -6888,7 +6270,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:15">
       <c r="A3">
         <v>1</v>
       </c>
@@ -6911,7 +6293,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:15">
       <c r="A4">
         <v>2</v>
       </c>
@@ -6928,7 +6310,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
+    <row r="5" spans="1:15">
       <c r="A5">
         <v>3</v>
       </c>
@@ -6963,7 +6345,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:15">
       <c r="A6">
         <v>4</v>
       </c>
@@ -6986,7 +6368,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:15">
       <c r="A7">
         <v>5</v>
       </c>
@@ -7009,7 +6391,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="8" spans="1:7">
+    <row r="8" spans="1:15">
       <c r="A8">
         <v>6</v>
       </c>
@@ -7032,7 +6414,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:15">
       <c r="A9">
         <v>7</v>
       </c>
@@ -7055,7 +6437,7 @@
         <v>-0.5</v>
       </c>
     </row>
-    <row r="10" spans="1:7">
+    <row r="10" spans="1:15">
       <c r="A10">
         <v>8</v>
       </c>
@@ -7078,7 +6460,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:9">
+    <row r="11" spans="1:15">
       <c r="A11">
         <v>9</v>
       </c>
@@ -7107,7 +6489,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="12" spans="1:9">
+    <row r="12" spans="1:15">
       <c r="A12">
         <v>10</v>
       </c>
@@ -7136,7 +6518,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="13" spans="1:7">
+    <row r="13" spans="1:15">
       <c r="A13">
         <v>11</v>
       </c>
@@ -7159,7 +6541,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:7">
+    <row r="14" spans="1:15">
       <c r="A14">
         <v>12</v>
       </c>
@@ -7182,7 +6564,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:7">
+    <row r="15" spans="1:15">
       <c r="A15">
         <v>13</v>
       </c>
@@ -7205,7 +6587,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="1:7">
+    <row r="16" spans="1:15">
       <c r="A16">
         <v>14</v>
       </c>
@@ -7274,7 +6656,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:5">
+    <row r="19" spans="1:7">
       <c r="A19">
         <v>17</v>
       </c>
@@ -7291,7 +6673,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:5">
+    <row r="20" spans="1:7">
       <c r="A20">
         <v>18</v>
       </c>
@@ -7308,7 +6690,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:5">
+    <row r="21" spans="1:7">
       <c r="A21">
         <v>19</v>
       </c>
@@ -7350,24 +6732,22 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
-  <headerFooter/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:G11"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="4.85833333333333" customWidth="1"/>
-    <col min="2" max="2" width="22.7083333333333" customWidth="1"/>
-    <col min="3" max="3" width="28.5666666666667" customWidth="1"/>
-    <col min="4" max="4" width="15.5666666666667" customWidth="1"/>
-    <col min="5" max="5" width="16.1416666666667" customWidth="1"/>
+    <col min="1" max="1" width="4.85546875" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="3" max="3" width="28.5703125" customWidth="1"/>
+    <col min="4" max="4" width="15.5703125" customWidth="1"/>
+    <col min="5" max="5" width="16.140625" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="11.1416666666667" customWidth="1"/>
+    <col min="7" max="7" width="11.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -7393,7 +6773,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:7">
       <c r="A2">
         <v>0</v>
       </c>
@@ -7413,7 +6793,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" ht="12.95" customHeight="1" spans="1:6">
+    <row r="3" spans="1:7" ht="12.95" customHeight="1">
       <c r="A3">
         <v>1</v>
       </c>
@@ -7430,7 +6810,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="4" ht="12.95" customHeight="1" spans="1:6">
+    <row r="4" spans="1:7" ht="12.95" customHeight="1">
       <c r="A4">
         <v>2</v>
       </c>
@@ -7447,7 +6827,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:7">
       <c r="A5">
         <v>3</v>
       </c>
@@ -7467,7 +6847,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:7">
       <c r="A6">
         <v>4</v>
       </c>
@@ -7487,7 +6867,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:7">
       <c r="A7">
         <v>5</v>
       </c>
@@ -7507,7 +6887,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:7">
       <c r="A8">
         <v>6</v>
       </c>
@@ -7527,7 +6907,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:7">
       <c r="A9">
         <v>7</v>
       </c>
@@ -7547,7 +6927,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:7">
       <c r="A10">
         <v>8</v>
       </c>
@@ -7567,7 +6947,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:7">
       <c r="A11">
         <v>9</v>
       </c>
@@ -7589,7 +6969,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
-  <headerFooter/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
the game can run again!!
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Configurations/Cards.xlsx
+++ b/Assets/StreamingAssets/Configurations/Cards.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29029"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity\VTuberSim\Assets\StreamingAssets\Configurations\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA9C686B-D039-42AD-93AF-A2A11D8274B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView windowWidth="24750" windowHeight="10480" activeTab="1"/>
+    <workbookView xWindow="25490" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cards" sheetId="1" r:id="rId1"/>
@@ -24,8 +30,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -1019,167 +1023,17 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="20">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="34">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1198,188 +1052,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="11">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -1405,251 +1079,9 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
   <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -1664,71 +1096,27 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="49">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
-    <cellStyle name="货币" xfId="2" builtinId="4"/>
-    <cellStyle name="百分比" xfId="3" builtinId="5"/>
-    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
-    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
-    <cellStyle name="超链接" xfId="6" builtinId="8"/>
-    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
-    <cellStyle name="注释" xfId="8" builtinId="10"/>
-    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
-    <cellStyle name="标题" xfId="10" builtinId="15"/>
-    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
-    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
-    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
-    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
-    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
-    <cellStyle name="输入" xfId="16" builtinId="20"/>
-    <cellStyle name="输出" xfId="17" builtinId="21"/>
-    <cellStyle name="计算" xfId="18" builtinId="22"/>
-    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
-    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
-    <cellStyle name="汇总" xfId="21" builtinId="25"/>
-    <cellStyle name="好" xfId="22" builtinId="26"/>
-    <cellStyle name="差" xfId="23" builtinId="27"/>
-    <cellStyle name="适中" xfId="24" builtinId="28"/>
-    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
-    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
-    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
-    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
-    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
-    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
-      <color rgb="00FFFFFF"/>
-      <color rgb="00AB0580"/>
-      <color rgb="0000B050"/>
-      <color rgb="00FFB200"/>
-      <color rgb="004B58FF"/>
-      <color rgb="00FF2160"/>
+      <color rgb="FFFFFFFF"/>
+      <color rgb="FFAB0580"/>
+      <color rgb="FF00B050"/>
+      <color rgb="FFFFB200"/>
+      <color rgb="FF4B58FF"/>
+      <color rgb="FFFF2160"/>
     </mruColors>
   </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1986,49 +1374,49 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr filterMode="1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AH61"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="3.425" customWidth="1"/>
-    <col min="2" max="2" width="12.7083333333333" customWidth="1"/>
+    <col min="1" max="1" width="3.42578125" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" customWidth="1"/>
     <col min="3" max="3" width="35" customWidth="1"/>
-    <col min="4" max="4" width="57.7083333333333" customWidth="1"/>
-    <col min="5" max="5" width="10.425" style="2" customWidth="1"/>
-    <col min="6" max="6" width="4.85833333333333" customWidth="1"/>
-    <col min="7" max="7" width="7.85833333333333" customWidth="1"/>
+    <col min="4" max="4" width="57.7109375" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" style="2" customWidth="1"/>
+    <col min="6" max="6" width="4.85546875" customWidth="1"/>
+    <col min="7" max="7" width="7.85546875" customWidth="1"/>
     <col min="8" max="8" width="5" customWidth="1"/>
-    <col min="9" max="9" width="5.56666666666667" style="3" customWidth="1"/>
-    <col min="10" max="10" width="10.5666666666667" customWidth="1"/>
-    <col min="11" max="11" width="9.70833333333333" style="3" customWidth="1"/>
-    <col min="12" max="12" width="7.14166666666667" customWidth="1"/>
+    <col min="9" max="9" width="5.5703125" style="3" customWidth="1"/>
+    <col min="10" max="10" width="10.5703125" customWidth="1"/>
+    <col min="11" max="11" width="9.7109375" style="3" customWidth="1"/>
+    <col min="12" max="12" width="7.140625" customWidth="1"/>
     <col min="13" max="13" width="14" style="3" customWidth="1"/>
-    <col min="14" max="14" width="10.2833333333333" customWidth="1"/>
-    <col min="15" max="15" width="13.7083333333333" customWidth="1"/>
-    <col min="16" max="16" width="9.70833333333333" style="3" customWidth="1"/>
-    <col min="17" max="17" width="9.70833333333333" customWidth="1"/>
-    <col min="18" max="18" width="12.1416666666667" customWidth="1"/>
-    <col min="19" max="19" width="17.7083333333333" style="3" customWidth="1"/>
+    <col min="14" max="14" width="10.28515625" customWidth="1"/>
+    <col min="15" max="15" width="13.7109375" customWidth="1"/>
+    <col min="16" max="16" width="9.7109375" style="3" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" customWidth="1"/>
+    <col min="18" max="18" width="12.140625" customWidth="1"/>
+    <col min="19" max="19" width="17.7109375" style="3" customWidth="1"/>
     <col min="20" max="20" width="11" customWidth="1"/>
-    <col min="21" max="21" width="12.2833333333333" customWidth="1"/>
-    <col min="22" max="22" width="17.1416666666667" style="3" customWidth="1"/>
-    <col min="25" max="25" width="17.7083333333333" style="3" customWidth="1"/>
-    <col min="26" max="26" width="10.7083333333333" customWidth="1"/>
+    <col min="21" max="21" width="12.28515625" customWidth="1"/>
+    <col min="22" max="22" width="17.140625" style="3" customWidth="1"/>
+    <col min="25" max="25" width="17.7109375" style="3" customWidth="1"/>
+    <col min="26" max="26" width="10.7109375" customWidth="1"/>
     <col min="27" max="27" width="11" customWidth="1"/>
-    <col min="28" max="28" width="17.7083333333333" style="3" customWidth="1"/>
-    <col min="29" max="29" width="12.425" customWidth="1"/>
-    <col min="30" max="30" width="12.425" style="3" customWidth="1"/>
-    <col min="31" max="31" width="12.2833333333333" customWidth="1"/>
+    <col min="28" max="28" width="17.7109375" style="3" customWidth="1"/>
+    <col min="29" max="29" width="12.42578125" customWidth="1"/>
+    <col min="30" max="30" width="12.42578125" style="3" customWidth="1"/>
+    <col min="31" max="31" width="12.28515625" customWidth="1"/>
     <col min="32" max="32" width="9" style="3"/>
-    <col min="33" max="33" width="4.28333333333333" customWidth="1"/>
+    <col min="33" max="33" width="4.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33">
+    <row r="1" spans="1:34">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2129,7 +1517,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="2" hidden="1" spans="1:33">
+    <row r="2" spans="1:34">
       <c r="A2">
         <v>0</v>
       </c>
@@ -2184,7 +1572,7 @@
       <c r="AF2"/>
       <c r="AG2" s="5"/>
     </row>
-    <row r="3" hidden="1" spans="1:33">
+    <row r="3" spans="1:34">
       <c r="A3">
         <v>1</v>
       </c>
@@ -2239,7 +1627,7 @@
       <c r="AF3"/>
       <c r="AG3" s="5"/>
     </row>
-    <row r="4" spans="1:33">
+    <row r="4" spans="1:34">
       <c r="A4">
         <v>2</v>
       </c>
@@ -2299,7 +1687,7 @@
       </c>
       <c r="AG4" s="5"/>
     </row>
-    <row r="5" hidden="1" spans="1:33">
+    <row r="5" spans="1:34">
       <c r="A5">
         <v>3</v>
       </c>
@@ -2362,7 +1750,7 @@
       <c r="AF5"/>
       <c r="AG5" s="5"/>
     </row>
-    <row r="6" spans="1:33">
+    <row r="6" spans="1:34">
       <c r="A6">
         <v>4</v>
       </c>
@@ -2428,7 +1816,7 @@
       </c>
       <c r="AG6" s="5"/>
     </row>
-    <row r="7" hidden="1" spans="1:33">
+    <row r="7" spans="1:34">
       <c r="A7">
         <v>5</v>
       </c>
@@ -2494,7 +1882,7 @@
       <c r="AF7"/>
       <c r="AG7" s="5"/>
     </row>
-    <row r="8" hidden="1" spans="1:33">
+    <row r="8" spans="1:34">
       <c r="A8">
         <v>6</v>
       </c>
@@ -2567,7 +1955,7 @@
       <c r="AF8"/>
       <c r="AG8" s="5"/>
     </row>
-    <row r="9" hidden="1" spans="1:33">
+    <row r="9" spans="1:34">
       <c r="A9">
         <v>8</v>
       </c>
@@ -2630,7 +2018,7 @@
       <c r="AF9"/>
       <c r="AG9" s="5"/>
     </row>
-    <row r="10" hidden="1" spans="1:33">
+    <row r="10" spans="1:34">
       <c r="A10">
         <v>9</v>
       </c>
@@ -2693,7 +2081,7 @@
       <c r="AF10"/>
       <c r="AG10" s="5"/>
     </row>
-    <row r="11" spans="1:33">
+    <row r="11" spans="1:34">
       <c r="A11">
         <v>10</v>
       </c>
@@ -2753,7 +2141,7 @@
       </c>
       <c r="AG11" s="5"/>
     </row>
-    <row r="12" hidden="1" spans="1:34">
+    <row r="12" spans="1:34">
       <c r="A12">
         <v>11</v>
       </c>
@@ -2819,7 +2207,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="13" hidden="1" spans="1:33">
+    <row r="13" spans="1:34">
       <c r="A13">
         <v>12</v>
       </c>
@@ -2882,7 +2270,7 @@
       <c r="AF13"/>
       <c r="AG13" s="5"/>
     </row>
-    <row r="14" hidden="1" spans="1:33">
+    <row r="14" spans="1:34">
       <c r="A14">
         <v>13</v>
       </c>
@@ -2937,7 +2325,7 @@
       <c r="AF14"/>
       <c r="AG14" s="5"/>
     </row>
-    <row r="15" hidden="1" spans="1:33">
+    <row r="15" spans="1:34">
       <c r="A15">
         <v>14</v>
       </c>
@@ -2992,7 +2380,7 @@
       <c r="AF15"/>
       <c r="AG15" s="5"/>
     </row>
-    <row r="16" hidden="1" spans="1:33">
+    <row r="16" spans="1:34">
       <c r="A16">
         <v>15</v>
       </c>
@@ -3047,7 +2435,7 @@
         <v>0.8</v>
       </c>
       <c r="V16" s="3">
-        <v>1.1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="Y16"/>
       <c r="AB16"/>
@@ -3055,7 +2443,7 @@
       <c r="AF16"/>
       <c r="AG16" s="5"/>
     </row>
-    <row r="17" hidden="1" spans="1:33">
+    <row r="17" spans="1:33">
       <c r="A17">
         <v>16</v>
       </c>
@@ -3179,14 +2567,14 @@
         <v>7</v>
       </c>
       <c r="AC18">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="AD18" s="3">
         <v>1.5</v>
       </c>
       <c r="AG18" s="5"/>
     </row>
-    <row r="19" hidden="1" spans="1:33">
+    <row r="19" spans="1:33">
       <c r="A19">
         <v>19</v>
       </c>
@@ -3378,7 +2766,7 @@
       </c>
       <c r="AG21" s="5"/>
     </row>
-    <row r="22" hidden="1" spans="1:33">
+    <row r="22" spans="1:33">
       <c r="A22">
         <v>22</v>
       </c>
@@ -3441,7 +2829,7 @@
       <c r="AF22"/>
       <c r="AG22" s="5"/>
     </row>
-    <row r="23" hidden="1" spans="1:33">
+    <row r="23" spans="1:33">
       <c r="A23">
         <v>23</v>
       </c>
@@ -3562,15 +2950,9 @@
       <c r="V24" s="3">
         <v>11</v>
       </c>
-      <c r="AC24">
-        <v>63</v>
-      </c>
-      <c r="AD24" s="3">
-        <v>3</v>
-      </c>
       <c r="AG24" s="5"/>
     </row>
-    <row r="25" hidden="1" spans="1:33">
+    <row r="25" spans="1:33">
       <c r="A25">
         <v>25</v>
       </c>
@@ -3625,7 +3007,7 @@
       <c r="AF25"/>
       <c r="AG25" s="5"/>
     </row>
-    <row r="26" hidden="1" spans="1:33">
+    <row r="26" spans="1:33">
       <c r="A26">
         <v>26</v>
       </c>
@@ -3817,7 +3199,7 @@
       </c>
       <c r="AG28" s="5"/>
     </row>
-    <row r="29" hidden="1" spans="1:33">
+    <row r="29" spans="1:33">
       <c r="A29">
         <v>30</v>
       </c>
@@ -3888,7 +3270,7 @@
       <c r="AF29"/>
       <c r="AG29" s="5"/>
     </row>
-    <row r="30" hidden="1" spans="1:33">
+    <row r="30" spans="1:33">
       <c r="A30">
         <v>31</v>
       </c>
@@ -3951,7 +3333,7 @@
       <c r="AF30"/>
       <c r="AG30" s="6"/>
     </row>
-    <row r="31" hidden="1" spans="1:33">
+    <row r="31" spans="1:33">
       <c r="A31">
         <v>32</v>
       </c>
@@ -4014,7 +3396,7 @@
       <c r="AF31"/>
       <c r="AG31" s="6"/>
     </row>
-    <row r="32" hidden="1" spans="1:32">
+    <row r="32" spans="1:33">
       <c r="A32">
         <v>33</v>
       </c>
@@ -4060,7 +3442,7 @@
       <c r="AD32"/>
       <c r="AF32"/>
     </row>
-    <row r="33" spans="1:30">
+    <row r="33" spans="1:32">
       <c r="A33">
         <v>34</v>
       </c>
@@ -4116,7 +3498,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:19">
+    <row r="34" spans="1:32">
       <c r="A34">
         <v>35</v>
       </c>
@@ -4169,7 +3551,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="35" spans="1:19">
+    <row r="35" spans="1:32">
       <c r="A35">
         <v>36</v>
       </c>
@@ -4219,7 +3601,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="36" spans="1:22">
+    <row r="36" spans="1:32">
       <c r="A36">
         <v>37</v>
       </c>
@@ -4278,7 +3660,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="37" hidden="1" spans="1:32">
+    <row r="37" spans="1:32">
       <c r="A37">
         <v>38</v>
       </c>
@@ -4340,7 +3722,7 @@
       <c r="AD37"/>
       <c r="AF37"/>
     </row>
-    <row r="38" hidden="1" spans="1:32">
+    <row r="38" spans="1:32">
       <c r="A38">
         <v>39</v>
       </c>
@@ -4402,7 +3784,7 @@
       <c r="AD38"/>
       <c r="AF38"/>
     </row>
-    <row r="39" hidden="1" spans="1:32">
+    <row r="39" spans="1:32">
       <c r="A39">
         <v>40</v>
       </c>
@@ -4464,7 +3846,7 @@
       <c r="AD39"/>
       <c r="AF39"/>
     </row>
-    <row r="40" hidden="1" spans="1:32">
+    <row r="40" spans="1:32">
       <c r="A40">
         <v>41</v>
       </c>
@@ -4526,7 +3908,7 @@
       <c r="AD40"/>
       <c r="AF40"/>
     </row>
-    <row r="41" hidden="1" spans="1:32">
+    <row r="41" spans="1:32">
       <c r="A41">
         <v>42</v>
       </c>
@@ -4588,7 +3970,7 @@
       <c r="AD41"/>
       <c r="AF41"/>
     </row>
-    <row r="42" hidden="1" spans="1:32">
+    <row r="42" spans="1:32">
       <c r="A42">
         <v>43</v>
       </c>
@@ -4650,7 +4032,7 @@
       <c r="AD42"/>
       <c r="AF42"/>
     </row>
-    <row r="43" hidden="1" spans="1:32">
+    <row r="43" spans="1:32">
       <c r="A43">
         <v>44</v>
       </c>
@@ -4720,7 +4102,7 @@
       <c r="AD43"/>
       <c r="AF43"/>
     </row>
-    <row r="44" spans="1:22">
+    <row r="44" spans="1:32">
       <c r="A44">
         <v>45</v>
       </c>
@@ -4779,7 +4161,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="45" hidden="1" spans="1:32">
+    <row r="45" spans="1:32">
       <c r="A45">
         <v>46</v>
       </c>
@@ -4849,7 +4231,7 @@
       <c r="AD45"/>
       <c r="AF45"/>
     </row>
-    <row r="46" hidden="1" spans="1:32">
+    <row r="46" spans="1:32">
       <c r="A46">
         <v>47</v>
       </c>
@@ -4919,7 +4301,7 @@
       <c r="AD46"/>
       <c r="AF46"/>
     </row>
-    <row r="47" hidden="1" spans="1:32">
+    <row r="47" spans="1:32">
       <c r="A47">
         <v>48</v>
       </c>
@@ -4973,7 +4355,7 @@
       <c r="AD47"/>
       <c r="AF47"/>
     </row>
-    <row r="48" hidden="1" spans="1:32">
+    <row r="48" spans="1:32">
       <c r="A48">
         <v>49</v>
       </c>
@@ -5035,7 +4417,7 @@
       <c r="AD48"/>
       <c r="AF48"/>
     </row>
-    <row r="49" spans="1:22">
+    <row r="49" spans="1:32">
       <c r="A49">
         <v>50</v>
       </c>
@@ -5094,7 +4476,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="50" hidden="1" spans="1:32">
+    <row r="50" spans="1:32">
       <c r="A50">
         <v>51</v>
       </c>
@@ -5146,7 +4528,7 @@
         <v>18</v>
       </c>
       <c r="U50">
-        <v>1.1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="V50" s="3">
         <v>1.7</v>
@@ -5156,7 +4538,7 @@
       <c r="AD50"/>
       <c r="AF50"/>
     </row>
-    <row r="51" hidden="1" spans="1:32">
+    <row r="51" spans="1:32">
       <c r="A51">
         <v>52</v>
       </c>
@@ -5218,7 +4600,7 @@
       <c r="AD51"/>
       <c r="AF51"/>
     </row>
-    <row r="52" hidden="1" spans="1:32">
+    <row r="52" spans="1:32">
       <c r="A52">
         <v>53</v>
       </c>
@@ -5280,7 +4662,7 @@
       <c r="AD52"/>
       <c r="AF52"/>
     </row>
-    <row r="53" spans="1:22">
+    <row r="53" spans="1:32">
       <c r="A53">
         <v>54</v>
       </c>
@@ -5342,7 +4724,7 @@
         <v>-0.5</v>
       </c>
     </row>
-    <row r="54" spans="1:25">
+    <row r="54" spans="1:32">
       <c r="A54">
         <v>55</v>
       </c>
@@ -5413,7 +4795,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="55" spans="1:31">
+    <row r="55" spans="1:32">
       <c r="A55">
         <v>56</v>
       </c>
@@ -5473,7 +4855,7 @@
       </c>
       <c r="AE55" s="3"/>
     </row>
-    <row r="56" spans="1:31">
+    <row r="56" spans="1:32">
       <c r="A56">
         <v>57</v>
       </c>
@@ -5545,7 +4927,7 @@
       </c>
       <c r="AE56" s="3"/>
     </row>
-    <row r="57" spans="1:22">
+    <row r="57" spans="1:32">
       <c r="A57">
         <v>58</v>
       </c>
@@ -5607,7 +4989,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="58" spans="1:15">
+    <row r="58" spans="1:32">
       <c r="A58">
         <v>59</v>
       </c>
@@ -5648,7 +5030,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:19">
+    <row r="59" spans="1:32">
       <c r="A59">
         <v>60</v>
       </c>
@@ -5698,7 +5080,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="60" spans="1:15">
+    <row r="60" spans="1:32">
       <c r="A60">
         <v>61</v>
       </c>
@@ -5739,7 +5121,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" hidden="1" spans="1:15">
+    <row r="61" spans="1:32">
       <c r="A61">
         <v>62</v>
       </c>
@@ -5778,34 +5160,25 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:AH61" etc:filterBottomFollowUsedRange="0">
-    <filterColumn colId="6">
-      <filters>
-        <filter val="C"/>
-      </filters>
-    </filterColumn>
-    <extLst/>
-  </autoFilter>
+  <autoFilter ref="A1:AH61" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
-  <headerFooter/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:I67"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="3.425" customWidth="1"/>
-    <col min="2" max="2" width="27.425" customWidth="1"/>
+    <col min="1" max="1" width="3.42578125" customWidth="1"/>
+    <col min="2" max="2" width="27.42578125" customWidth="1"/>
     <col min="3" max="3" width="35" customWidth="1"/>
     <col min="4" max="4" width="33" customWidth="1"/>
-    <col min="5" max="5" width="19.2833333333333" customWidth="1"/>
-    <col min="6" max="6" width="18.8583333333333" customWidth="1"/>
-    <col min="7" max="8" width="10.2833333333333" customWidth="1"/>
-    <col min="9" max="9" width="15.1416666666667" customWidth="1"/>
+    <col min="5" max="5" width="19.28515625" customWidth="1"/>
+    <col min="6" max="6" width="18.85546875" customWidth="1"/>
+    <col min="7" max="8" width="10.28515625" customWidth="1"/>
+    <col min="9" max="9" width="15.140625" customWidth="1"/>
     <col min="10" max="10" width="22" customWidth="1"/>
   </cols>
   <sheetData>
@@ -7127,7 +6500,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="63" customFormat="1" spans="1:9">
+    <row r="63" spans="1:9">
       <c r="A63">
         <v>61</v>
       </c>
@@ -7187,7 +6560,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="66" customFormat="1" spans="1:9">
+    <row r="66" spans="1:9">
       <c r="A66">
         <v>64</v>
       </c>
@@ -7232,26 +6605,24 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
-  <headerFooter/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:O24"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="9.425" customWidth="1"/>
-    <col min="2" max="2" width="27.425" customWidth="1"/>
-    <col min="3" max="3" width="14.425" customWidth="1"/>
-    <col min="4" max="5" width="16.1416666666667" customWidth="1"/>
-    <col min="6" max="6" width="12.425" customWidth="1"/>
-    <col min="7" max="7" width="14.425" customWidth="1"/>
+    <col min="1" max="1" width="9.42578125" customWidth="1"/>
+    <col min="2" max="2" width="27.42578125" customWidth="1"/>
+    <col min="3" max="3" width="14.42578125" customWidth="1"/>
+    <col min="4" max="5" width="16.140625" customWidth="1"/>
+    <col min="6" max="6" width="12.42578125" customWidth="1"/>
+    <col min="7" max="7" width="14.42578125" customWidth="1"/>
     <col min="8" max="8" width="10" customWidth="1"/>
     <col min="9" max="9" width="13" customWidth="1"/>
-    <col min="10" max="10" width="10.1416666666667" customWidth="1"/>
+    <col min="10" max="10" width="10.140625" customWidth="1"/>
     <col min="11" max="11" width="13" customWidth="1"/>
   </cols>
   <sheetData>
@@ -7302,7 +6673,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:15">
       <c r="A2">
         <v>0</v>
       </c>
@@ -7331,7 +6702,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:15">
       <c r="A3">
         <v>1</v>
       </c>
@@ -7354,7 +6725,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:15">
       <c r="A4">
         <v>2</v>
       </c>
@@ -7371,7 +6742,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
+    <row r="5" spans="1:15">
       <c r="A5">
         <v>3</v>
       </c>
@@ -7406,7 +6777,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:15">
       <c r="A6">
         <v>4</v>
       </c>
@@ -7429,7 +6800,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:15">
       <c r="A7">
         <v>5</v>
       </c>
@@ -7452,7 +6823,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="8" spans="1:7">
+    <row r="8" spans="1:15">
       <c r="A8">
         <v>6</v>
       </c>
@@ -7475,7 +6846,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:15">
       <c r="A9">
         <v>7</v>
       </c>
@@ -7498,7 +6869,7 @@
         <v>-0.5</v>
       </c>
     </row>
-    <row r="10" spans="1:7">
+    <row r="10" spans="1:15">
       <c r="A10">
         <v>8</v>
       </c>
@@ -7521,7 +6892,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:9">
+    <row r="11" spans="1:15">
       <c r="A11">
         <v>9</v>
       </c>
@@ -7550,7 +6921,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="12" spans="1:9">
+    <row r="12" spans="1:15">
       <c r="A12">
         <v>10</v>
       </c>
@@ -7579,7 +6950,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="13" spans="1:7">
+    <row r="13" spans="1:15">
       <c r="A13">
         <v>11</v>
       </c>
@@ -7602,7 +6973,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:7">
+    <row r="14" spans="1:15">
       <c r="A14">
         <v>12</v>
       </c>
@@ -7625,7 +6996,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:7">
+    <row r="15" spans="1:15">
       <c r="A15">
         <v>13</v>
       </c>
@@ -7648,7 +7019,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="1:7">
+    <row r="16" spans="1:15">
       <c r="A16">
         <v>14</v>
       </c>
@@ -7717,7 +7088,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:5">
+    <row r="19" spans="1:7">
       <c r="A19">
         <v>17</v>
       </c>
@@ -7734,7 +7105,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:5">
+    <row r="20" spans="1:7">
       <c r="A20">
         <v>18</v>
       </c>
@@ -7751,7 +7122,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:5">
+    <row r="21" spans="1:7">
       <c r="A21">
         <v>19</v>
       </c>
@@ -7839,24 +7210,22 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
-  <headerFooter/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:G11"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="4.85833333333333" customWidth="1"/>
-    <col min="2" max="2" width="22.7083333333333" customWidth="1"/>
-    <col min="3" max="3" width="28.5666666666667" customWidth="1"/>
-    <col min="4" max="4" width="15.5666666666667" customWidth="1"/>
-    <col min="5" max="5" width="16.1416666666667" customWidth="1"/>
+    <col min="1" max="1" width="4.85546875" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="3" max="3" width="28.5703125" customWidth="1"/>
+    <col min="4" max="4" width="15.5703125" customWidth="1"/>
+    <col min="5" max="5" width="16.140625" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="11.1416666666667" customWidth="1"/>
+    <col min="7" max="7" width="11.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -7882,7 +7251,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:7">
       <c r="A2">
         <v>0</v>
       </c>
@@ -7902,7 +7271,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" ht="12.95" customHeight="1" spans="1:6">
+    <row r="3" spans="1:7" ht="12.95" customHeight="1">
       <c r="A3">
         <v>1</v>
       </c>
@@ -7919,7 +7288,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="4" ht="12.95" customHeight="1" spans="1:6">
+    <row r="4" spans="1:7" ht="12.95" customHeight="1">
       <c r="A4">
         <v>2</v>
       </c>
@@ -7936,7 +7305,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:7">
       <c r="A5">
         <v>3</v>
       </c>
@@ -7956,7 +7325,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:7">
       <c r="A6">
         <v>4</v>
       </c>
@@ -7976,7 +7345,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:7">
       <c r="A7">
         <v>5</v>
       </c>
@@ -7996,7 +7365,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:7">
       <c r="A8">
         <v>6</v>
       </c>
@@ -8016,7 +7385,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:7">
       <c r="A9">
         <v>7</v>
       </c>
@@ -8036,7 +7405,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:7">
       <c r="A10">
         <v>8</v>
       </c>
@@ -8056,7 +7425,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:7">
       <c r="A11">
         <v>9</v>
       </c>
@@ -8078,7 +7447,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
-  <headerFooter/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added and fixed buncha stuff
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Configurations/Cards.xlsx
+++ b/Assets/StreamingAssets/Configurations/Cards.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29029"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity\VTuberSim\Assets\StreamingAssets\Configurations\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24F47183-F6A7-4E70-A44F-2E8DAA5F15B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView windowWidth="24750" windowHeight="10480"/>
+    <workbookView xWindow="0" yWindow="540" windowWidth="38730" windowHeight="20850" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cards" sheetId="1" r:id="rId1"/>
@@ -13,7 +19,7 @@
     <sheet name="Conditions" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Cards!$A$1:$AH$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Cards!$A$1:$AI$61</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -24,8 +30,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -33,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="847" uniqueCount="338">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="848" uniqueCount="339">
   <si>
     <t>ID</t>
   </si>
@@ -1047,172 +1051,32 @@
   </si>
   <si>
     <t>VCardTypeUsedCountCondition</t>
+  </si>
+  <si>
+    <t>Priority</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="20">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="等线"/>
-      <charset val="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="34">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1231,188 +1095,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="11">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -1438,253 +1122,11 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1696,72 +1138,29 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="49">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
-    <cellStyle name="货币" xfId="2" builtinId="4"/>
-    <cellStyle name="百分比" xfId="3" builtinId="5"/>
-    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
-    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
-    <cellStyle name="超链接" xfId="6" builtinId="8"/>
-    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
-    <cellStyle name="注释" xfId="8" builtinId="10"/>
-    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
-    <cellStyle name="标题" xfId="10" builtinId="15"/>
-    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
-    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
-    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
-    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
-    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
-    <cellStyle name="输入" xfId="16" builtinId="20"/>
-    <cellStyle name="输出" xfId="17" builtinId="21"/>
-    <cellStyle name="计算" xfId="18" builtinId="22"/>
-    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
-    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
-    <cellStyle name="汇总" xfId="21" builtinId="25"/>
-    <cellStyle name="好" xfId="22" builtinId="26"/>
-    <cellStyle name="差" xfId="23" builtinId="27"/>
-    <cellStyle name="适中" xfId="24" builtinId="28"/>
-    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
-    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
-    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
-    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
-    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
-    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
-      <color rgb="00FFFFFF"/>
-      <color rgb="00AB0580"/>
-      <color rgb="0000B050"/>
-      <color rgb="00FFB200"/>
-      <color rgb="004B58FF"/>
-      <color rgb="00FF2160"/>
+      <color rgb="FFFFFFFF"/>
+      <color rgb="FFAB0580"/>
+      <color rgb="FF00B050"/>
+      <color rgb="FFFFB200"/>
+      <color rgb="FF4B58FF"/>
+      <color rgb="FFFF2160"/>
     </mruColors>
   </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -2019,49 +1418,49 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:AH61"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:AI61"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="3.425" customWidth="1"/>
-    <col min="2" max="2" width="12.7083333333333" customWidth="1"/>
+    <col min="1" max="1" width="3.42578125" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" customWidth="1"/>
     <col min="3" max="3" width="35" customWidth="1"/>
-    <col min="4" max="4" width="57.7083333333333" customWidth="1"/>
-    <col min="5" max="5" width="10.425" style="2" customWidth="1"/>
-    <col min="6" max="6" width="4.85833333333333" customWidth="1"/>
-    <col min="7" max="7" width="7.85833333333333" customWidth="1"/>
+    <col min="4" max="4" width="57.7109375" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" style="2" customWidth="1"/>
+    <col min="6" max="6" width="4.85546875" customWidth="1"/>
+    <col min="7" max="7" width="7.85546875" customWidth="1"/>
     <col min="8" max="8" width="5" customWidth="1"/>
-    <col min="9" max="9" width="5.56666666666667" style="3" customWidth="1"/>
-    <col min="10" max="10" width="10.5666666666667" customWidth="1"/>
-    <col min="11" max="11" width="9.70833333333333" style="3" customWidth="1"/>
-    <col min="12" max="12" width="7.14166666666667" customWidth="1"/>
+    <col min="9" max="9" width="5.5703125" style="3" customWidth="1"/>
+    <col min="10" max="10" width="10.5703125" customWidth="1"/>
+    <col min="11" max="11" width="9.7109375" style="3" customWidth="1"/>
+    <col min="12" max="12" width="7.140625" customWidth="1"/>
     <col min="13" max="13" width="14" style="3" customWidth="1"/>
-    <col min="14" max="14" width="10.2833333333333" customWidth="1"/>
-    <col min="15" max="15" width="13.7083333333333" customWidth="1"/>
-    <col min="16" max="16" width="9.70833333333333" style="3" customWidth="1"/>
-    <col min="17" max="17" width="9.70833333333333" customWidth="1"/>
-    <col min="18" max="18" width="12.1416666666667" customWidth="1"/>
-    <col min="19" max="19" width="17.7083333333333" style="3" customWidth="1"/>
-    <col min="20" max="20" width="11" customWidth="1"/>
-    <col min="21" max="21" width="12.2833333333333" customWidth="1"/>
-    <col min="22" max="22" width="17.1416666666667" style="3" customWidth="1"/>
-    <col min="25" max="25" width="17.7083333333333" style="3" customWidth="1"/>
-    <col min="26" max="26" width="10.7083333333333" customWidth="1"/>
-    <col min="27" max="27" width="11" customWidth="1"/>
-    <col min="28" max="28" width="17.7083333333333" style="3" customWidth="1"/>
-    <col min="29" max="29" width="12.425" customWidth="1"/>
-    <col min="30" max="30" width="12.425" style="3" customWidth="1"/>
-    <col min="31" max="31" width="12.2833333333333" customWidth="1"/>
-    <col min="32" max="32" width="9" style="3"/>
-    <col min="33" max="33" width="4.28333333333333" customWidth="1"/>
+    <col min="14" max="14" width="10.28515625" customWidth="1"/>
+    <col min="15" max="16" width="13.7109375" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" style="3" customWidth="1"/>
+    <col min="18" max="18" width="9.7109375" customWidth="1"/>
+    <col min="19" max="19" width="12.140625" customWidth="1"/>
+    <col min="20" max="20" width="17.7109375" style="3" customWidth="1"/>
+    <col min="21" max="21" width="11" customWidth="1"/>
+    <col min="22" max="22" width="12.28515625" customWidth="1"/>
+    <col min="23" max="23" width="17.140625" style="3" customWidth="1"/>
+    <col min="26" max="26" width="17.7109375" style="3" customWidth="1"/>
+    <col min="27" max="27" width="10.7109375" customWidth="1"/>
+    <col min="28" max="28" width="11" customWidth="1"/>
+    <col min="29" max="29" width="17.7109375" style="3" customWidth="1"/>
+    <col min="30" max="30" width="12.42578125" customWidth="1"/>
+    <col min="31" max="31" width="12.42578125" style="3" customWidth="1"/>
+    <col min="32" max="32" width="12.28515625" customWidth="1"/>
+    <col min="33" max="33" width="9" style="3"/>
+    <col min="34" max="34" width="4.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33">
+    <row r="1" spans="1:35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2107,62 +1506,65 @@
       <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="P1" t="s">
+        <v>338</v>
+      </c>
+      <c r="Q1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="R1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="S1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="3" t="s">
+      <c r="T1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="U1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="V1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="3" t="s">
+      <c r="W1" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="2" t="s">
+      <c r="X1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s">
+      <c r="Y1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="3" t="s">
+      <c r="Z1" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="2" t="s">
+      <c r="AA1" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AB1" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="3" t="s">
+      <c r="AC1" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="2" t="s">
+      <c r="AD1" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" s="3" t="s">
+      <c r="AE1" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" t="s">
+      <c r="AF1" t="s">
         <v>30</v>
       </c>
-      <c r="AF1" s="3" t="s">
+      <c r="AG1" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="AG1" t="s">
+      <c r="AH1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:33">
+    <row r="2" spans="1:35">
       <c r="A2">
         <v>0</v>
       </c>
@@ -2175,7 +1577,7 @@
       <c r="D2" t="s">
         <v>35</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="7" t="s">
         <v>36</v>
       </c>
       <c r="F2" t="s">
@@ -2200,24 +1602,27 @@
       <c r="O2">
         <v>0</v>
       </c>
-      <c r="P2"/>
-      <c r="Q2" s="2">
+      <c r="P2">
+        <v>1</v>
+      </c>
+      <c r="Q2"/>
+      <c r="R2" s="2">
         <v>11</v>
       </c>
-      <c r="R2">
+      <c r="S2">
         <v>7</v>
       </c>
-      <c r="S2" s="3">
+      <c r="T2" s="3">
         <v>7</v>
       </c>
-      <c r="V2"/>
-      <c r="Y2"/>
-      <c r="AB2"/>
-      <c r="AD2"/>
-      <c r="AF2"/>
-      <c r="AG2" s="5"/>
-    </row>
-    <row r="3" spans="1:33">
+      <c r="W2"/>
+      <c r="Z2"/>
+      <c r="AC2"/>
+      <c r="AE2"/>
+      <c r="AG2"/>
+      <c r="AH2" s="5"/>
+    </row>
+    <row r="3" spans="1:35">
       <c r="A3">
         <v>1</v>
       </c>
@@ -2255,24 +1660,27 @@
       <c r="O3">
         <v>0</v>
       </c>
-      <c r="P3"/>
-      <c r="Q3" s="2">
-        <v>2</v>
-      </c>
-      <c r="R3">
+      <c r="P3">
+        <v>1</v>
+      </c>
+      <c r="Q3"/>
+      <c r="R3" s="2">
+        <v>2</v>
+      </c>
+      <c r="S3">
         <v>4</v>
       </c>
-      <c r="S3" s="3">
+      <c r="T3" s="3">
         <v>4</v>
       </c>
-      <c r="V3"/>
-      <c r="Y3"/>
-      <c r="AB3"/>
-      <c r="AD3"/>
-      <c r="AF3"/>
-      <c r="AG3" s="5"/>
-    </row>
-    <row r="4" spans="1:33">
+      <c r="W3"/>
+      <c r="Z3"/>
+      <c r="AC3"/>
+      <c r="AE3"/>
+      <c r="AG3"/>
+      <c r="AH3" s="5"/>
+    </row>
+    <row r="4" spans="1:35">
       <c r="A4">
         <v>2</v>
       </c>
@@ -2312,27 +1720,30 @@
       <c r="O4">
         <v>0</v>
       </c>
-      <c r="Q4" s="2">
+      <c r="P4">
+        <v>1</v>
+      </c>
+      <c r="R4" s="2">
         <v>11</v>
       </c>
-      <c r="R4">
+      <c r="S4">
         <v>15</v>
       </c>
-      <c r="S4" s="3">
+      <c r="T4" s="3">
         <v>18</v>
       </c>
-      <c r="T4">
+      <c r="U4">
         <v>56</v>
       </c>
-      <c r="U4">
+      <c r="V4">
         <v>9</v>
       </c>
-      <c r="V4" s="3">
+      <c r="W4" s="3">
         <v>12</v>
       </c>
-      <c r="AG4" s="5"/>
-    </row>
-    <row r="5" spans="1:33">
+      <c r="AH4" s="5"/>
+    </row>
+    <row r="5" spans="1:35">
       <c r="A5">
         <v>3</v>
       </c>
@@ -2370,32 +1781,32 @@
       <c r="O5">
         <v>0</v>
       </c>
-      <c r="P5"/>
-      <c r="Q5" s="2">
+      <c r="Q5"/>
+      <c r="R5" s="2">
         <v>11</v>
       </c>
-      <c r="R5">
+      <c r="S5">
         <v>5</v>
       </c>
-      <c r="S5" s="3">
+      <c r="T5" s="3">
         <v>5</v>
       </c>
-      <c r="T5" s="2">
-        <v>2</v>
-      </c>
-      <c r="U5">
-        <v>2</v>
-      </c>
-      <c r="V5" s="3">
-        <v>2</v>
-      </c>
-      <c r="Y5"/>
-      <c r="AB5"/>
-      <c r="AD5"/>
-      <c r="AF5"/>
-      <c r="AG5" s="5"/>
-    </row>
-    <row r="6" spans="1:33">
+      <c r="U5" s="2">
+        <v>2</v>
+      </c>
+      <c r="V5">
+        <v>2</v>
+      </c>
+      <c r="W5" s="3">
+        <v>2</v>
+      </c>
+      <c r="Z5"/>
+      <c r="AC5"/>
+      <c r="AE5"/>
+      <c r="AG5"/>
+      <c r="AH5" s="5"/>
+    </row>
+    <row r="6" spans="1:35">
       <c r="A6">
         <v>4</v>
       </c>
@@ -2438,30 +1849,30 @@
       <c r="O6">
         <v>1</v>
       </c>
-      <c r="Q6" s="2">
-        <v>0</v>
-      </c>
-      <c r="T6">
-        <v>2</v>
+      <c r="R6" s="2">
+        <v>0</v>
       </c>
       <c r="U6">
         <v>2</v>
       </c>
-      <c r="V6" s="3">
+      <c r="V6">
+        <v>2</v>
+      </c>
+      <c r="W6" s="3">
         <v>7</v>
       </c>
-      <c r="W6">
+      <c r="X6">
         <v>9</v>
       </c>
-      <c r="X6">
-        <v>1</v>
-      </c>
-      <c r="Y6" s="3">
-        <v>1</v>
-      </c>
-      <c r="AG6" s="5"/>
-    </row>
-    <row r="7" spans="1:33">
+      <c r="Y6">
+        <v>1</v>
+      </c>
+      <c r="Z6" s="3">
+        <v>1</v>
+      </c>
+      <c r="AH6" s="5"/>
+    </row>
+    <row r="7" spans="1:35">
       <c r="A7">
         <v>5</v>
       </c>
@@ -2499,35 +1910,35 @@
       <c r="O7">
         <v>1</v>
       </c>
-      <c r="P7"/>
-      <c r="Q7" s="2">
+      <c r="Q7"/>
+      <c r="R7" s="2">
         <v>4</v>
       </c>
-      <c r="S7"/>
-      <c r="T7" s="2">
+      <c r="T7"/>
+      <c r="U7" s="2">
         <v>21</v>
       </c>
-      <c r="U7">
-        <v>2</v>
-      </c>
-      <c r="V7" s="3">
-        <v>2</v>
-      </c>
-      <c r="W7" s="2">
+      <c r="V7">
+        <v>2</v>
+      </c>
+      <c r="W7" s="3">
+        <v>2</v>
+      </c>
+      <c r="X7" s="2">
         <v>14</v>
       </c>
-      <c r="X7">
-        <v>1</v>
-      </c>
-      <c r="Y7" s="3">
-        <v>1</v>
-      </c>
-      <c r="AB7"/>
-      <c r="AD7"/>
-      <c r="AF7"/>
-      <c r="AG7" s="5"/>
-    </row>
-    <row r="8" spans="1:33">
+      <c r="Y7">
+        <v>1</v>
+      </c>
+      <c r="Z7" s="3">
+        <v>1</v>
+      </c>
+      <c r="AC7"/>
+      <c r="AE7"/>
+      <c r="AG7"/>
+      <c r="AH7" s="5"/>
+    </row>
+    <row r="8" spans="1:35">
       <c r="A8">
         <v>6</v>
       </c>
@@ -2567,40 +1978,40 @@
       <c r="O8">
         <v>1</v>
       </c>
-      <c r="P8"/>
-      <c r="Q8" s="2">
-        <v>2</v>
-      </c>
-      <c r="R8">
+      <c r="Q8"/>
+      <c r="R8" s="2">
+        <v>2</v>
+      </c>
+      <c r="S8">
         <v>7</v>
       </c>
-      <c r="S8" s="3">
+      <c r="T8" s="3">
         <v>7</v>
       </c>
-      <c r="T8" s="2">
-        <v>3</v>
-      </c>
-      <c r="U8">
-        <v>1</v>
-      </c>
-      <c r="V8" s="3">
-        <v>1</v>
-      </c>
-      <c r="W8" s="2">
+      <c r="U8" s="2">
+        <v>3</v>
+      </c>
+      <c r="V8">
+        <v>1</v>
+      </c>
+      <c r="W8" s="3">
+        <v>1</v>
+      </c>
+      <c r="X8" s="2">
         <v>14</v>
       </c>
-      <c r="X8">
-        <v>1</v>
-      </c>
-      <c r="Y8" s="3">
-        <v>1</v>
-      </c>
-      <c r="AB8"/>
-      <c r="AD8"/>
-      <c r="AF8"/>
-      <c r="AG8" s="5"/>
-    </row>
-    <row r="9" spans="1:33">
+      <c r="Y8">
+        <v>1</v>
+      </c>
+      <c r="Z8" s="3">
+        <v>1</v>
+      </c>
+      <c r="AC8"/>
+      <c r="AE8"/>
+      <c r="AG8"/>
+      <c r="AH8" s="5"/>
+    </row>
+    <row r="9" spans="1:35">
       <c r="A9">
         <v>8</v>
       </c>
@@ -2638,32 +2049,32 @@
       <c r="O9">
         <v>0</v>
       </c>
-      <c r="P9"/>
-      <c r="Q9" s="2">
+      <c r="Q9"/>
+      <c r="R9" s="2">
         <v>6</v>
       </c>
-      <c r="R9">
-        <v>3</v>
-      </c>
-      <c r="S9" s="3">
+      <c r="S9">
+        <v>3</v>
+      </c>
+      <c r="T9" s="3">
         <v>4</v>
       </c>
-      <c r="T9" s="2">
-        <v>2</v>
-      </c>
-      <c r="U9">
-        <v>3</v>
-      </c>
-      <c r="V9" s="3">
+      <c r="U9" s="2">
+        <v>2</v>
+      </c>
+      <c r="V9">
+        <v>3</v>
+      </c>
+      <c r="W9" s="3">
         <v>4</v>
       </c>
-      <c r="Y9"/>
-      <c r="AB9"/>
-      <c r="AD9"/>
-      <c r="AF9"/>
-      <c r="AG9" s="5"/>
-    </row>
-    <row r="10" spans="1:33">
+      <c r="Z9"/>
+      <c r="AC9"/>
+      <c r="AE9"/>
+      <c r="AG9"/>
+      <c r="AH9" s="5"/>
+    </row>
+    <row r="10" spans="1:35">
       <c r="A10">
         <v>9</v>
       </c>
@@ -2701,32 +2112,32 @@
       <c r="O10">
         <v>0</v>
       </c>
-      <c r="P10"/>
-      <c r="Q10" s="2">
+      <c r="Q10"/>
+      <c r="R10" s="2">
         <v>7</v>
       </c>
-      <c r="R10">
-        <v>2</v>
-      </c>
-      <c r="S10" s="3">
-        <v>3</v>
-      </c>
-      <c r="T10" s="2">
-        <v>2</v>
-      </c>
-      <c r="U10">
-        <v>2</v>
-      </c>
-      <c r="V10" s="3">
-        <v>3</v>
-      </c>
-      <c r="Y10"/>
-      <c r="AB10"/>
-      <c r="AD10"/>
-      <c r="AF10"/>
-      <c r="AG10" s="5"/>
-    </row>
-    <row r="11" spans="1:33">
+      <c r="S10">
+        <v>2</v>
+      </c>
+      <c r="T10" s="3">
+        <v>3</v>
+      </c>
+      <c r="U10" s="2">
+        <v>2</v>
+      </c>
+      <c r="V10">
+        <v>2</v>
+      </c>
+      <c r="W10" s="3">
+        <v>3</v>
+      </c>
+      <c r="Z10"/>
+      <c r="AC10"/>
+      <c r="AE10"/>
+      <c r="AG10"/>
+      <c r="AH10" s="5"/>
+    </row>
+    <row r="11" spans="1:35">
       <c r="A11">
         <v>10</v>
       </c>
@@ -2766,27 +2177,27 @@
       <c r="O11">
         <v>0</v>
       </c>
-      <c r="Q11" s="2">
+      <c r="R11" s="2">
         <v>15</v>
       </c>
-      <c r="R11">
-        <v>2</v>
-      </c>
-      <c r="S11" s="3">
-        <v>3</v>
-      </c>
-      <c r="T11" s="2">
-        <v>2</v>
-      </c>
-      <c r="U11">
-        <v>2</v>
-      </c>
-      <c r="V11" s="3">
-        <v>3</v>
-      </c>
-      <c r="AG11" s="5"/>
-    </row>
-    <row r="12" spans="1:34">
+      <c r="S11">
+        <v>2</v>
+      </c>
+      <c r="T11" s="3">
+        <v>3</v>
+      </c>
+      <c r="U11" s="2">
+        <v>2</v>
+      </c>
+      <c r="V11">
+        <v>2</v>
+      </c>
+      <c r="W11" s="3">
+        <v>3</v>
+      </c>
+      <c r="AH11" s="5"/>
+    </row>
+    <row r="12" spans="1:35">
       <c r="A12">
         <v>11</v>
       </c>
@@ -2824,35 +2235,35 @@
       <c r="O12">
         <v>0</v>
       </c>
-      <c r="P12"/>
-      <c r="Q12" s="2">
+      <c r="Q12"/>
+      <c r="R12" s="2">
         <v>11</v>
       </c>
-      <c r="R12">
+      <c r="S12">
         <v>9</v>
       </c>
-      <c r="S12" s="3">
+      <c r="T12" s="3">
         <v>13</v>
       </c>
-      <c r="T12" s="2">
+      <c r="U12" s="2">
         <v>11</v>
       </c>
-      <c r="U12">
+      <c r="V12">
         <v>9</v>
       </c>
-      <c r="V12" s="3">
+      <c r="W12" s="3">
         <v>13</v>
       </c>
-      <c r="Y12"/>
-      <c r="AB12"/>
-      <c r="AD12"/>
-      <c r="AF12"/>
-      <c r="AG12" s="5"/>
-      <c r="AH12" t="s">
+      <c r="Z12"/>
+      <c r="AC12"/>
+      <c r="AE12"/>
+      <c r="AG12"/>
+      <c r="AH12" s="5"/>
+      <c r="AI12" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="13" spans="1:33">
+    <row r="13" spans="1:35">
       <c r="A13">
         <v>12</v>
       </c>
@@ -2890,32 +2301,32 @@
       <c r="O13">
         <v>0</v>
       </c>
-      <c r="P13"/>
-      <c r="Q13" s="2">
+      <c r="Q13"/>
+      <c r="R13" s="2">
         <v>11</v>
       </c>
-      <c r="R13">
+      <c r="S13">
         <v>11</v>
       </c>
-      <c r="S13" s="3">
+      <c r="T13" s="3">
         <v>15</v>
       </c>
-      <c r="T13" s="2">
-        <v>2</v>
-      </c>
-      <c r="U13">
+      <c r="U13" s="2">
+        <v>2</v>
+      </c>
+      <c r="V13">
         <v>7</v>
       </c>
-      <c r="V13" s="3">
+      <c r="W13" s="3">
         <v>9</v>
       </c>
-      <c r="Y13"/>
-      <c r="AB13"/>
-      <c r="AD13"/>
-      <c r="AF13"/>
-      <c r="AG13" s="5"/>
-    </row>
-    <row r="14" spans="1:33">
+      <c r="Z13"/>
+      <c r="AC13"/>
+      <c r="AE13"/>
+      <c r="AG13"/>
+      <c r="AH13" s="5"/>
+    </row>
+    <row r="14" spans="1:35">
       <c r="A14">
         <v>13</v>
       </c>
@@ -2953,24 +2364,24 @@
       <c r="O14">
         <v>0</v>
       </c>
-      <c r="P14"/>
-      <c r="Q14" s="2">
+      <c r="Q14"/>
+      <c r="R14" s="2">
         <v>6</v>
       </c>
-      <c r="R14">
+      <c r="S14">
         <v>6</v>
       </c>
-      <c r="S14" s="3">
+      <c r="T14" s="3">
         <v>8</v>
       </c>
-      <c r="V14"/>
-      <c r="Y14"/>
-      <c r="AB14"/>
-      <c r="AD14"/>
-      <c r="AF14"/>
-      <c r="AG14" s="5"/>
-    </row>
-    <row r="15" spans="1:33">
+      <c r="W14"/>
+      <c r="Z14"/>
+      <c r="AC14"/>
+      <c r="AE14"/>
+      <c r="AG14"/>
+      <c r="AH14" s="5"/>
+    </row>
+    <row r="15" spans="1:35">
       <c r="A15">
         <v>14</v>
       </c>
@@ -3008,24 +2419,24 @@
       <c r="O15">
         <v>0</v>
       </c>
-      <c r="P15"/>
-      <c r="Q15" s="2">
+      <c r="Q15"/>
+      <c r="R15" s="2">
         <v>18</v>
       </c>
-      <c r="R15">
+      <c r="S15">
         <v>1.4</v>
       </c>
-      <c r="S15" s="3">
+      <c r="T15" s="3">
         <v>1.8</v>
       </c>
-      <c r="V15"/>
-      <c r="Y15"/>
-      <c r="AB15"/>
-      <c r="AD15"/>
-      <c r="AF15"/>
-      <c r="AG15" s="5"/>
-    </row>
-    <row r="16" spans="1:33">
+      <c r="W15"/>
+      <c r="Z15"/>
+      <c r="AC15"/>
+      <c r="AE15"/>
+      <c r="AG15"/>
+      <c r="AH15" s="5"/>
+    </row>
+    <row r="16" spans="1:35">
       <c r="A16">
         <v>15</v>
       </c>
@@ -3063,32 +2474,32 @@
       <c r="O16">
         <v>0</v>
       </c>
-      <c r="P16"/>
-      <c r="Q16" s="2">
+      <c r="Q16"/>
+      <c r="R16" s="2">
         <v>6</v>
       </c>
-      <c r="R16">
+      <c r="S16">
         <v>4</v>
       </c>
-      <c r="S16" s="3">
+      <c r="T16" s="3">
         <v>5</v>
       </c>
-      <c r="T16" s="2">
+      <c r="U16" s="2">
         <v>18</v>
       </c>
-      <c r="U16">
+      <c r="V16">
         <v>0.8</v>
       </c>
-      <c r="V16" s="3">
-        <v>1.1</v>
-      </c>
-      <c r="Y16"/>
-      <c r="AB16"/>
-      <c r="AD16"/>
-      <c r="AF16"/>
-      <c r="AG16" s="5"/>
-    </row>
-    <row r="17" spans="1:33">
+      <c r="W16" s="3">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="Z16"/>
+      <c r="AC16"/>
+      <c r="AE16"/>
+      <c r="AG16"/>
+      <c r="AH16" s="5"/>
+    </row>
+    <row r="17" spans="1:34">
       <c r="A17">
         <v>16</v>
       </c>
@@ -3129,40 +2540,40 @@
       <c r="O17">
         <v>1</v>
       </c>
-      <c r="P17"/>
-      <c r="Q17" s="2">
+      <c r="Q17"/>
+      <c r="R17" s="2">
         <v>19</v>
       </c>
-      <c r="R17">
-        <v>1</v>
-      </c>
-      <c r="S17" s="3">
-        <v>1</v>
-      </c>
-      <c r="T17" s="2">
-        <v>2</v>
-      </c>
-      <c r="U17">
+      <c r="S17">
+        <v>1</v>
+      </c>
+      <c r="T17" s="3">
+        <v>1</v>
+      </c>
+      <c r="U17" s="2">
+        <v>2</v>
+      </c>
+      <c r="V17">
         <v>4</v>
       </c>
-      <c r="V17" s="3">
+      <c r="W17" s="3">
         <v>6</v>
       </c>
-      <c r="W17" s="2">
+      <c r="X17" s="2">
         <v>21</v>
       </c>
-      <c r="X17">
-        <v>2</v>
-      </c>
-      <c r="Y17" s="3">
-        <v>3</v>
-      </c>
-      <c r="AB17"/>
-      <c r="AD17"/>
-      <c r="AF17"/>
-      <c r="AG17" s="6"/>
-    </row>
-    <row r="18" spans="1:33">
+      <c r="Y17">
+        <v>2</v>
+      </c>
+      <c r="Z17" s="3">
+        <v>3</v>
+      </c>
+      <c r="AC17"/>
+      <c r="AE17"/>
+      <c r="AG17"/>
+      <c r="AH17" s="6"/>
+    </row>
+    <row r="18" spans="1:34">
       <c r="A18">
         <v>18</v>
       </c>
@@ -3202,24 +2613,24 @@
       <c r="O18">
         <v>0</v>
       </c>
-      <c r="Q18" s="2">
+      <c r="R18" s="2">
         <v>15</v>
       </c>
-      <c r="R18">
+      <c r="S18">
         <v>5</v>
       </c>
-      <c r="S18" s="3">
+      <c r="T18" s="3">
         <v>7</v>
       </c>
-      <c r="AC18">
+      <c r="AD18">
         <v>63</v>
       </c>
-      <c r="AD18" s="3">
+      <c r="AE18" s="3">
         <v>1.5</v>
       </c>
-      <c r="AG18" s="5"/>
-    </row>
-    <row r="19" spans="1:33">
+      <c r="AH18" s="5"/>
+    </row>
+    <row r="19" spans="1:34">
       <c r="A19">
         <v>19</v>
       </c>
@@ -3257,32 +2668,32 @@
       <c r="O19">
         <v>1</v>
       </c>
-      <c r="P19"/>
-      <c r="Q19" s="2">
+      <c r="Q19"/>
+      <c r="R19" s="2">
         <v>23</v>
       </c>
-      <c r="R19">
-        <v>1</v>
-      </c>
-      <c r="S19" s="3">
-        <v>1</v>
-      </c>
-      <c r="T19" s="2">
+      <c r="S19">
+        <v>1</v>
+      </c>
+      <c r="T19" s="3">
+        <v>1</v>
+      </c>
+      <c r="U19" s="2">
         <v>7</v>
       </c>
-      <c r="U19">
-        <v>1</v>
-      </c>
-      <c r="V19" s="3">
-        <v>2</v>
-      </c>
-      <c r="Y19"/>
-      <c r="AB19"/>
-      <c r="AD19"/>
-      <c r="AF19"/>
-      <c r="AG19" s="5"/>
-    </row>
-    <row r="20" spans="1:33">
+      <c r="V19">
+        <v>1</v>
+      </c>
+      <c r="W19" s="3">
+        <v>2</v>
+      </c>
+      <c r="Z19"/>
+      <c r="AC19"/>
+      <c r="AE19"/>
+      <c r="AG19"/>
+      <c r="AH19" s="5"/>
+    </row>
+    <row r="20" spans="1:34">
       <c r="A20">
         <v>20</v>
       </c>
@@ -3322,27 +2733,27 @@
       <c r="O20">
         <v>0</v>
       </c>
-      <c r="P20" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q20" s="2">
+      <c r="Q20" s="3">
+        <v>0</v>
+      </c>
+      <c r="R20" s="2">
         <v>11</v>
       </c>
-      <c r="R20">
+      <c r="S20">
         <v>24</v>
       </c>
-      <c r="S20" s="3">
+      <c r="T20" s="3">
         <v>30</v>
       </c>
-      <c r="AC20">
+      <c r="AD20">
         <v>62</v>
       </c>
-      <c r="AD20" s="3">
+      <c r="AE20" s="3">
         <v>7</v>
       </c>
-      <c r="AG20" s="6"/>
-    </row>
-    <row r="21" spans="1:33">
+      <c r="AH20" s="6"/>
+    </row>
+    <row r="21" spans="1:34">
       <c r="A21">
         <v>21</v>
       </c>
@@ -3382,36 +2793,36 @@
       <c r="O21">
         <v>1</v>
       </c>
-      <c r="Q21" s="2">
+      <c r="R21" s="2">
         <v>26</v>
       </c>
-      <c r="R21">
-        <v>2</v>
-      </c>
-      <c r="S21" s="3">
-        <v>2</v>
-      </c>
-      <c r="T21" s="2">
+      <c r="S21">
+        <v>2</v>
+      </c>
+      <c r="T21" s="3">
+        <v>2</v>
+      </c>
+      <c r="U21" s="2">
         <v>11</v>
       </c>
-      <c r="U21">
+      <c r="V21">
         <v>30</v>
       </c>
-      <c r="V21" s="3">
+      <c r="W21" s="3">
         <v>42</v>
       </c>
-      <c r="W21">
-        <v>2</v>
-      </c>
       <c r="X21">
+        <v>2</v>
+      </c>
+      <c r="Y21">
         <v>5</v>
       </c>
-      <c r="Y21" s="3">
+      <c r="Z21" s="3">
         <v>7</v>
       </c>
-      <c r="AG21" s="5"/>
-    </row>
-    <row r="22" spans="1:33">
+      <c r="AH21" s="5"/>
+    </row>
+    <row r="22" spans="1:34">
       <c r="A22">
         <v>22</v>
       </c>
@@ -3449,32 +2860,32 @@
       <c r="O22">
         <v>1</v>
       </c>
-      <c r="P22"/>
-      <c r="Q22" s="2">
+      <c r="Q22"/>
+      <c r="R22" s="2">
         <v>6</v>
       </c>
-      <c r="R22">
-        <v>2</v>
-      </c>
-      <c r="S22" s="3">
+      <c r="S22">
+        <v>2</v>
+      </c>
+      <c r="T22" s="3">
         <v>4</v>
       </c>
-      <c r="T22" s="2">
+      <c r="U22" s="2">
         <v>28</v>
       </c>
-      <c r="U22">
-        <v>1</v>
-      </c>
-      <c r="V22" s="3">
-        <v>1</v>
-      </c>
-      <c r="Y22"/>
-      <c r="AB22"/>
-      <c r="AD22"/>
-      <c r="AF22"/>
-      <c r="AG22" s="5"/>
-    </row>
-    <row r="23" spans="1:33">
+      <c r="V22">
+        <v>1</v>
+      </c>
+      <c r="W22" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z22"/>
+      <c r="AC22"/>
+      <c r="AE22"/>
+      <c r="AG22"/>
+      <c r="AH22" s="5"/>
+    </row>
+    <row r="23" spans="1:34">
       <c r="A23">
         <v>23</v>
       </c>
@@ -3512,32 +2923,32 @@
       <c r="O23">
         <v>0</v>
       </c>
-      <c r="P23"/>
-      <c r="Q23" s="2">
+      <c r="Q23"/>
+      <c r="R23" s="2">
         <v>6</v>
       </c>
-      <c r="R23">
+      <c r="S23">
         <v>5</v>
       </c>
-      <c r="S23" s="3">
+      <c r="T23" s="3">
         <v>7</v>
       </c>
-      <c r="T23" s="2">
-        <v>2</v>
-      </c>
-      <c r="U23">
-        <v>1</v>
-      </c>
-      <c r="V23" s="3">
-        <v>1</v>
-      </c>
-      <c r="Y23"/>
-      <c r="AB23"/>
-      <c r="AD23"/>
-      <c r="AF23"/>
-      <c r="AG23" s="5"/>
-    </row>
-    <row r="24" spans="1:33">
+      <c r="U23" s="2">
+        <v>2</v>
+      </c>
+      <c r="V23">
+        <v>1</v>
+      </c>
+      <c r="W23" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z23"/>
+      <c r="AC23"/>
+      <c r="AE23"/>
+      <c r="AG23"/>
+      <c r="AH23" s="5"/>
+    </row>
+    <row r="24" spans="1:34">
       <c r="A24">
         <v>24</v>
       </c>
@@ -3577,33 +2988,33 @@
       <c r="O24">
         <v>0</v>
       </c>
-      <c r="Q24" s="2">
+      <c r="R24" s="2">
         <v>15</v>
       </c>
-      <c r="R24">
-        <v>3</v>
-      </c>
-      <c r="S24" s="3">
+      <c r="S24">
+        <v>3</v>
+      </c>
+      <c r="T24" s="3">
         <v>4</v>
       </c>
-      <c r="T24" s="2">
+      <c r="U24" s="2">
         <v>11</v>
       </c>
-      <c r="U24">
+      <c r="V24">
         <v>8</v>
       </c>
-      <c r="V24" s="3">
+      <c r="W24" s="3">
         <v>11</v>
       </c>
-      <c r="AC24">
+      <c r="AD24">
         <v>63</v>
       </c>
-      <c r="AD24" s="3">
-        <v>3</v>
-      </c>
-      <c r="AG24" s="5"/>
-    </row>
-    <row r="25" spans="1:33">
+      <c r="AE24" s="3">
+        <v>3</v>
+      </c>
+      <c r="AH24" s="5"/>
+    </row>
+    <row r="25" spans="1:34">
       <c r="A25">
         <v>25</v>
       </c>
@@ -3641,24 +3052,24 @@
       <c r="O25">
         <v>0</v>
       </c>
-      <c r="P25"/>
-      <c r="Q25" s="2">
+      <c r="Q25"/>
+      <c r="R25" s="2">
         <v>7</v>
       </c>
-      <c r="R25">
-        <v>3</v>
-      </c>
-      <c r="S25" s="3">
+      <c r="S25">
+        <v>3</v>
+      </c>
+      <c r="T25" s="3">
         <v>5</v>
       </c>
-      <c r="V25"/>
-      <c r="Y25"/>
-      <c r="AB25"/>
-      <c r="AD25"/>
-      <c r="AF25"/>
-      <c r="AG25" s="5"/>
-    </row>
-    <row r="26" spans="1:33">
+      <c r="W25"/>
+      <c r="Z25"/>
+      <c r="AC25"/>
+      <c r="AE25"/>
+      <c r="AG25"/>
+      <c r="AH25" s="5"/>
+    </row>
+    <row r="26" spans="1:34">
       <c r="A26">
         <v>26</v>
       </c>
@@ -3696,32 +3107,32 @@
       <c r="O26">
         <v>0</v>
       </c>
-      <c r="P26"/>
-      <c r="Q26" s="2">
+      <c r="Q26"/>
+      <c r="R26" s="2">
         <v>7</v>
       </c>
-      <c r="R26">
-        <v>3</v>
-      </c>
-      <c r="S26" s="3">
+      <c r="S26">
+        <v>3</v>
+      </c>
+      <c r="T26" s="3">
         <v>4</v>
       </c>
-      <c r="T26" s="2">
-        <v>2</v>
-      </c>
-      <c r="U26">
+      <c r="U26" s="2">
+        <v>2</v>
+      </c>
+      <c r="V26">
         <v>4</v>
       </c>
-      <c r="V26" s="3">
+      <c r="W26" s="3">
         <v>6</v>
       </c>
-      <c r="Y26"/>
-      <c r="AB26"/>
-      <c r="AD26"/>
-      <c r="AF26"/>
-      <c r="AG26" s="5"/>
-    </row>
-    <row r="27" spans="1:33">
+      <c r="Z26"/>
+      <c r="AC26"/>
+      <c r="AE26"/>
+      <c r="AG26"/>
+      <c r="AH26" s="5"/>
+    </row>
+    <row r="27" spans="1:34">
       <c r="A27">
         <v>27</v>
       </c>
@@ -3761,39 +3172,39 @@
       <c r="O27">
         <v>1</v>
       </c>
-      <c r="P27" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q27" s="2">
+      <c r="Q27" s="3">
+        <v>0</v>
+      </c>
+      <c r="R27" s="2">
         <v>11</v>
       </c>
-      <c r="R27">
+      <c r="S27">
         <v>12</v>
       </c>
-      <c r="S27" s="3">
+      <c r="T27" s="3">
         <v>18</v>
       </c>
-      <c r="T27" s="2">
+      <c r="U27" s="2">
         <v>56</v>
       </c>
-      <c r="U27">
+      <c r="V27">
         <v>24</v>
       </c>
-      <c r="V27" s="3">
+      <c r="W27" s="3">
         <v>30</v>
       </c>
-      <c r="W27">
+      <c r="X27">
         <v>57</v>
       </c>
-      <c r="X27">
+      <c r="Y27">
         <v>36</v>
       </c>
-      <c r="Y27" s="3">
+      <c r="Z27" s="3">
         <v>44</v>
       </c>
-      <c r="AG27" s="6"/>
-    </row>
-    <row r="28" spans="1:33">
+      <c r="AH27" s="6"/>
+    </row>
+    <row r="28" spans="1:34">
       <c r="A28">
         <v>28</v>
       </c>
@@ -3833,24 +3244,24 @@
       <c r="O28">
         <v>0</v>
       </c>
-      <c r="Q28" s="2">
-        <v>2</v>
-      </c>
-      <c r="R28">
+      <c r="R28" s="2">
+        <v>2</v>
+      </c>
+      <c r="S28">
         <v>6</v>
       </c>
-      <c r="S28" s="3">
+      <c r="T28" s="3">
         <v>8</v>
       </c>
-      <c r="AC28">
+      <c r="AD28">
         <v>21</v>
       </c>
-      <c r="AD28" s="3">
+      <c r="AE28" s="3">
         <v>12</v>
       </c>
-      <c r="AG28" s="5"/>
-    </row>
-    <row r="29" spans="1:33">
+      <c r="AH28" s="5"/>
+    </row>
+    <row r="29" spans="1:34">
       <c r="A29">
         <v>30</v>
       </c>
@@ -3888,40 +3299,40 @@
       <c r="O29">
         <v>1</v>
       </c>
-      <c r="P29"/>
-      <c r="Q29" s="2">
+      <c r="Q29"/>
+      <c r="R29" s="2">
         <v>32</v>
       </c>
-      <c r="R29">
+      <c r="S29">
         <v>30</v>
       </c>
-      <c r="S29" s="3">
+      <c r="T29" s="3">
         <v>30</v>
       </c>
-      <c r="T29" s="2">
-        <v>2</v>
-      </c>
-      <c r="U29">
-        <v>3</v>
-      </c>
-      <c r="V29" s="3">
+      <c r="U29" s="2">
+        <v>2</v>
+      </c>
+      <c r="V29">
+        <v>3</v>
+      </c>
+      <c r="W29" s="3">
         <v>5</v>
       </c>
-      <c r="W29" s="2">
+      <c r="X29" s="2">
         <v>21</v>
       </c>
-      <c r="X29">
-        <v>2</v>
-      </c>
-      <c r="Y29" s="3">
-        <v>3</v>
-      </c>
-      <c r="AB29"/>
-      <c r="AD29"/>
-      <c r="AF29"/>
-      <c r="AG29" s="5"/>
-    </row>
-    <row r="30" spans="1:33">
+      <c r="Y29">
+        <v>2</v>
+      </c>
+      <c r="Z29" s="3">
+        <v>3</v>
+      </c>
+      <c r="AC29"/>
+      <c r="AE29"/>
+      <c r="AG29"/>
+      <c r="AH29" s="5"/>
+    </row>
+    <row r="30" spans="1:34">
       <c r="A30">
         <v>31</v>
       </c>
@@ -3959,32 +3370,32 @@
       <c r="O30">
         <v>1</v>
       </c>
-      <c r="P30"/>
-      <c r="Q30" s="2">
+      <c r="Q30"/>
+      <c r="R30" s="2">
         <v>33</v>
       </c>
-      <c r="R30">
+      <c r="S30">
         <v>50</v>
       </c>
-      <c r="S30" s="3">
+      <c r="T30" s="3">
         <v>70</v>
       </c>
-      <c r="T30" s="2">
-        <v>2</v>
-      </c>
-      <c r="U30">
-        <v>2</v>
-      </c>
-      <c r="V30" s="3">
+      <c r="U30" s="2">
+        <v>2</v>
+      </c>
+      <c r="V30">
+        <v>2</v>
+      </c>
+      <c r="W30" s="3">
         <v>4</v>
       </c>
-      <c r="Y30"/>
-      <c r="AB30"/>
-      <c r="AD30"/>
-      <c r="AF30"/>
-      <c r="AG30" s="6"/>
-    </row>
-    <row r="31" spans="1:33">
+      <c r="Z30"/>
+      <c r="AC30"/>
+      <c r="AE30"/>
+      <c r="AG30"/>
+      <c r="AH30" s="6"/>
+    </row>
+    <row r="31" spans="1:34">
       <c r="A31">
         <v>32</v>
       </c>
@@ -4022,32 +3433,32 @@
       <c r="O31">
         <v>1</v>
       </c>
-      <c r="P31"/>
-      <c r="Q31" s="2">
+      <c r="Q31"/>
+      <c r="R31" s="2">
         <v>33</v>
       </c>
-      <c r="R31">
+      <c r="S31">
         <v>20</v>
       </c>
-      <c r="S31" s="3">
+      <c r="T31" s="3">
         <v>30</v>
       </c>
-      <c r="T31" s="2">
+      <c r="U31" s="2">
         <v>35</v>
       </c>
-      <c r="U31">
-        <v>1</v>
-      </c>
-      <c r="V31" s="3">
-        <v>1</v>
-      </c>
-      <c r="Y31"/>
-      <c r="AB31"/>
-      <c r="AD31"/>
-      <c r="AF31"/>
-      <c r="AG31" s="6"/>
-    </row>
-    <row r="32" spans="1:32">
+      <c r="V31">
+        <v>1</v>
+      </c>
+      <c r="W31" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z31"/>
+      <c r="AC31"/>
+      <c r="AE31"/>
+      <c r="AG31"/>
+      <c r="AH31" s="6"/>
+    </row>
+    <row r="32" spans="1:34">
       <c r="A32">
         <v>33</v>
       </c>
@@ -4085,15 +3496,15 @@
       <c r="O32">
         <v>1</v>
       </c>
-      <c r="P32"/>
-      <c r="S32"/>
-      <c r="V32"/>
-      <c r="Y32"/>
-      <c r="AB32"/>
-      <c r="AD32"/>
-      <c r="AF32"/>
-    </row>
-    <row r="33" spans="1:30">
+      <c r="Q32"/>
+      <c r="T32"/>
+      <c r="W32"/>
+      <c r="Z32"/>
+      <c r="AC32"/>
+      <c r="AE32"/>
+      <c r="AG32"/>
+    </row>
+    <row r="33" spans="1:33">
       <c r="A33">
         <v>34</v>
       </c>
@@ -4133,23 +3544,23 @@
       <c r="O33">
         <v>1</v>
       </c>
-      <c r="Q33" s="2">
+      <c r="R33" s="2">
         <v>11</v>
       </c>
-      <c r="R33">
+      <c r="S33">
         <v>38</v>
       </c>
-      <c r="S33" s="3">
+      <c r="T33" s="3">
         <v>52</v>
       </c>
-      <c r="AC33">
+      <c r="AD33">
         <v>64</v>
       </c>
-      <c r="AD33" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34" spans="1:19">
+      <c r="AE33" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:33">
       <c r="A34">
         <v>35</v>
       </c>
@@ -4189,20 +3600,20 @@
       <c r="O34">
         <v>0</v>
       </c>
-      <c r="P34" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q34" s="2">
+      <c r="Q34" s="3">
+        <v>0</v>
+      </c>
+      <c r="R34" s="2">
         <v>15</v>
       </c>
-      <c r="R34">
-        <v>3</v>
-      </c>
-      <c r="S34" s="3">
+      <c r="S34">
+        <v>3</v>
+      </c>
+      <c r="T34" s="3">
         <v>4</v>
       </c>
     </row>
-    <row r="35" spans="1:19">
+    <row r="35" spans="1:33">
       <c r="A35">
         <v>36</v>
       </c>
@@ -4242,17 +3653,17 @@
       <c r="O35">
         <v>0</v>
       </c>
-      <c r="Q35" s="2">
+      <c r="R35" s="2">
         <v>11</v>
       </c>
-      <c r="R35">
+      <c r="S35">
         <v>18</v>
       </c>
-      <c r="S35" s="3">
+      <c r="T35" s="3">
         <v>22</v>
       </c>
     </row>
-    <row r="36" spans="1:22">
+    <row r="36" spans="1:33">
       <c r="A36">
         <v>37</v>
       </c>
@@ -4292,26 +3703,26 @@
       <c r="O36">
         <v>0</v>
       </c>
-      <c r="Q36" s="2">
+      <c r="R36" s="2">
         <v>15</v>
       </c>
-      <c r="R36">
-        <v>3</v>
-      </c>
-      <c r="S36" s="3">
+      <c r="S36">
+        <v>3</v>
+      </c>
+      <c r="T36" s="3">
         <v>4</v>
       </c>
-      <c r="T36" s="2">
-        <v>2</v>
-      </c>
-      <c r="U36">
+      <c r="U36" s="2">
+        <v>2</v>
+      </c>
+      <c r="V36">
         <v>6</v>
       </c>
-      <c r="V36" s="3">
+      <c r="W36" s="3">
         <v>8</v>
       </c>
     </row>
-    <row r="37" spans="1:32">
+    <row r="37" spans="1:33">
       <c r="A37">
         <v>38</v>
       </c>
@@ -4349,31 +3760,31 @@
       <c r="O37">
         <v>0</v>
       </c>
-      <c r="P37"/>
-      <c r="Q37" s="2">
+      <c r="Q37"/>
+      <c r="R37" s="2">
         <v>7</v>
       </c>
-      <c r="R37">
-        <v>3</v>
-      </c>
-      <c r="S37" s="3">
+      <c r="S37">
+        <v>3</v>
+      </c>
+      <c r="T37" s="3">
         <v>4</v>
       </c>
-      <c r="T37" s="2">
-        <v>2</v>
-      </c>
-      <c r="U37">
+      <c r="U37" s="2">
+        <v>2</v>
+      </c>
+      <c r="V37">
         <v>6</v>
       </c>
-      <c r="V37" s="3">
+      <c r="W37" s="3">
         <v>8</v>
       </c>
-      <c r="Y37"/>
-      <c r="AB37"/>
-      <c r="AD37"/>
-      <c r="AF37"/>
-    </row>
-    <row r="38" spans="1:32">
+      <c r="Z37"/>
+      <c r="AC37"/>
+      <c r="AE37"/>
+      <c r="AG37"/>
+    </row>
+    <row r="38" spans="1:33">
       <c r="A38">
         <v>39</v>
       </c>
@@ -4411,31 +3822,31 @@
       <c r="O38">
         <v>1</v>
       </c>
-      <c r="P38"/>
-      <c r="Q38" s="2">
+      <c r="Q38"/>
+      <c r="R38" s="2">
         <v>21</v>
       </c>
-      <c r="R38">
+      <c r="S38">
         <v>4</v>
       </c>
-      <c r="S38" s="3">
+      <c r="T38" s="3">
         <v>5</v>
       </c>
-      <c r="T38" s="2">
-        <v>2</v>
-      </c>
-      <c r="U38">
-        <v>3</v>
-      </c>
-      <c r="V38" s="3">
+      <c r="U38" s="2">
+        <v>2</v>
+      </c>
+      <c r="V38">
+        <v>3</v>
+      </c>
+      <c r="W38" s="3">
         <v>5</v>
       </c>
-      <c r="Y38"/>
-      <c r="AB38"/>
-      <c r="AD38"/>
-      <c r="AF38"/>
-    </row>
-    <row r="39" spans="1:32">
+      <c r="Z38"/>
+      <c r="AC38"/>
+      <c r="AE38"/>
+      <c r="AG38"/>
+    </row>
+    <row r="39" spans="1:33">
       <c r="A39">
         <v>40</v>
       </c>
@@ -4473,31 +3884,31 @@
       <c r="O39">
         <v>1</v>
       </c>
-      <c r="P39"/>
-      <c r="Q39" s="2">
+      <c r="Q39"/>
+      <c r="R39" s="2">
         <v>5</v>
       </c>
-      <c r="R39">
-        <v>1</v>
-      </c>
-      <c r="S39" s="3">
-        <v>2</v>
-      </c>
-      <c r="T39" s="2">
-        <v>2</v>
-      </c>
-      <c r="U39">
+      <c r="S39">
+        <v>1</v>
+      </c>
+      <c r="T39" s="3">
+        <v>2</v>
+      </c>
+      <c r="U39" s="2">
+        <v>2</v>
+      </c>
+      <c r="V39">
         <v>6</v>
       </c>
-      <c r="V39" s="3">
+      <c r="W39" s="3">
         <v>7</v>
       </c>
-      <c r="Y39"/>
-      <c r="AB39"/>
-      <c r="AD39"/>
-      <c r="AF39"/>
-    </row>
-    <row r="40" spans="1:32">
+      <c r="Z39"/>
+      <c r="AC39"/>
+      <c r="AE39"/>
+      <c r="AG39"/>
+    </row>
+    <row r="40" spans="1:33">
       <c r="A40">
         <v>41</v>
       </c>
@@ -4535,31 +3946,31 @@
       <c r="O40">
         <v>1</v>
       </c>
-      <c r="P40"/>
-      <c r="Q40" s="2">
+      <c r="Q40"/>
+      <c r="R40" s="2">
         <v>7</v>
       </c>
-      <c r="R40">
+      <c r="S40">
         <v>4</v>
       </c>
-      <c r="S40" s="3">
+      <c r="T40" s="3">
         <v>5</v>
       </c>
-      <c r="T40" s="2">
+      <c r="U40" s="2">
         <v>38</v>
       </c>
-      <c r="U40">
+      <c r="V40">
         <v>4</v>
       </c>
-      <c r="V40" s="3">
+      <c r="W40" s="3">
         <v>5</v>
       </c>
-      <c r="Y40"/>
-      <c r="AB40"/>
-      <c r="AD40"/>
-      <c r="AF40"/>
-    </row>
-    <row r="41" spans="1:32">
+      <c r="Z40"/>
+      <c r="AC40"/>
+      <c r="AE40"/>
+      <c r="AG40"/>
+    </row>
+    <row r="41" spans="1:33">
       <c r="A41">
         <v>42</v>
       </c>
@@ -4597,31 +4008,31 @@
       <c r="O41">
         <v>0</v>
       </c>
-      <c r="P41"/>
-      <c r="Q41" s="2">
+      <c r="Q41"/>
+      <c r="R41" s="2">
         <v>6</v>
       </c>
-      <c r="R41">
-        <v>3</v>
-      </c>
-      <c r="S41" s="3">
-        <v>3</v>
-      </c>
-      <c r="T41" s="2">
+      <c r="S41">
+        <v>3</v>
+      </c>
+      <c r="T41" s="3">
+        <v>3</v>
+      </c>
+      <c r="U41" s="2">
         <v>39</v>
       </c>
-      <c r="U41">
-        <v>2</v>
-      </c>
-      <c r="V41" s="3">
-        <v>3</v>
-      </c>
-      <c r="Y41"/>
-      <c r="AB41"/>
-      <c r="AD41"/>
-      <c r="AF41"/>
-    </row>
-    <row r="42" spans="1:32">
+      <c r="V41">
+        <v>2</v>
+      </c>
+      <c r="W41" s="3">
+        <v>3</v>
+      </c>
+      <c r="Z41"/>
+      <c r="AC41"/>
+      <c r="AE41"/>
+      <c r="AG41"/>
+    </row>
+    <row r="42" spans="1:33">
       <c r="A42">
         <v>43</v>
       </c>
@@ -4659,31 +4070,31 @@
       <c r="O42">
         <v>1</v>
       </c>
-      <c r="P42"/>
-      <c r="Q42" s="2">
+      <c r="Q42"/>
+      <c r="R42" s="2">
         <v>7</v>
       </c>
-      <c r="R42">
-        <v>1</v>
-      </c>
-      <c r="S42" s="3">
-        <v>3</v>
-      </c>
-      <c r="T42" s="2">
+      <c r="S42">
+        <v>1</v>
+      </c>
+      <c r="T42" s="3">
+        <v>3</v>
+      </c>
+      <c r="U42" s="2">
         <v>41</v>
       </c>
-      <c r="U42">
-        <v>1</v>
-      </c>
-      <c r="V42" s="3">
-        <v>1</v>
-      </c>
-      <c r="Y42"/>
-      <c r="AB42"/>
-      <c r="AD42"/>
-      <c r="AF42"/>
-    </row>
-    <row r="43" spans="1:32">
+      <c r="V42">
+        <v>1</v>
+      </c>
+      <c r="W42" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z42"/>
+      <c r="AC42"/>
+      <c r="AE42"/>
+      <c r="AG42"/>
+    </row>
+    <row r="43" spans="1:33">
       <c r="A43">
         <v>44</v>
       </c>
@@ -4721,39 +4132,39 @@
       <c r="O43">
         <v>1</v>
       </c>
-      <c r="P43"/>
-      <c r="Q43" s="2">
+      <c r="Q43"/>
+      <c r="R43" s="2">
         <v>6</v>
       </c>
-      <c r="R43">
+      <c r="S43">
         <v>5</v>
       </c>
-      <c r="S43" s="3">
+      <c r="T43" s="3">
         <v>5</v>
       </c>
-      <c r="T43" s="2">
+      <c r="U43" s="2">
         <v>14</v>
       </c>
-      <c r="U43">
-        <v>1</v>
-      </c>
-      <c r="V43" s="3">
-        <v>1</v>
-      </c>
-      <c r="W43" s="2">
+      <c r="V43">
+        <v>1</v>
+      </c>
+      <c r="W43" s="3">
+        <v>1</v>
+      </c>
+      <c r="X43" s="2">
         <v>18</v>
       </c>
-      <c r="X43">
+      <c r="Y43">
         <v>0.9</v>
       </c>
-      <c r="Y43" s="3">
+      <c r="Z43" s="3">
         <v>1.2</v>
       </c>
-      <c r="AB43"/>
-      <c r="AD43"/>
-      <c r="AF43"/>
-    </row>
-    <row r="44" spans="1:22">
+      <c r="AC43"/>
+      <c r="AE43"/>
+      <c r="AG43"/>
+    </row>
+    <row r="44" spans="1:33">
       <c r="A44">
         <v>45</v>
       </c>
@@ -4793,26 +4204,26 @@
       <c r="O44">
         <v>1</v>
       </c>
-      <c r="Q44" s="2">
+      <c r="R44" s="2">
         <v>15</v>
       </c>
-      <c r="R44">
-        <v>2</v>
-      </c>
-      <c r="S44" s="3">
-        <v>2</v>
-      </c>
-      <c r="T44" s="2">
+      <c r="S44">
+        <v>2</v>
+      </c>
+      <c r="T44" s="3">
+        <v>2</v>
+      </c>
+      <c r="U44" s="2">
         <v>42</v>
       </c>
-      <c r="U44">
+      <c r="V44">
         <v>8</v>
       </c>
-      <c r="V44" s="3">
+      <c r="W44" s="3">
         <v>12</v>
       </c>
     </row>
-    <row r="45" spans="1:32">
+    <row r="45" spans="1:33">
       <c r="A45">
         <v>46</v>
       </c>
@@ -4850,39 +4261,39 @@
       <c r="O45">
         <v>1</v>
       </c>
-      <c r="P45"/>
-      <c r="Q45" s="2">
+      <c r="Q45"/>
+      <c r="R45" s="2">
         <v>7</v>
       </c>
-      <c r="R45">
+      <c r="S45">
         <v>7</v>
       </c>
-      <c r="S45" s="3">
+      <c r="T45" s="3">
         <v>9</v>
       </c>
-      <c r="T45" s="2">
+      <c r="U45" s="2">
         <v>26</v>
       </c>
-      <c r="U45">
-        <v>2</v>
-      </c>
-      <c r="V45" s="3">
-        <v>2</v>
-      </c>
-      <c r="W45" s="2">
-        <v>2</v>
-      </c>
-      <c r="X45">
+      <c r="V45">
+        <v>2</v>
+      </c>
+      <c r="W45" s="3">
+        <v>2</v>
+      </c>
+      <c r="X45" s="2">
+        <v>2</v>
+      </c>
+      <c r="Y45">
         <v>7</v>
       </c>
-      <c r="Y45" s="3">
+      <c r="Z45" s="3">
         <v>8</v>
       </c>
-      <c r="AB45"/>
-      <c r="AD45"/>
-      <c r="AF45"/>
-    </row>
-    <row r="46" spans="1:32">
+      <c r="AC45"/>
+      <c r="AE45"/>
+      <c r="AG45"/>
+    </row>
+    <row r="46" spans="1:33">
       <c r="A46">
         <v>47</v>
       </c>
@@ -4920,39 +4331,39 @@
       <c r="O46">
         <v>1</v>
       </c>
-      <c r="P46"/>
-      <c r="Q46" s="2">
+      <c r="Q46"/>
+      <c r="R46" s="2">
         <v>32</v>
       </c>
-      <c r="R46">
+      <c r="S46">
         <v>40</v>
       </c>
-      <c r="S46" s="3">
+      <c r="T46" s="3">
         <v>40</v>
       </c>
-      <c r="T46" s="2">
+      <c r="U46" s="2">
         <v>33</v>
       </c>
-      <c r="U46">
+      <c r="V46">
         <v>30</v>
       </c>
-      <c r="V46" s="3">
+      <c r="W46" s="3">
         <v>30</v>
       </c>
-      <c r="W46" s="2">
+      <c r="X46" s="2">
         <v>19</v>
       </c>
-      <c r="X46">
-        <v>1</v>
-      </c>
-      <c r="Y46" s="3">
-        <v>1</v>
-      </c>
-      <c r="AB46"/>
-      <c r="AD46"/>
-      <c r="AF46"/>
-    </row>
-    <row r="47" spans="1:32">
+      <c r="Y46">
+        <v>1</v>
+      </c>
+      <c r="Z46" s="3">
+        <v>1</v>
+      </c>
+      <c r="AC46"/>
+      <c r="AE46"/>
+      <c r="AG46"/>
+    </row>
+    <row r="47" spans="1:33">
       <c r="A47">
         <v>48</v>
       </c>
@@ -4990,23 +4401,23 @@
       <c r="O47">
         <v>0</v>
       </c>
-      <c r="P47"/>
-      <c r="Q47" s="2">
+      <c r="Q47"/>
+      <c r="R47" s="2">
         <v>11</v>
       </c>
-      <c r="R47">
+      <c r="S47">
         <v>10</v>
       </c>
-      <c r="S47" s="3">
+      <c r="T47" s="3">
         <v>14</v>
       </c>
-      <c r="V47"/>
-      <c r="Y47"/>
-      <c r="AB47"/>
-      <c r="AD47"/>
-      <c r="AF47"/>
-    </row>
-    <row r="48" spans="1:32">
+      <c r="W47"/>
+      <c r="Z47"/>
+      <c r="AC47"/>
+      <c r="AE47"/>
+      <c r="AG47"/>
+    </row>
+    <row r="48" spans="1:33">
       <c r="A48">
         <v>49</v>
       </c>
@@ -5044,31 +4455,31 @@
       <c r="O48">
         <v>0</v>
       </c>
-      <c r="P48"/>
-      <c r="Q48" s="2">
+      <c r="Q48"/>
+      <c r="R48" s="2">
         <v>11</v>
       </c>
-      <c r="R48">
+      <c r="S48">
         <v>8</v>
       </c>
-      <c r="S48" s="3">
+      <c r="T48" s="3">
         <v>11</v>
       </c>
-      <c r="T48" s="2">
+      <c r="U48" s="2">
         <v>6</v>
       </c>
-      <c r="U48">
-        <v>3</v>
-      </c>
-      <c r="V48" s="3">
-        <v>3</v>
-      </c>
-      <c r="Y48"/>
-      <c r="AB48"/>
-      <c r="AD48"/>
-      <c r="AF48"/>
-    </row>
-    <row r="49" spans="1:22">
+      <c r="V48">
+        <v>3</v>
+      </c>
+      <c r="W48" s="3">
+        <v>3</v>
+      </c>
+      <c r="Z48"/>
+      <c r="AC48"/>
+      <c r="AE48"/>
+      <c r="AG48"/>
+    </row>
+    <row r="49" spans="1:33">
       <c r="A49">
         <v>50</v>
       </c>
@@ -5108,26 +4519,26 @@
       <c r="O49">
         <v>0</v>
       </c>
-      <c r="Q49" s="2">
+      <c r="R49" s="2">
         <v>11</v>
       </c>
-      <c r="R49">
+      <c r="S49">
         <v>7</v>
       </c>
-      <c r="S49" s="3">
+      <c r="T49" s="3">
         <v>11</v>
       </c>
-      <c r="T49" s="2">
+      <c r="U49" s="2">
         <v>45</v>
       </c>
-      <c r="U49">
-        <v>2</v>
-      </c>
-      <c r="V49" s="3">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="50" spans="1:32">
+      <c r="V49">
+        <v>2</v>
+      </c>
+      <c r="W49" s="3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="50" spans="1:33">
       <c r="A50">
         <v>51</v>
       </c>
@@ -5165,31 +4576,31 @@
       <c r="O50">
         <v>1</v>
       </c>
-      <c r="P50"/>
-      <c r="Q50" s="2">
+      <c r="Q50"/>
+      <c r="R50" s="2">
         <v>6</v>
       </c>
-      <c r="R50">
+      <c r="S50">
         <v>5</v>
       </c>
-      <c r="S50" s="3">
+      <c r="T50" s="3">
         <v>7</v>
       </c>
-      <c r="T50" s="2">
+      <c r="U50" s="2">
         <v>18</v>
       </c>
-      <c r="U50">
-        <v>1.1</v>
-      </c>
-      <c r="V50" s="3">
+      <c r="V50">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="W50" s="3">
         <v>1.7</v>
       </c>
-      <c r="Y50"/>
-      <c r="AB50"/>
-      <c r="AD50"/>
-      <c r="AF50"/>
-    </row>
-    <row r="51" spans="1:32">
+      <c r="Z50"/>
+      <c r="AC50"/>
+      <c r="AE50"/>
+      <c r="AG50"/>
+    </row>
+    <row r="51" spans="1:33">
       <c r="A51">
         <v>52</v>
       </c>
@@ -5227,31 +4638,31 @@
       <c r="O51">
         <v>1</v>
       </c>
-      <c r="P51"/>
-      <c r="Q51" s="2">
+      <c r="Q51"/>
+      <c r="R51" s="2">
         <v>6</v>
       </c>
-      <c r="R51">
-        <v>1</v>
-      </c>
-      <c r="S51" s="3">
-        <v>3</v>
-      </c>
-      <c r="T51" s="2">
+      <c r="S51">
+        <v>1</v>
+      </c>
+      <c r="T51" s="3">
+        <v>3</v>
+      </c>
+      <c r="U51" s="2">
         <v>49</v>
       </c>
-      <c r="U51">
-        <v>1</v>
-      </c>
-      <c r="V51" s="3">
-        <v>1</v>
-      </c>
-      <c r="Y51"/>
-      <c r="AB51"/>
-      <c r="AD51"/>
-      <c r="AF51"/>
-    </row>
-    <row r="52" spans="1:32">
+      <c r="V51">
+        <v>1</v>
+      </c>
+      <c r="W51" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z51"/>
+      <c r="AC51"/>
+      <c r="AE51"/>
+      <c r="AG51"/>
+    </row>
+    <row r="52" spans="1:33">
       <c r="A52">
         <v>53</v>
       </c>
@@ -5289,31 +4700,31 @@
       <c r="O52">
         <v>1</v>
       </c>
-      <c r="P52"/>
-      <c r="Q52" s="2">
+      <c r="Q52"/>
+      <c r="R52" s="2">
         <v>9</v>
       </c>
-      <c r="R52">
-        <v>2</v>
-      </c>
-      <c r="S52" s="3">
-        <v>2</v>
-      </c>
-      <c r="T52" s="2">
+      <c r="S52">
+        <v>2</v>
+      </c>
+      <c r="T52" s="3">
+        <v>2</v>
+      </c>
+      <c r="U52" s="2">
         <v>21</v>
       </c>
-      <c r="U52">
-        <v>2</v>
-      </c>
-      <c r="V52" s="3">
-        <v>2</v>
-      </c>
-      <c r="Y52"/>
-      <c r="AB52"/>
-      <c r="AD52"/>
-      <c r="AF52"/>
-    </row>
-    <row r="53" spans="1:22">
+      <c r="V52">
+        <v>2</v>
+      </c>
+      <c r="W52" s="3">
+        <v>2</v>
+      </c>
+      <c r="Z52"/>
+      <c r="AC52"/>
+      <c r="AE52"/>
+      <c r="AG52"/>
+    </row>
+    <row r="53" spans="1:33">
       <c r="A53">
         <v>54</v>
       </c>
@@ -5353,29 +4764,29 @@
       <c r="O53">
         <v>1</v>
       </c>
-      <c r="P53" s="3">
+      <c r="Q53" s="3">
         <v>6</v>
       </c>
-      <c r="Q53">
+      <c r="R53">
         <v>50</v>
       </c>
-      <c r="R53">
-        <v>3</v>
-      </c>
-      <c r="S53" s="3">
+      <c r="S53">
+        <v>3</v>
+      </c>
+      <c r="T53" s="3">
         <v>4</v>
       </c>
-      <c r="T53">
+      <c r="U53">
         <v>51</v>
       </c>
-      <c r="U53">
+      <c r="V53">
         <v>-0.5</v>
       </c>
-      <c r="V53" s="3">
+      <c r="W53" s="3">
         <v>-0.5</v>
       </c>
     </row>
-    <row r="54" spans="1:25">
+    <row r="54" spans="1:33">
       <c r="A54">
         <v>55</v>
       </c>
@@ -5418,35 +4829,35 @@
       <c r="O54">
         <v>1</v>
       </c>
-      <c r="Q54">
+      <c r="R54">
         <v>15</v>
       </c>
-      <c r="R54">
-        <v>3</v>
-      </c>
-      <c r="S54" s="3">
+      <c r="S54">
+        <v>3</v>
+      </c>
+      <c r="T54" s="3">
         <v>4</v>
       </c>
-      <c r="T54">
+      <c r="U54">
         <v>14</v>
       </c>
-      <c r="U54">
-        <v>1</v>
-      </c>
-      <c r="V54" s="3">
-        <v>1</v>
-      </c>
-      <c r="W54">
+      <c r="V54">
+        <v>1</v>
+      </c>
+      <c r="W54" s="3">
+        <v>1</v>
+      </c>
+      <c r="X54">
         <v>52</v>
       </c>
-      <c r="X54">
-        <v>3</v>
-      </c>
-      <c r="Y54" s="3">
+      <c r="Y54">
+        <v>3</v>
+      </c>
+      <c r="Z54" s="3">
         <v>5</v>
       </c>
     </row>
-    <row r="55" spans="1:31">
+    <row r="55" spans="1:33">
       <c r="A55">
         <v>56</v>
       </c>
@@ -5486,27 +4897,27 @@
       <c r="O55">
         <v>1</v>
       </c>
-      <c r="Q55">
+      <c r="R55">
         <v>15</v>
       </c>
-      <c r="R55">
-        <v>1</v>
-      </c>
-      <c r="S55" s="3">
-        <v>3</v>
-      </c>
-      <c r="T55">
+      <c r="S55">
+        <v>1</v>
+      </c>
+      <c r="T55" s="3">
+        <v>3</v>
+      </c>
+      <c r="U55">
         <v>60</v>
       </c>
-      <c r="U55">
-        <v>1</v>
-      </c>
-      <c r="V55" s="3">
-        <v>1</v>
-      </c>
-      <c r="AE55" s="3"/>
-    </row>
-    <row r="56" spans="1:31">
+      <c r="V55">
+        <v>1</v>
+      </c>
+      <c r="W55" s="3">
+        <v>1</v>
+      </c>
+      <c r="AF55" s="3"/>
+    </row>
+    <row r="56" spans="1:33">
       <c r="A56">
         <v>57</v>
       </c>
@@ -5549,36 +4960,36 @@
       <c r="O56">
         <v>1</v>
       </c>
-      <c r="Q56">
+      <c r="R56">
         <v>45</v>
       </c>
-      <c r="R56">
-        <v>3</v>
-      </c>
-      <c r="S56" s="3">
+      <c r="S56">
+        <v>3</v>
+      </c>
+      <c r="T56" s="3">
         <v>4</v>
       </c>
-      <c r="T56">
+      <c r="U56">
         <v>11</v>
       </c>
-      <c r="U56">
+      <c r="V56">
         <v>12</v>
       </c>
-      <c r="V56" s="3">
+      <c r="W56" s="3">
         <v>18</v>
       </c>
-      <c r="W56">
+      <c r="X56">
         <v>14</v>
       </c>
-      <c r="X56">
-        <v>1</v>
-      </c>
-      <c r="Y56" s="3">
-        <v>1</v>
-      </c>
-      <c r="AE56" s="3"/>
-    </row>
-    <row r="57" spans="1:22">
+      <c r="Y56">
+        <v>1</v>
+      </c>
+      <c r="Z56" s="3">
+        <v>1</v>
+      </c>
+      <c r="AF56" s="3"/>
+    </row>
+    <row r="57" spans="1:33">
       <c r="A57">
         <v>58</v>
       </c>
@@ -5621,26 +5032,26 @@
       <c r="O57">
         <v>1</v>
       </c>
-      <c r="Q57">
-        <v>2</v>
-      </c>
       <c r="R57">
+        <v>2</v>
+      </c>
+      <c r="S57">
         <v>5</v>
       </c>
-      <c r="S57" s="3">
+      <c r="T57" s="3">
         <v>6</v>
       </c>
-      <c r="T57">
-        <v>2</v>
-      </c>
       <c r="U57">
+        <v>2</v>
+      </c>
+      <c r="V57">
         <v>5</v>
       </c>
-      <c r="V57" s="3">
+      <c r="W57" s="3">
         <v>6</v>
       </c>
     </row>
-    <row r="58" spans="1:15">
+    <row r="58" spans="1:33">
       <c r="A58">
         <v>59</v>
       </c>
@@ -5681,7 +5092,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:19">
+    <row r="59" spans="1:33">
       <c r="A59">
         <v>60</v>
       </c>
@@ -5721,17 +5132,17 @@
       <c r="O59">
         <v>0</v>
       </c>
-      <c r="Q59">
-        <v>2</v>
-      </c>
       <c r="R59">
+        <v>2</v>
+      </c>
+      <c r="S59">
         <v>7</v>
       </c>
-      <c r="S59" s="3">
+      <c r="T59" s="3">
         <v>9</v>
       </c>
     </row>
-    <row r="60" spans="1:15">
+    <row r="60" spans="1:33">
       <c r="A60">
         <v>61</v>
       </c>
@@ -5772,7 +5183,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:15">
+    <row r="61" spans="1:33">
       <c r="A61">
         <v>62</v>
       </c>
@@ -5818,25 +5229,23 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
-  <headerFooter/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:I67"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="3.425" customWidth="1"/>
-    <col min="2" max="2" width="27.425" customWidth="1"/>
+    <col min="1" max="1" width="3.42578125" customWidth="1"/>
+    <col min="2" max="2" width="27.42578125" customWidth="1"/>
     <col min="3" max="3" width="35" customWidth="1"/>
     <col min="4" max="4" width="33" customWidth="1"/>
-    <col min="5" max="5" width="19.2833333333333" customWidth="1"/>
-    <col min="6" max="6" width="18.8583333333333" customWidth="1"/>
-    <col min="7" max="8" width="10.2833333333333" customWidth="1"/>
-    <col min="9" max="9" width="15.1416666666667" customWidth="1"/>
+    <col min="5" max="5" width="19.28515625" customWidth="1"/>
+    <col min="6" max="6" width="18.85546875" customWidth="1"/>
+    <col min="7" max="8" width="10.28515625" customWidth="1"/>
+    <col min="9" max="9" width="15.140625" customWidth="1"/>
     <col min="10" max="10" width="22" customWidth="1"/>
   </cols>
   <sheetData>
@@ -7158,7 +6567,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="63" customFormat="1" spans="1:9">
+    <row r="63" spans="1:9">
       <c r="A63">
         <v>61</v>
       </c>
@@ -7218,7 +6627,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="66" customFormat="1" spans="1:9">
+    <row r="66" spans="1:9">
       <c r="A66">
         <v>64</v>
       </c>
@@ -7263,26 +6672,24 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
-  <headerFooter/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:O34"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="9.425" customWidth="1"/>
-    <col min="2" max="2" width="27.425" customWidth="1"/>
-    <col min="3" max="3" width="14.425" customWidth="1"/>
-    <col min="4" max="5" width="16.1416666666667" customWidth="1"/>
-    <col min="6" max="6" width="12.425" customWidth="1"/>
-    <col min="7" max="7" width="14.425" customWidth="1"/>
+    <col min="1" max="1" width="9.42578125" customWidth="1"/>
+    <col min="2" max="2" width="27.42578125" customWidth="1"/>
+    <col min="3" max="3" width="14.42578125" customWidth="1"/>
+    <col min="4" max="5" width="16.140625" customWidth="1"/>
+    <col min="6" max="6" width="12.42578125" customWidth="1"/>
+    <col min="7" max="7" width="14.42578125" customWidth="1"/>
     <col min="8" max="8" width="10" customWidth="1"/>
     <col min="9" max="9" width="13" customWidth="1"/>
-    <col min="10" max="10" width="10.1416666666667" customWidth="1"/>
+    <col min="10" max="10" width="10.140625" customWidth="1"/>
     <col min="11" max="11" width="13" customWidth="1"/>
   </cols>
   <sheetData>
@@ -7333,7 +6740,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:15">
       <c r="A2">
         <v>0</v>
       </c>
@@ -7362,7 +6769,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:15">
       <c r="A3">
         <v>1</v>
       </c>
@@ -7385,7 +6792,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:15">
       <c r="A4">
         <v>2</v>
       </c>
@@ -7402,7 +6809,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
+    <row r="5" spans="1:15">
       <c r="A5">
         <v>3</v>
       </c>
@@ -7437,7 +6844,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:15">
       <c r="A6">
         <v>4</v>
       </c>
@@ -7460,7 +6867,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:15">
       <c r="A7">
         <v>5</v>
       </c>
@@ -7483,7 +6890,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="8" spans="1:7">
+    <row r="8" spans="1:15">
       <c r="A8">
         <v>6</v>
       </c>
@@ -7506,7 +6913,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:15">
       <c r="A9">
         <v>7</v>
       </c>
@@ -7529,7 +6936,7 @@
         <v>-0.5</v>
       </c>
     </row>
-    <row r="10" spans="1:7">
+    <row r="10" spans="1:15">
       <c r="A10">
         <v>8</v>
       </c>
@@ -7552,7 +6959,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:9">
+    <row r="11" spans="1:15">
       <c r="A11">
         <v>9</v>
       </c>
@@ -7581,7 +6988,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="12" spans="1:9">
+    <row r="12" spans="1:15">
       <c r="A12">
         <v>10</v>
       </c>
@@ -7610,7 +7017,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="13" spans="1:7">
+    <row r="13" spans="1:15">
       <c r="A13">
         <v>11</v>
       </c>
@@ -7633,7 +7040,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:7">
+    <row r="14" spans="1:15">
       <c r="A14">
         <v>12</v>
       </c>
@@ -7656,7 +7063,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:7">
+    <row r="15" spans="1:15">
       <c r="A15">
         <v>13</v>
       </c>
@@ -7679,7 +7086,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="1:7">
+    <row r="16" spans="1:15">
       <c r="A16">
         <v>14</v>
       </c>
@@ -7748,7 +7155,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:5">
+    <row r="19" spans="1:7">
       <c r="A19">
         <v>17</v>
       </c>
@@ -7765,7 +7172,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:5">
+    <row r="20" spans="1:7">
       <c r="A20">
         <v>18</v>
       </c>
@@ -7782,7 +7189,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:5">
+    <row r="21" spans="1:7">
       <c r="A21">
         <v>19</v>
       </c>
@@ -7868,7 +7275,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:5">
+    <row r="25" spans="1:7">
       <c r="A25">
         <v>23</v>
       </c>
@@ -7885,7 +7292,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:5">
+    <row r="26" spans="1:7">
       <c r="A26">
         <v>24</v>
       </c>
@@ -7902,7 +7309,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:5">
+    <row r="27" spans="1:7">
       <c r="A27">
         <v>25</v>
       </c>
@@ -7919,7 +7326,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:5">
+    <row r="28" spans="1:7">
       <c r="A28">
         <v>26</v>
       </c>
@@ -7936,7 +7343,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:5">
+    <row r="29" spans="1:7">
       <c r="A29">
         <v>27</v>
       </c>
@@ -7953,7 +7360,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:5">
+    <row r="30" spans="1:7">
       <c r="A30">
         <v>28</v>
       </c>
@@ -7970,7 +7377,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:5">
+    <row r="31" spans="1:7">
       <c r="A31">
         <v>29</v>
       </c>
@@ -7987,7 +7394,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:5">
+    <row r="32" spans="1:7">
       <c r="A32">
         <v>30</v>
       </c>
@@ -8040,24 +7447,22 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
-  <headerFooter/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:G11"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="4.85833333333333" customWidth="1"/>
-    <col min="2" max="2" width="22.7083333333333" customWidth="1"/>
-    <col min="3" max="3" width="28.5666666666667" customWidth="1"/>
-    <col min="4" max="4" width="15.5666666666667" customWidth="1"/>
-    <col min="5" max="5" width="16.1416666666667" customWidth="1"/>
+    <col min="1" max="1" width="4.85546875" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="3" max="3" width="28.5703125" customWidth="1"/>
+    <col min="4" max="4" width="15.5703125" customWidth="1"/>
+    <col min="5" max="5" width="16.140625" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="11.1416666666667" customWidth="1"/>
+    <col min="7" max="7" width="11.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -8083,7 +7488,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:7">
       <c r="A2">
         <v>0</v>
       </c>
@@ -8103,7 +7508,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" ht="12.95" customHeight="1" spans="1:6">
+    <row r="3" spans="1:7" ht="12.95" customHeight="1">
       <c r="A3">
         <v>1</v>
       </c>
@@ -8120,7 +7525,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="4" ht="12.95" customHeight="1" spans="1:6">
+    <row r="4" spans="1:7" ht="12.95" customHeight="1">
       <c r="A4">
         <v>2</v>
       </c>
@@ -8137,7 +7542,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:7">
       <c r="A5">
         <v>3</v>
       </c>
@@ -8157,7 +7562,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:7">
       <c r="A6">
         <v>4</v>
       </c>
@@ -8177,7 +7582,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:7">
       <c r="A7">
         <v>5</v>
       </c>
@@ -8197,7 +7602,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:7">
       <c r="A8">
         <v>6</v>
       </c>
@@ -8217,7 +7622,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:7">
       <c r="A9">
         <v>7</v>
       </c>
@@ -8237,7 +7642,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:7">
       <c r="A10">
         <v>8</v>
       </c>
@@ -8257,7 +7662,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:7">
       <c r="A11">
         <v>9</v>
       </c>
@@ -8279,7 +7684,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
-  <headerFooter/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added account selection menu, VAddSpecifiedCardEffect
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Configurations/Cards.xlsx
+++ b/Assets/StreamingAssets/Configurations/Cards.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29029"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity\VTuberSim\Assets\StreamingAssets\Configurations\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA0FBF0A-7FAD-4F89-97EF-B2A0B61F6812}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView windowWidth="24750" windowHeight="10480"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cards" sheetId="1" r:id="rId1"/>
@@ -24,8 +30,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -1058,167 +1062,17 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="20">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="34">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1237,188 +1091,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="11">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -1444,251 +1118,9 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
   <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -1703,71 +1135,27 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="49">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
-    <cellStyle name="货币" xfId="2" builtinId="4"/>
-    <cellStyle name="百分比" xfId="3" builtinId="5"/>
-    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
-    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
-    <cellStyle name="超链接" xfId="6" builtinId="8"/>
-    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
-    <cellStyle name="注释" xfId="8" builtinId="10"/>
-    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
-    <cellStyle name="标题" xfId="10" builtinId="15"/>
-    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
-    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
-    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
-    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
-    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
-    <cellStyle name="输入" xfId="16" builtinId="20"/>
-    <cellStyle name="输出" xfId="17" builtinId="21"/>
-    <cellStyle name="计算" xfId="18" builtinId="22"/>
-    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
-    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
-    <cellStyle name="汇总" xfId="21" builtinId="25"/>
-    <cellStyle name="好" xfId="22" builtinId="26"/>
-    <cellStyle name="差" xfId="23" builtinId="27"/>
-    <cellStyle name="适中" xfId="24" builtinId="28"/>
-    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
-    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
-    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
-    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
-    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
-    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
-      <color rgb="00FFFFFF"/>
-      <color rgb="00AB0580"/>
-      <color rgb="0000B050"/>
-      <color rgb="00FFB200"/>
-      <color rgb="004B58FF"/>
-      <color rgb="00FF2160"/>
+      <color rgb="FFFFFFFF"/>
+      <color rgb="FFAB0580"/>
+      <color rgb="FF00B050"/>
+      <color rgb="FFFFB200"/>
+      <color rgb="FF4B58FF"/>
+      <color rgb="FFFF2160"/>
     </mruColors>
   </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -2025,50 +1413,49 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AI61"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="3.425" customWidth="1"/>
-    <col min="2" max="2" width="12.7083333333333" customWidth="1"/>
+    <col min="1" max="1" width="3.42578125" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" customWidth="1"/>
     <col min="3" max="3" width="35" customWidth="1"/>
-    <col min="4" max="4" width="57.7083333333333" customWidth="1"/>
-    <col min="5" max="5" width="10.425" style="2" customWidth="1"/>
-    <col min="6" max="6" width="4.85833333333333" customWidth="1"/>
-    <col min="7" max="7" width="7.85833333333333" customWidth="1"/>
+    <col min="4" max="4" width="57.7109375" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" style="2" customWidth="1"/>
+    <col min="6" max="6" width="4.85546875" customWidth="1"/>
+    <col min="7" max="7" width="7.85546875" customWidth="1"/>
     <col min="8" max="8" width="5" customWidth="1"/>
-    <col min="9" max="9" width="5.56666666666667" style="3" customWidth="1"/>
-    <col min="10" max="10" width="10.5666666666667" customWidth="1"/>
-    <col min="11" max="11" width="9.70833333333333" style="3" customWidth="1"/>
-    <col min="12" max="12" width="7.14166666666667" customWidth="1"/>
+    <col min="9" max="9" width="5.5703125" style="3" customWidth="1"/>
+    <col min="10" max="10" width="10.5703125" customWidth="1"/>
+    <col min="11" max="11" width="9.7109375" style="3" customWidth="1"/>
+    <col min="12" max="12" width="7.140625" customWidth="1"/>
     <col min="13" max="13" width="14" style="3" customWidth="1"/>
-    <col min="14" max="14" width="10.2833333333333" customWidth="1"/>
-    <col min="15" max="15" width="13.7083333333333" customWidth="1"/>
-    <col min="16" max="16" width="13.7083333333333" customWidth="1"/>
-    <col min="17" max="17" width="9.70833333333333" style="3" customWidth="1"/>
-    <col min="18" max="18" width="9.70833333333333" customWidth="1"/>
-    <col min="19" max="19" width="12.1416666666667" customWidth="1"/>
-    <col min="20" max="20" width="17.7083333333333" style="3" customWidth="1"/>
+    <col min="14" max="14" width="10.28515625" customWidth="1"/>
+    <col min="15" max="16" width="13.7109375" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" style="3" customWidth="1"/>
+    <col min="18" max="18" width="9.7109375" customWidth="1"/>
+    <col min="19" max="19" width="12.140625" customWidth="1"/>
+    <col min="20" max="20" width="17.7109375" style="3" customWidth="1"/>
     <col min="21" max="21" width="11" customWidth="1"/>
-    <col min="22" max="22" width="12.2833333333333" customWidth="1"/>
-    <col min="23" max="23" width="17.1416666666667" style="3" customWidth="1"/>
-    <col min="26" max="26" width="17.7083333333333" style="3" customWidth="1"/>
-    <col min="27" max="27" width="10.7083333333333" customWidth="1"/>
+    <col min="22" max="22" width="12.28515625" customWidth="1"/>
+    <col min="23" max="23" width="17.140625" style="3" customWidth="1"/>
+    <col min="26" max="26" width="17.7109375" style="3" customWidth="1"/>
+    <col min="27" max="27" width="10.7109375" customWidth="1"/>
     <col min="28" max="28" width="11" customWidth="1"/>
-    <col min="29" max="29" width="17.7083333333333" style="3" customWidth="1"/>
-    <col min="30" max="30" width="12.425" customWidth="1"/>
-    <col min="31" max="31" width="12.425" style="3" customWidth="1"/>
-    <col min="32" max="32" width="12.2833333333333" customWidth="1"/>
+    <col min="29" max="29" width="17.7109375" style="3" customWidth="1"/>
+    <col min="30" max="30" width="12.42578125" customWidth="1"/>
+    <col min="31" max="31" width="12.42578125" style="3" customWidth="1"/>
+    <col min="32" max="32" width="12.28515625" customWidth="1"/>
     <col min="33" max="33" width="9" style="3"/>
-    <col min="34" max="34" width="4.28333333333333" customWidth="1"/>
+    <col min="34" max="34" width="4.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34">
+    <row r="1" spans="1:35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2172,7 +1559,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:34">
+    <row r="2" spans="1:35">
       <c r="A2">
         <v>0</v>
       </c>
@@ -2227,7 +1614,7 @@
       <c r="AG2"/>
       <c r="AH2" s="5"/>
     </row>
-    <row r="3" spans="1:34">
+    <row r="3" spans="1:35">
       <c r="A3">
         <v>1</v>
       </c>
@@ -2282,7 +1669,7 @@
       <c r="AG3"/>
       <c r="AH3" s="5"/>
     </row>
-    <row r="4" spans="1:34">
+    <row r="4" spans="1:35">
       <c r="A4">
         <v>2</v>
       </c>
@@ -2342,7 +1729,7 @@
       </c>
       <c r="AH4" s="5"/>
     </row>
-    <row r="5" spans="1:34">
+    <row r="5" spans="1:35">
       <c r="A5">
         <v>3</v>
       </c>
@@ -2405,7 +1792,7 @@
       <c r="AG5"/>
       <c r="AH5" s="5"/>
     </row>
-    <row r="6" spans="1:34">
+    <row r="6" spans="1:35">
       <c r="A6">
         <v>4</v>
       </c>
@@ -2471,7 +1858,7 @@
       </c>
       <c r="AH6" s="5"/>
     </row>
-    <row r="7" spans="1:34">
+    <row r="7" spans="1:35">
       <c r="A7">
         <v>5</v>
       </c>
@@ -2537,7 +1924,7 @@
       <c r="AG7"/>
       <c r="AH7" s="5"/>
     </row>
-    <row r="8" spans="1:34">
+    <row r="8" spans="1:35">
       <c r="A8">
         <v>6</v>
       </c>
@@ -2610,7 +1997,7 @@
       <c r="AG8"/>
       <c r="AH8" s="5"/>
     </row>
-    <row r="9" spans="1:34">
+    <row r="9" spans="1:35">
       <c r="A9">
         <v>8</v>
       </c>
@@ -2673,7 +2060,7 @@
       <c r="AG9"/>
       <c r="AH9" s="5"/>
     </row>
-    <row r="10" spans="1:34">
+    <row r="10" spans="1:35">
       <c r="A10">
         <v>9</v>
       </c>
@@ -2736,7 +2123,7 @@
       <c r="AG10"/>
       <c r="AH10" s="5"/>
     </row>
-    <row r="11" spans="1:34">
+    <row r="11" spans="1:35">
       <c r="A11">
         <v>10</v>
       </c>
@@ -2862,7 +2249,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="13" spans="1:34">
+    <row r="13" spans="1:35">
       <c r="A13">
         <v>12</v>
       </c>
@@ -2925,7 +2312,7 @@
       <c r="AG13"/>
       <c r="AH13" s="5"/>
     </row>
-    <row r="14" spans="1:34">
+    <row r="14" spans="1:35">
       <c r="A14">
         <v>13</v>
       </c>
@@ -2980,7 +2367,7 @@
       <c r="AG14"/>
       <c r="AH14" s="5"/>
     </row>
-    <row r="15" spans="1:34">
+    <row r="15" spans="1:35">
       <c r="A15">
         <v>14</v>
       </c>
@@ -3035,7 +2422,7 @@
       <c r="AG15"/>
       <c r="AH15" s="5"/>
     </row>
-    <row r="16" spans="1:34">
+    <row r="16" spans="1:35">
       <c r="A16">
         <v>15</v>
       </c>
@@ -3090,7 +2477,7 @@
         <v>0.8</v>
       </c>
       <c r="W16" s="3">
-        <v>1.1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="Z16"/>
       <c r="AC16"/>
@@ -4066,7 +3453,7 @@
       <c r="AG31"/>
       <c r="AH31" s="6"/>
     </row>
-    <row r="32" spans="1:33">
+    <row r="32" spans="1:34">
       <c r="A32">
         <v>33</v>
       </c>
@@ -4115,7 +3502,7 @@
       <c r="AE32"/>
       <c r="AG32"/>
     </row>
-    <row r="33" spans="1:31">
+    <row r="33" spans="1:33">
       <c r="A33">
         <v>34</v>
       </c>
@@ -4171,7 +3558,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:20">
+    <row r="34" spans="1:33">
       <c r="A34">
         <v>35</v>
       </c>
@@ -4224,7 +3611,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="35" spans="1:20">
+    <row r="35" spans="1:33">
       <c r="A35">
         <v>36</v>
       </c>
@@ -4274,7 +3661,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="36" spans="1:23">
+    <row r="36" spans="1:33">
       <c r="A36">
         <v>37</v>
       </c>
@@ -4775,7 +4162,7 @@
       <c r="AE43"/>
       <c r="AG43"/>
     </row>
-    <row r="44" spans="1:23">
+    <row r="44" spans="1:33">
       <c r="A44">
         <v>45</v>
       </c>
@@ -5093,7 +4480,7 @@
       <c r="AE48"/>
       <c r="AG48"/>
     </row>
-    <row r="49" spans="1:23">
+    <row r="49" spans="1:33">
       <c r="A49">
         <v>50</v>
       </c>
@@ -5204,7 +4591,7 @@
         <v>18</v>
       </c>
       <c r="V50">
-        <v>1.1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="W50" s="3">
         <v>1.7</v>
@@ -5338,7 +4725,7 @@
       <c r="AE52"/>
       <c r="AG52"/>
     </row>
-    <row r="53" spans="1:23">
+    <row r="53" spans="1:33">
       <c r="A53">
         <v>54</v>
       </c>
@@ -5400,7 +4787,7 @@
         <v>-0.5</v>
       </c>
     </row>
-    <row r="54" spans="1:26">
+    <row r="54" spans="1:33">
       <c r="A54">
         <v>55</v>
       </c>
@@ -5471,7 +4858,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="55" spans="1:32">
+    <row r="55" spans="1:33">
       <c r="A55">
         <v>56</v>
       </c>
@@ -5531,7 +4918,7 @@
       </c>
       <c r="AF55" s="3"/>
     </row>
-    <row r="56" spans="1:32">
+    <row r="56" spans="1:33">
       <c r="A56">
         <v>57</v>
       </c>
@@ -5603,7 +4990,7 @@
       </c>
       <c r="AF56" s="3"/>
     </row>
-    <row r="57" spans="1:23">
+    <row r="57" spans="1:33">
       <c r="A57">
         <v>58</v>
       </c>
@@ -5665,7 +5052,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="58" spans="1:15">
+    <row r="58" spans="1:33">
       <c r="A58">
         <v>59</v>
       </c>
@@ -5706,7 +5093,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:20">
+    <row r="59" spans="1:33">
       <c r="A59">
         <v>60</v>
       </c>
@@ -5756,7 +5143,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="60" spans="1:15">
+    <row r="60" spans="1:33">
       <c r="A60">
         <v>61</v>
       </c>
@@ -5797,7 +5184,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:15">
+    <row r="61" spans="1:33">
       <c r="A61">
         <v>62</v>
       </c>
@@ -5843,25 +5230,23 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
-  <headerFooter/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:I67"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="3.425" customWidth="1"/>
-    <col min="2" max="2" width="27.425" customWidth="1"/>
+    <col min="1" max="1" width="3.42578125" customWidth="1"/>
+    <col min="2" max="2" width="27.42578125" customWidth="1"/>
     <col min="3" max="3" width="35" customWidth="1"/>
     <col min="4" max="4" width="33" customWidth="1"/>
-    <col min="5" max="5" width="19.2833333333333" customWidth="1"/>
-    <col min="6" max="6" width="18.8583333333333" customWidth="1"/>
-    <col min="7" max="8" width="10.2833333333333" customWidth="1"/>
-    <col min="9" max="9" width="15.1416666666667" customWidth="1"/>
+    <col min="5" max="5" width="19.28515625" customWidth="1"/>
+    <col min="6" max="6" width="18.85546875" customWidth="1"/>
+    <col min="7" max="8" width="10.28515625" customWidth="1"/>
+    <col min="9" max="9" width="15.140625" customWidth="1"/>
     <col min="10" max="10" width="22" customWidth="1"/>
   </cols>
   <sheetData>
@@ -7183,7 +6568,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="63" customFormat="1" spans="1:9">
+    <row r="63" spans="1:9">
       <c r="A63">
         <v>61</v>
       </c>
@@ -7243,7 +6628,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="66" customFormat="1" spans="1:9">
+    <row r="66" spans="1:9">
       <c r="A66">
         <v>64</v>
       </c>
@@ -7288,26 +6673,24 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
-  <headerFooter/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:O34"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="9.425" customWidth="1"/>
-    <col min="2" max="2" width="27.425" customWidth="1"/>
-    <col min="3" max="3" width="14.425" customWidth="1"/>
-    <col min="4" max="5" width="16.1416666666667" customWidth="1"/>
-    <col min="6" max="6" width="12.425" customWidth="1"/>
-    <col min="7" max="7" width="14.425" customWidth="1"/>
+    <col min="1" max="1" width="9.42578125" customWidth="1"/>
+    <col min="2" max="2" width="27.42578125" customWidth="1"/>
+    <col min="3" max="3" width="14.42578125" customWidth="1"/>
+    <col min="4" max="5" width="16.140625" customWidth="1"/>
+    <col min="6" max="6" width="12.42578125" customWidth="1"/>
+    <col min="7" max="7" width="14.42578125" customWidth="1"/>
     <col min="8" max="8" width="10" customWidth="1"/>
     <col min="9" max="9" width="13" customWidth="1"/>
-    <col min="10" max="10" width="10.1416666666667" customWidth="1"/>
+    <col min="10" max="10" width="10.140625" customWidth="1"/>
     <col min="11" max="11" width="13" customWidth="1"/>
   </cols>
   <sheetData>
@@ -7358,7 +6741,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:15">
       <c r="A2">
         <v>0</v>
       </c>
@@ -7387,7 +6770,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:15">
       <c r="A3">
         <v>1</v>
       </c>
@@ -7410,7 +6793,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:15">
       <c r="A4">
         <v>2</v>
       </c>
@@ -7427,7 +6810,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
+    <row r="5" spans="1:15">
       <c r="A5">
         <v>3</v>
       </c>
@@ -7462,7 +6845,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:15">
       <c r="A6">
         <v>4</v>
       </c>
@@ -7485,7 +6868,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:15">
       <c r="A7">
         <v>5</v>
       </c>
@@ -7508,7 +6891,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="8" spans="1:7">
+    <row r="8" spans="1:15">
       <c r="A8">
         <v>6</v>
       </c>
@@ -7531,7 +6914,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:15">
       <c r="A9">
         <v>7</v>
       </c>
@@ -7554,7 +6937,7 @@
         <v>-0.5</v>
       </c>
     </row>
-    <row r="10" spans="1:7">
+    <row r="10" spans="1:15">
       <c r="A10">
         <v>8</v>
       </c>
@@ -7577,7 +6960,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:9">
+    <row r="11" spans="1:15">
       <c r="A11">
         <v>9</v>
       </c>
@@ -7606,7 +6989,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="12" spans="1:9">
+    <row r="12" spans="1:15">
       <c r="A12">
         <v>10</v>
       </c>
@@ -7635,7 +7018,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="13" spans="1:7">
+    <row r="13" spans="1:15">
       <c r="A13">
         <v>11</v>
       </c>
@@ -7658,7 +7041,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:7">
+    <row r="14" spans="1:15">
       <c r="A14">
         <v>12</v>
       </c>
@@ -7681,7 +7064,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:7">
+    <row r="15" spans="1:15">
       <c r="A15">
         <v>13</v>
       </c>
@@ -7704,7 +7087,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="1:7">
+    <row r="16" spans="1:15">
       <c r="A16">
         <v>14</v>
       </c>
@@ -7773,7 +7156,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:5">
+    <row r="19" spans="1:7">
       <c r="A19">
         <v>17</v>
       </c>
@@ -7790,7 +7173,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:5">
+    <row r="20" spans="1:7">
       <c r="A20">
         <v>18</v>
       </c>
@@ -7807,7 +7190,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:5">
+    <row r="21" spans="1:7">
       <c r="A21">
         <v>19</v>
       </c>
@@ -7893,7 +7276,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:5">
+    <row r="25" spans="1:7">
       <c r="A25">
         <v>23</v>
       </c>
@@ -7910,7 +7293,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:5">
+    <row r="26" spans="1:7">
       <c r="A26">
         <v>24</v>
       </c>
@@ -7927,7 +7310,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:5">
+    <row r="27" spans="1:7">
       <c r="A27">
         <v>25</v>
       </c>
@@ -7944,7 +7327,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:5">
+    <row r="28" spans="1:7">
       <c r="A28">
         <v>26</v>
       </c>
@@ -7961,7 +7344,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:5">
+    <row r="29" spans="1:7">
       <c r="A29">
         <v>27</v>
       </c>
@@ -7978,7 +7361,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:5">
+    <row r="30" spans="1:7">
       <c r="A30">
         <v>28</v>
       </c>
@@ -7995,7 +7378,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:5">
+    <row r="31" spans="1:7">
       <c r="A31">
         <v>29</v>
       </c>
@@ -8012,7 +7395,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:5">
+    <row r="32" spans="1:7">
       <c r="A32">
         <v>30</v>
       </c>
@@ -8065,24 +7448,22 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
-  <headerFooter/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:G11"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="4.85833333333333" customWidth="1"/>
-    <col min="2" max="2" width="22.7083333333333" customWidth="1"/>
-    <col min="3" max="3" width="28.5666666666667" customWidth="1"/>
-    <col min="4" max="4" width="15.5666666666667" customWidth="1"/>
-    <col min="5" max="5" width="16.1416666666667" customWidth="1"/>
+    <col min="1" max="1" width="4.85546875" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="3" max="3" width="28.5703125" customWidth="1"/>
+    <col min="4" max="4" width="15.5703125" customWidth="1"/>
+    <col min="5" max="5" width="16.140625" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="11.1416666666667" customWidth="1"/>
+    <col min="7" max="7" width="11.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -8108,7 +7489,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:7">
       <c r="A2">
         <v>0</v>
       </c>
@@ -8128,7 +7509,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" ht="12.95" customHeight="1" spans="1:6">
+    <row r="3" spans="1:7" ht="12.95" customHeight="1">
       <c r="A3">
         <v>1</v>
       </c>
@@ -8145,7 +7526,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="4" ht="12.95" customHeight="1" spans="1:6">
+    <row r="4" spans="1:7" ht="12.95" customHeight="1">
       <c r="A4">
         <v>2</v>
       </c>
@@ -8162,7 +7543,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:7">
       <c r="A5">
         <v>3</v>
       </c>
@@ -8182,7 +7563,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:7">
       <c r="A6">
         <v>4</v>
       </c>
@@ -8202,7 +7583,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:7">
       <c r="A7">
         <v>5</v>
       </c>
@@ -8222,7 +7603,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:7">
       <c r="A8">
         <v>6</v>
       </c>
@@ -8242,7 +7623,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:7">
       <c r="A9">
         <v>7</v>
       </c>
@@ -8262,7 +7643,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:7">
       <c r="A10">
         <v>8</v>
       </c>
@@ -8282,7 +7663,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:7">
       <c r="A11">
         <v>9</v>
       </c>
@@ -8304,7 +7685,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
-  <headerFooter/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fixing bug in coop events generation
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Configurations/Cards.xlsx
+++ b/Assets/StreamingAssets/Configurations/Cards.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29029"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity\VTuberSim\Assets\StreamingAssets\Configurations\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D923D163-F5B5-4B72-925B-C70A1A44A05F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView windowWidth="24750" windowHeight="10480" activeTab="3"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cards" sheetId="1" r:id="rId1"/>
@@ -24,8 +30,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -1340,167 +1344,17 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="20">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="35">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1525,188 +1379,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="11">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -1732,251 +1406,9 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
   <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -1992,71 +1424,27 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="49">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
-    <cellStyle name="货币" xfId="2" builtinId="4"/>
-    <cellStyle name="百分比" xfId="3" builtinId="5"/>
-    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
-    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
-    <cellStyle name="超链接" xfId="6" builtinId="8"/>
-    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
-    <cellStyle name="注释" xfId="8" builtinId="10"/>
-    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
-    <cellStyle name="标题" xfId="10" builtinId="15"/>
-    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
-    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
-    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
-    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
-    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
-    <cellStyle name="输入" xfId="16" builtinId="20"/>
-    <cellStyle name="输出" xfId="17" builtinId="21"/>
-    <cellStyle name="计算" xfId="18" builtinId="22"/>
-    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
-    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
-    <cellStyle name="汇总" xfId="21" builtinId="25"/>
-    <cellStyle name="好" xfId="22" builtinId="26"/>
-    <cellStyle name="差" xfId="23" builtinId="27"/>
-    <cellStyle name="适中" xfId="24" builtinId="28"/>
-    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
-    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
-    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
-    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
-    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
-    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
-      <color rgb="00FFFFFF"/>
-      <color rgb="00AB0580"/>
-      <color rgb="0000B050"/>
-      <color rgb="00FFB200"/>
-      <color rgb="004B58FF"/>
-      <color rgb="00FF2160"/>
+      <color rgb="FFFFFFFF"/>
+      <color rgb="FFAB0580"/>
+      <color rgb="FF00B050"/>
+      <color rgb="FFFFB200"/>
+      <color rgb="FF4B58FF"/>
+      <color rgb="FFFF2160"/>
     </mruColors>
   </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -2314,49 +1702,49 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AJ72"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="3.45" customWidth="1"/>
-    <col min="2" max="2" width="12.725" customWidth="1"/>
+    <col min="1" max="1" width="3.42578125" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" customWidth="1"/>
     <col min="3" max="3" width="35" customWidth="1"/>
-    <col min="4" max="4" width="57.725" customWidth="1"/>
-    <col min="5" max="5" width="10.45" style="3" customWidth="1"/>
-    <col min="6" max="6" width="4.81666666666667" customWidth="1"/>
-    <col min="7" max="7" width="7.81666666666667" customWidth="1"/>
+    <col min="4" max="4" width="57.7109375" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" style="3" customWidth="1"/>
+    <col min="6" max="6" width="4.85546875" customWidth="1"/>
+    <col min="7" max="7" width="7.85546875" customWidth="1"/>
     <col min="8" max="8" width="5" customWidth="1"/>
-    <col min="9" max="9" width="5.54166666666667" style="2" customWidth="1"/>
-    <col min="10" max="11" width="10.5416666666667" customWidth="1"/>
-    <col min="12" max="12" width="9.725" style="2" customWidth="1"/>
-    <col min="13" max="13" width="7.18333333333333" customWidth="1"/>
+    <col min="9" max="9" width="5.5703125" style="2" customWidth="1"/>
+    <col min="10" max="11" width="10.5703125" customWidth="1"/>
+    <col min="12" max="12" width="9.7109375" style="2" customWidth="1"/>
+    <col min="13" max="13" width="7.140625" customWidth="1"/>
     <col min="14" max="14" width="14" style="2" customWidth="1"/>
-    <col min="15" max="15" width="10.2666666666667" customWidth="1"/>
-    <col min="16" max="17" width="13.725" customWidth="1"/>
-    <col min="18" max="18" width="9.725" style="2" customWidth="1"/>
-    <col min="19" max="19" width="9.725" customWidth="1"/>
-    <col min="20" max="20" width="12.1833333333333" customWidth="1"/>
-    <col min="21" max="21" width="17.725" style="2" customWidth="1"/>
+    <col min="15" max="15" width="10.28515625" customWidth="1"/>
+    <col min="16" max="17" width="13.7109375" customWidth="1"/>
+    <col min="18" max="18" width="9.7109375" style="2" customWidth="1"/>
+    <col min="19" max="19" width="9.7109375" customWidth="1"/>
+    <col min="20" max="20" width="12.140625" customWidth="1"/>
+    <col min="21" max="21" width="17.7109375" style="2" customWidth="1"/>
     <col min="22" max="22" width="11" customWidth="1"/>
-    <col min="23" max="23" width="12.2666666666667" customWidth="1"/>
-    <col min="24" max="24" width="17.1833333333333" style="2" customWidth="1"/>
-    <col min="27" max="27" width="17.725" style="2" customWidth="1"/>
-    <col min="28" max="28" width="10.725" customWidth="1"/>
+    <col min="23" max="23" width="12.28515625" customWidth="1"/>
+    <col min="24" max="24" width="17.140625" style="2" customWidth="1"/>
+    <col min="27" max="27" width="17.7109375" style="2" customWidth="1"/>
+    <col min="28" max="28" width="10.7109375" customWidth="1"/>
     <col min="29" max="29" width="11" customWidth="1"/>
-    <col min="30" max="30" width="17.725" style="2" customWidth="1"/>
-    <col min="31" max="31" width="12.45" customWidth="1"/>
-    <col min="32" max="32" width="12.45" style="2" customWidth="1"/>
-    <col min="33" max="33" width="12.2666666666667" customWidth="1"/>
+    <col min="30" max="30" width="17.7109375" style="2" customWidth="1"/>
+    <col min="31" max="31" width="12.42578125" customWidth="1"/>
+    <col min="32" max="32" width="12.42578125" style="2" customWidth="1"/>
+    <col min="33" max="33" width="12.28515625" customWidth="1"/>
     <col min="34" max="34" width="9" style="2"/>
-    <col min="35" max="35" width="4.26666666666667" customWidth="1"/>
+    <col min="35" max="35" width="4.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35">
+    <row r="1" spans="1:36">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2463,7 +1851,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:35">
+    <row r="2" spans="1:36">
       <c r="A2">
         <v>0</v>
       </c>
@@ -2518,7 +1906,7 @@
       <c r="AH2"/>
       <c r="AI2" s="6"/>
     </row>
-    <row r="3" spans="1:35">
+    <row r="3" spans="1:36">
       <c r="A3">
         <v>1</v>
       </c>
@@ -2573,7 +1961,7 @@
       <c r="AH3"/>
       <c r="AI3" s="6"/>
     </row>
-    <row r="4" spans="1:35">
+    <row r="4" spans="1:36">
       <c r="A4">
         <v>2</v>
       </c>
@@ -2633,7 +2021,7 @@
       </c>
       <c r="AI4" s="6"/>
     </row>
-    <row r="5" spans="1:35">
+    <row r="5" spans="1:36">
       <c r="A5">
         <v>3</v>
       </c>
@@ -2696,7 +2084,7 @@
       <c r="AH5"/>
       <c r="AI5" s="6"/>
     </row>
-    <row r="6" spans="1:35">
+    <row r="6" spans="1:36">
       <c r="A6">
         <v>4</v>
       </c>
@@ -2762,7 +2150,7 @@
       </c>
       <c r="AI6" s="6"/>
     </row>
-    <row r="7" spans="1:35">
+    <row r="7" spans="1:36">
       <c r="A7">
         <v>5</v>
       </c>
@@ -2828,7 +2216,7 @@
       <c r="AH7"/>
       <c r="AI7" s="6"/>
     </row>
-    <row r="8" spans="1:35">
+    <row r="8" spans="1:36">
       <c r="A8">
         <v>6</v>
       </c>
@@ -2901,7 +2289,7 @@
       <c r="AH8"/>
       <c r="AI8" s="6"/>
     </row>
-    <row r="9" spans="1:35">
+    <row r="9" spans="1:36">
       <c r="A9">
         <v>8</v>
       </c>
@@ -2964,7 +2352,7 @@
       <c r="AH9"/>
       <c r="AI9" s="6"/>
     </row>
-    <row r="10" spans="1:35">
+    <row r="10" spans="1:36">
       <c r="A10">
         <v>9</v>
       </c>
@@ -3027,7 +2415,7 @@
       <c r="AH10"/>
       <c r="AI10" s="6"/>
     </row>
-    <row r="11" spans="1:35">
+    <row r="11" spans="1:36">
       <c r="A11">
         <v>10</v>
       </c>
@@ -3153,7 +2541,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="13" spans="1:35">
+    <row r="13" spans="1:36">
       <c r="A13">
         <v>12</v>
       </c>
@@ -3216,7 +2604,7 @@
       <c r="AH13"/>
       <c r="AI13" s="6"/>
     </row>
-    <row r="14" spans="1:35">
+    <row r="14" spans="1:36">
       <c r="A14">
         <v>13</v>
       </c>
@@ -3271,7 +2659,7 @@
       <c r="AH14"/>
       <c r="AI14" s="6"/>
     </row>
-    <row r="15" spans="1:35">
+    <row r="15" spans="1:36">
       <c r="A15">
         <v>14</v>
       </c>
@@ -3326,7 +2714,7 @@
       <c r="AH15"/>
       <c r="AI15" s="6"/>
     </row>
-    <row r="16" spans="1:35">
+    <row r="16" spans="1:36">
       <c r="A16">
         <v>15</v>
       </c>
@@ -3381,7 +2769,7 @@
         <v>0.8</v>
       </c>
       <c r="X16" s="2">
-        <v>1.1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="AA16"/>
       <c r="AD16"/>
@@ -4357,7 +3745,7 @@
       <c r="AH31"/>
       <c r="AI31" s="7"/>
     </row>
-    <row r="32" spans="1:34">
+    <row r="32" spans="1:35">
       <c r="A32">
         <v>33</v>
       </c>
@@ -4406,7 +3794,7 @@
       <c r="AF32"/>
       <c r="AH32"/>
     </row>
-    <row r="33" spans="1:32">
+    <row r="33" spans="1:34">
       <c r="A33">
         <v>34</v>
       </c>
@@ -4462,7 +3850,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:21">
+    <row r="34" spans="1:34">
       <c r="A34">
         <v>35</v>
       </c>
@@ -4515,7 +3903,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="35" spans="1:24">
+    <row r="35" spans="1:34">
       <c r="A35">
         <v>36</v>
       </c>
@@ -4574,7 +3962,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:24">
+    <row r="36" spans="1:34">
       <c r="A36">
         <v>37</v>
       </c>
@@ -5075,7 +4463,7 @@
       <c r="AF43"/>
       <c r="AH43"/>
     </row>
-    <row r="44" spans="1:24">
+    <row r="44" spans="1:34">
       <c r="A44">
         <v>45</v>
       </c>
@@ -5393,7 +4781,7 @@
       <c r="AF48"/>
       <c r="AH48"/>
     </row>
-    <row r="49" spans="1:24">
+    <row r="49" spans="1:34">
       <c r="A49">
         <v>50</v>
       </c>
@@ -5504,7 +4892,7 @@
         <v>18</v>
       </c>
       <c r="W50">
-        <v>1.1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="X50" s="2">
         <v>1.7</v>
@@ -5638,7 +5026,7 @@
       <c r="AF52"/>
       <c r="AH52"/>
     </row>
-    <row r="53" spans="1:24">
+    <row r="53" spans="1:34">
       <c r="A53">
         <v>54</v>
       </c>
@@ -5700,7 +5088,7 @@
         <v>-0.5</v>
       </c>
     </row>
-    <row r="54" spans="1:27">
+    <row r="54" spans="1:34">
       <c r="A54">
         <v>55</v>
       </c>
@@ -5771,7 +5159,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="55" spans="1:33">
+    <row r="55" spans="1:34">
       <c r="A55">
         <v>56</v>
       </c>
@@ -5831,7 +5219,7 @@
       </c>
       <c r="AG55" s="2"/>
     </row>
-    <row r="56" spans="1:33">
+    <row r="56" spans="1:34">
       <c r="A56">
         <v>57</v>
       </c>
@@ -5903,7 +5291,7 @@
       </c>
       <c r="AG56" s="2"/>
     </row>
-    <row r="57" spans="1:27">
+    <row r="57" spans="1:34">
       <c r="A57">
         <v>58</v>
       </c>
@@ -5974,7 +5362,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="58" spans="1:21">
+    <row r="58" spans="1:34">
       <c r="A58">
         <v>59</v>
       </c>
@@ -6024,7 +5412,7 @@
         <v>1.7</v>
       </c>
     </row>
-    <row r="59" spans="1:24">
+    <row r="59" spans="1:34">
       <c r="A59">
         <v>60</v>
       </c>
@@ -6083,7 +5471,7 @@
         <v>1.4</v>
       </c>
     </row>
-    <row r="60" spans="1:24">
+    <row r="60" spans="1:34">
       <c r="A60">
         <v>61</v>
       </c>
@@ -6142,7 +5530,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="61" spans="1:24">
+    <row r="61" spans="1:34">
       <c r="A61">
         <v>62</v>
       </c>
@@ -6204,7 +5592,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:24">
+    <row r="62" spans="1:34">
       <c r="A62">
         <v>63</v>
       </c>
@@ -6266,7 +5654,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="63" spans="1:30">
+    <row r="63" spans="1:34">
       <c r="A63">
         <v>64</v>
       </c>
@@ -6346,7 +5734,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="64" spans="1:24">
+    <row r="64" spans="1:34">
       <c r="A64">
         <v>65</v>
       </c>
@@ -6402,7 +5790,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="65" spans="1:24">
+    <row r="65" spans="1:30">
       <c r="A65">
         <v>66</v>
       </c>
@@ -6532,7 +5920,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="67" spans="1:27">
+    <row r="67" spans="1:30">
       <c r="A67">
         <v>68</v>
       </c>
@@ -6600,7 +5988,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:24">
+    <row r="68" spans="1:30">
       <c r="A68">
         <v>69</v>
       </c>
@@ -6656,7 +6044,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:21">
+    <row r="69" spans="1:30">
       <c r="A69">
         <v>70</v>
       </c>
@@ -6706,7 +6094,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="70" spans="1:21">
+    <row r="70" spans="1:30">
       <c r="A70">
         <v>71</v>
       </c>
@@ -6753,7 +6141,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="71" spans="1:24">
+    <row r="71" spans="1:30">
       <c r="A71">
         <v>72</v>
       </c>
@@ -6809,7 +6197,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:24">
+    <row r="72" spans="1:30">
       <c r="A72">
         <v>73</v>
       </c>
@@ -6867,25 +6255,23 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
-  <headerFooter/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:I77"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="3.45" customWidth="1"/>
-    <col min="2" max="2" width="27.45" customWidth="1"/>
+    <col min="1" max="1" width="3.42578125" customWidth="1"/>
+    <col min="2" max="2" width="27.42578125" customWidth="1"/>
     <col min="3" max="3" width="35" customWidth="1"/>
     <col min="4" max="4" width="33" customWidth="1"/>
-    <col min="5" max="5" width="19.2666666666667" customWidth="1"/>
-    <col min="6" max="6" width="18.8166666666667" customWidth="1"/>
-    <col min="7" max="8" width="10.2666666666667" customWidth="1"/>
-    <col min="9" max="9" width="15.1833333333333" customWidth="1"/>
+    <col min="5" max="5" width="19.28515625" customWidth="1"/>
+    <col min="6" max="6" width="18.85546875" customWidth="1"/>
+    <col min="7" max="8" width="10.28515625" customWidth="1"/>
+    <col min="9" max="9" width="15.140625" customWidth="1"/>
     <col min="10" max="10" width="22" customWidth="1"/>
   </cols>
   <sheetData>
@@ -8497,26 +7883,24 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
-  <headerFooter/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:P37"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="9.45" customWidth="1"/>
-    <col min="2" max="2" width="27.45" customWidth="1"/>
-    <col min="3" max="3" width="14.45" customWidth="1"/>
-    <col min="4" max="6" width="16.1833333333333" customWidth="1"/>
-    <col min="7" max="7" width="12.45" customWidth="1"/>
-    <col min="8" max="8" width="14.45" customWidth="1"/>
+    <col min="1" max="1" width="9.42578125" customWidth="1"/>
+    <col min="2" max="2" width="27.42578125" customWidth="1"/>
+    <col min="3" max="3" width="14.42578125" customWidth="1"/>
+    <col min="4" max="6" width="16.140625" customWidth="1"/>
+    <col min="7" max="7" width="12.42578125" customWidth="1"/>
+    <col min="8" max="8" width="14.42578125" customWidth="1"/>
     <col min="9" max="9" width="10" customWidth="1"/>
     <col min="10" max="10" width="13" customWidth="1"/>
-    <col min="11" max="11" width="10.1833333333333" customWidth="1"/>
+    <col min="11" max="11" width="10.140625" customWidth="1"/>
     <col min="12" max="12" width="13" customWidth="1"/>
   </cols>
   <sheetData>
@@ -8570,7 +7954,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:16">
       <c r="A2">
         <v>0</v>
       </c>
@@ -8599,7 +7983,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="3" spans="1:8">
+    <row r="3" spans="1:16">
       <c r="A3">
         <v>1</v>
       </c>
@@ -8622,7 +8006,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:16">
       <c r="A4">
         <v>2</v>
       </c>
@@ -8639,7 +8023,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:12">
+    <row r="5" spans="1:16">
       <c r="A5">
         <v>3</v>
       </c>
@@ -8674,7 +8058,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="6" spans="1:8">
+    <row r="6" spans="1:16">
       <c r="A6">
         <v>4</v>
       </c>
@@ -8697,7 +8081,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:8">
+    <row r="7" spans="1:16">
       <c r="A7">
         <v>5</v>
       </c>
@@ -8720,7 +8104,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="8" spans="1:8">
+    <row r="8" spans="1:16">
       <c r="A8">
         <v>6</v>
       </c>
@@ -8743,7 +8127,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:8">
+    <row r="9" spans="1:16">
       <c r="A9">
         <v>7</v>
       </c>
@@ -8766,7 +8150,7 @@
         <v>-0.5</v>
       </c>
     </row>
-    <row r="10" spans="1:8">
+    <row r="10" spans="1:16">
       <c r="A10">
         <v>8</v>
       </c>
@@ -8789,7 +8173,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:16">
       <c r="A11">
         <v>9</v>
       </c>
@@ -8818,7 +8202,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="12" spans="1:10">
+    <row r="12" spans="1:16">
       <c r="A12">
         <v>10</v>
       </c>
@@ -8847,7 +8231,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="13" spans="1:8">
+    <row r="13" spans="1:16">
       <c r="A13">
         <v>11</v>
       </c>
@@ -8870,7 +8254,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:8">
+    <row r="14" spans="1:16">
       <c r="A14">
         <v>12</v>
       </c>
@@ -8893,7 +8277,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:8">
+    <row r="15" spans="1:16">
       <c r="A15">
         <v>13</v>
       </c>
@@ -8916,7 +8300,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="1:8">
+    <row r="16" spans="1:16">
       <c r="A16">
         <v>14</v>
       </c>
@@ -8985,7 +8369,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:5">
+    <row r="19" spans="1:8">
       <c r="A19">
         <v>17</v>
       </c>
@@ -9002,7 +8386,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:5">
+    <row r="20" spans="1:8">
       <c r="A20">
         <v>18</v>
       </c>
@@ -9019,7 +8403,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:5">
+    <row r="21" spans="1:8">
       <c r="A21">
         <v>19</v>
       </c>
@@ -9289,7 +8673,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="33" spans="1:8">
+    <row r="33" spans="1:12">
       <c r="A33">
         <v>31</v>
       </c>
@@ -9312,7 +8696,7 @@
         <v>0.45</v>
       </c>
     </row>
-    <row r="34" spans="1:8">
+    <row r="34" spans="1:12">
       <c r="A34">
         <v>32</v>
       </c>
@@ -9370,7 +8754,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:8">
+    <row r="36" spans="1:12">
       <c r="A36">
         <v>34</v>
       </c>
@@ -9393,7 +8777,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:8">
+    <row r="37" spans="1:12">
       <c r="A37">
         <v>35</v>
       </c>
@@ -9418,24 +8802,22 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
-  <headerFooter/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:G14"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="4.81666666666667" customWidth="1"/>
-    <col min="2" max="2" width="22.725" customWidth="1"/>
-    <col min="3" max="3" width="28.5416666666667" customWidth="1"/>
-    <col min="4" max="4" width="15.5416666666667" customWidth="1"/>
-    <col min="5" max="5" width="16.1833333333333" customWidth="1"/>
+    <col min="1" max="1" width="4.85546875" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="3" max="3" width="28.5703125" customWidth="1"/>
+    <col min="4" max="4" width="15.5703125" customWidth="1"/>
+    <col min="5" max="5" width="16.140625" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="11.1833333333333" customWidth="1"/>
+    <col min="7" max="7" width="11.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -9461,7 +8843,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:7">
       <c r="A2">
         <v>0</v>
       </c>
@@ -9481,7 +8863,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" ht="13" customHeight="1" spans="1:6">
+    <row r="3" spans="1:7" ht="12.95" customHeight="1">
       <c r="A3">
         <v>1</v>
       </c>
@@ -9498,7 +8880,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="4" ht="13" customHeight="1" spans="1:6">
+    <row r="4" spans="1:7" ht="12.95" customHeight="1">
       <c r="A4">
         <v>2</v>
       </c>
@@ -9515,7 +8897,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:7">
       <c r="A5">
         <v>3</v>
       </c>
@@ -9535,7 +8917,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:7">
       <c r="A6">
         <v>4</v>
       </c>
@@ -9555,7 +8937,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:7">
       <c r="A7">
         <v>5</v>
       </c>
@@ -9575,7 +8957,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:7">
       <c r="A8">
         <v>6</v>
       </c>
@@ -9595,7 +8977,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:7">
       <c r="A9">
         <v>7</v>
       </c>
@@ -9615,7 +8997,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:7">
       <c r="A10">
         <v>8</v>
       </c>
@@ -9635,7 +9017,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:7">
       <c r="A11">
         <v>9</v>
       </c>
@@ -9655,7 +9037,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:7">
       <c r="A12">
         <v>10</v>
       </c>
@@ -9672,7 +9054,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:7">
       <c r="A13">
         <v>11</v>
       </c>
@@ -9689,7 +9071,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:7">
       <c r="A14">
         <v>12</v>
       </c>
@@ -9708,7 +9090,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
-  <headerFooter/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
changed the rare revenue cards into repeatable
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Configurations/Cards.xlsx
+++ b/Assets/StreamingAssets/Configurations/Cards.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity\VTuberSim\Assets\StreamingAssets\Configurations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{962F0A1B-5012-4E04-A132-3C7B156CFDC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6C5BF06-5774-42A7-939B-E66CC7D992F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cards" sheetId="1" r:id="rId1"/>
@@ -1799,39 +1799,39 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AJ72"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="3.42578125" customWidth="1"/>
-    <col min="2" max="2" width="12.7109375" customWidth="1"/>
+    <col min="1" max="1" width="3.453125" customWidth="1"/>
+    <col min="2" max="2" width="12.7265625" customWidth="1"/>
     <col min="3" max="3" width="35" customWidth="1"/>
-    <col min="4" max="4" width="57.7109375" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" style="3" customWidth="1"/>
-    <col min="6" max="6" width="4.85546875" customWidth="1"/>
-    <col min="7" max="7" width="7.85546875" customWidth="1"/>
+    <col min="4" max="4" width="57.7265625" customWidth="1"/>
+    <col min="5" max="5" width="10.453125" style="3" customWidth="1"/>
+    <col min="6" max="6" width="4.81640625" customWidth="1"/>
+    <col min="7" max="7" width="7.81640625" customWidth="1"/>
     <col min="8" max="8" width="5" customWidth="1"/>
-    <col min="9" max="9" width="5.5703125" style="2" customWidth="1"/>
-    <col min="10" max="11" width="10.5703125" customWidth="1"/>
-    <col min="12" max="12" width="9.7109375" style="2" customWidth="1"/>
-    <col min="13" max="13" width="7.140625" customWidth="1"/>
+    <col min="9" max="9" width="5.54296875" style="2" customWidth="1"/>
+    <col min="10" max="11" width="10.54296875" customWidth="1"/>
+    <col min="12" max="12" width="9.7265625" style="2" customWidth="1"/>
+    <col min="13" max="13" width="7.1796875" customWidth="1"/>
     <col min="14" max="14" width="14" style="2" customWidth="1"/>
-    <col min="15" max="15" width="10.28515625" customWidth="1"/>
-    <col min="16" max="17" width="13.7109375" customWidth="1"/>
-    <col min="18" max="18" width="9.7109375" style="2" customWidth="1"/>
-    <col min="19" max="19" width="9.7109375" customWidth="1"/>
-    <col min="20" max="20" width="12.140625" customWidth="1"/>
-    <col min="21" max="21" width="17.7109375" style="2" customWidth="1"/>
+    <col min="15" max="15" width="10.26953125" customWidth="1"/>
+    <col min="16" max="17" width="13.7265625" customWidth="1"/>
+    <col min="18" max="18" width="9.7265625" style="2" customWidth="1"/>
+    <col min="19" max="19" width="9.7265625" customWidth="1"/>
+    <col min="20" max="20" width="12.1796875" customWidth="1"/>
+    <col min="21" max="21" width="17.7265625" style="2" customWidth="1"/>
     <col min="22" max="22" width="11" customWidth="1"/>
-    <col min="23" max="23" width="12.28515625" customWidth="1"/>
-    <col min="24" max="24" width="17.140625" style="2" customWidth="1"/>
-    <col min="27" max="27" width="17.7109375" style="2" customWidth="1"/>
-    <col min="28" max="28" width="10.7109375" customWidth="1"/>
+    <col min="23" max="23" width="12.26953125" customWidth="1"/>
+    <col min="24" max="24" width="17.1796875" style="2" customWidth="1"/>
+    <col min="27" max="27" width="17.7265625" style="2" customWidth="1"/>
+    <col min="28" max="28" width="10.7265625" customWidth="1"/>
     <col min="29" max="29" width="11" customWidth="1"/>
-    <col min="30" max="30" width="17.7109375" style="2" customWidth="1"/>
-    <col min="31" max="31" width="12.42578125" customWidth="1"/>
-    <col min="32" max="32" width="12.42578125" style="2" customWidth="1"/>
-    <col min="33" max="33" width="12.28515625" customWidth="1"/>
+    <col min="30" max="30" width="17.7265625" style="2" customWidth="1"/>
+    <col min="31" max="31" width="12.453125" customWidth="1"/>
+    <col min="32" max="32" width="12.453125" style="2" customWidth="1"/>
+    <col min="33" max="33" width="12.26953125" customWidth="1"/>
     <col min="34" max="34" width="9" style="2"/>
-    <col min="35" max="35" width="4.28515625" customWidth="1"/>
+    <col min="35" max="35" width="4.26953125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:36">
@@ -2915,7 +2915,7 @@
         <v>0</v>
       </c>
       <c r="P17">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R17"/>
       <c r="S17" s="3">
@@ -3677,7 +3677,7 @@
         <v>1</v>
       </c>
       <c r="P29">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R29"/>
       <c r="S29" s="3">
@@ -3751,7 +3751,7 @@
         <v>0</v>
       </c>
       <c r="P30">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R30"/>
       <c r="S30" s="3">
@@ -6379,16 +6379,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:I81"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="3.42578125" customWidth="1"/>
-    <col min="2" max="2" width="27.42578125" customWidth="1"/>
+    <col min="1" max="1" width="3.453125" customWidth="1"/>
+    <col min="2" max="2" width="27.453125" customWidth="1"/>
     <col min="3" max="3" width="35" customWidth="1"/>
     <col min="4" max="4" width="33" customWidth="1"/>
-    <col min="5" max="5" width="19.28515625" customWidth="1"/>
-    <col min="6" max="6" width="18.85546875" customWidth="1"/>
-    <col min="7" max="8" width="10.28515625" customWidth="1"/>
-    <col min="9" max="9" width="15.140625" customWidth="1"/>
+    <col min="5" max="5" width="19.26953125" customWidth="1"/>
+    <col min="6" max="6" width="18.81640625" customWidth="1"/>
+    <col min="7" max="8" width="10.26953125" customWidth="1"/>
+    <col min="9" max="9" width="15.1796875" customWidth="1"/>
     <col min="10" max="10" width="22" customWidth="1"/>
   </cols>
   <sheetData>
@@ -8081,17 +8081,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:Q37"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="9.42578125" customWidth="1"/>
-    <col min="2" max="3" width="27.42578125" customWidth="1"/>
-    <col min="4" max="4" width="14.42578125" customWidth="1"/>
-    <col min="5" max="7" width="16.140625" customWidth="1"/>
-    <col min="8" max="8" width="12.42578125" customWidth="1"/>
-    <col min="9" max="9" width="14.42578125" customWidth="1"/>
+    <col min="1" max="1" width="9.453125" customWidth="1"/>
+    <col min="2" max="3" width="27.453125" customWidth="1"/>
+    <col min="4" max="4" width="14.453125" customWidth="1"/>
+    <col min="5" max="7" width="16.1796875" customWidth="1"/>
+    <col min="8" max="8" width="12.453125" customWidth="1"/>
+    <col min="9" max="9" width="14.453125" customWidth="1"/>
     <col min="10" max="10" width="10" customWidth="1"/>
     <col min="11" max="11" width="13" customWidth="1"/>
-    <col min="12" max="12" width="10.140625" customWidth="1"/>
+    <col min="12" max="12" width="10.1796875" customWidth="1"/>
     <col min="13" max="13" width="13" customWidth="1"/>
   </cols>
   <sheetData>
@@ -9109,15 +9109,15 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:G16"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="4.85546875" customWidth="1"/>
-    <col min="2" max="2" width="22.7109375" customWidth="1"/>
-    <col min="3" max="3" width="28.5703125" customWidth="1"/>
-    <col min="4" max="4" width="15.5703125" customWidth="1"/>
-    <col min="5" max="5" width="16.140625" customWidth="1"/>
+    <col min="1" max="1" width="4.81640625" customWidth="1"/>
+    <col min="2" max="2" width="22.7265625" customWidth="1"/>
+    <col min="3" max="3" width="28.54296875" customWidth="1"/>
+    <col min="4" max="4" width="15.54296875" customWidth="1"/>
+    <col min="5" max="5" width="16.1796875" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="11.140625" customWidth="1"/>
+    <col min="7" max="7" width="11.1796875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -9163,7 +9163,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="12.95" customHeight="1">
+    <row r="3" spans="1:7" ht="13" customHeight="1">
       <c r="A3">
         <v>1</v>
       </c>
@@ -9180,7 +9180,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="12.95" customHeight="1">
+    <row r="4" spans="1:7" ht="13" customHeight="1">
       <c r="A4">
         <v>2</v>
       </c>

</xml_diff>

<commit_message>
Raising Animation System 2
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Configurations/Cards.xlsx
+++ b/Assets/StreamingAssets/Configurations/Cards.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity\VTuberSim\Assets\StreamingAssets\Configurations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A4F5C58-5A35-40F9-929B-061F0A10D7FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AADA56E-13CD-462F-AA0F-642CF4C0D21B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25490" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cards" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <sheet name="Conditions" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Cards!$A$1:$AK$74</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Cards!$A$1:$AJ$74</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1073" uniqueCount="485">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1072" uniqueCount="484">
   <si>
     <t>ID</t>
   </si>
@@ -1486,9 +1486,6 @@
   </si>
   <si>
     <t>GreaterEqual</t>
-  </si>
-  <si>
-    <t>第一回合减少层数</t>
   </si>
   <si>
     <t>第一回合时候消耗层数</t>
@@ -1862,7 +1859,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:AK74"/>
+  <dimension ref="A1:AJ74"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="3.42578125" customWidth="1"/>
@@ -1881,24 +1878,24 @@
     <col min="15" max="15" width="10.28515625" customWidth="1"/>
     <col min="16" max="17" width="13.7109375" customWidth="1"/>
     <col min="18" max="18" width="9.7109375" style="2" customWidth="1"/>
-    <col min="19" max="20" width="9.7109375" customWidth="1"/>
-    <col min="21" max="21" width="12.140625" customWidth="1"/>
-    <col min="22" max="22" width="17.7109375" style="2" customWidth="1"/>
-    <col min="23" max="23" width="11" customWidth="1"/>
-    <col min="24" max="24" width="12.28515625" customWidth="1"/>
-    <col min="25" max="25" width="17.140625" style="2" customWidth="1"/>
-    <col min="28" max="28" width="17.7109375" style="2" customWidth="1"/>
-    <col min="29" max="29" width="10.7109375" customWidth="1"/>
-    <col min="30" max="30" width="11" customWidth="1"/>
-    <col min="31" max="31" width="17.7109375" style="2" customWidth="1"/>
-    <col min="32" max="32" width="12.42578125" customWidth="1"/>
-    <col min="33" max="33" width="12.42578125" style="2" customWidth="1"/>
-    <col min="34" max="34" width="12.28515625" customWidth="1"/>
-    <col min="35" max="35" width="9" style="2"/>
-    <col min="36" max="36" width="4.28515625" customWidth="1"/>
+    <col min="19" max="19" width="9.7109375" customWidth="1"/>
+    <col min="20" max="20" width="12.140625" customWidth="1"/>
+    <col min="21" max="21" width="17.7109375" style="2" customWidth="1"/>
+    <col min="22" max="22" width="11" customWidth="1"/>
+    <col min="23" max="23" width="12.28515625" customWidth="1"/>
+    <col min="24" max="24" width="17.140625" style="2" customWidth="1"/>
+    <col min="27" max="27" width="17.7109375" style="2" customWidth="1"/>
+    <col min="28" max="28" width="10.7109375" customWidth="1"/>
+    <col min="29" max="29" width="11" customWidth="1"/>
+    <col min="30" max="30" width="17.7109375" style="2" customWidth="1"/>
+    <col min="31" max="31" width="12.42578125" customWidth="1"/>
+    <col min="32" max="32" width="12.42578125" style="2" customWidth="1"/>
+    <col min="33" max="33" width="12.28515625" customWidth="1"/>
+    <col min="34" max="34" width="9" style="2"/>
+    <col min="35" max="35" width="4.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37">
+    <row r="1" spans="1:36">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1953,62 +1950,59 @@
       <c r="R1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
-        <v>483</v>
-      </c>
-      <c r="T1" s="3" t="s">
+      <c r="S1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="U1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="V1" s="2" t="s">
+      <c r="U1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="W1" s="3" t="s">
+      <c r="V1" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="X1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
-      <c r="Y1" s="2" t="s">
+      <c r="X1" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="Z1" s="3" t="s">
+      <c r="Y1" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="Z1" t="s">
         <v>25</v>
       </c>
-      <c r="AB1" s="2" t="s">
+      <c r="AA1" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="AC1" s="3" t="s">
+      <c r="AB1" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="AD1" t="s">
+      <c r="AC1" t="s">
         <v>28</v>
       </c>
-      <c r="AE1" s="2" t="s">
+      <c r="AD1" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="AF1" s="3" t="s">
+      <c r="AE1" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="AG1" s="2" t="s">
+      <c r="AF1" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="AH1" t="s">
+      <c r="AG1" t="s">
         <v>32</v>
       </c>
-      <c r="AI1" s="2" t="s">
+      <c r="AH1" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="AJ1" t="s">
+      <c r="AI1" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:37">
+    <row r="2" spans="1:36">
       <c r="A2">
         <v>0</v>
       </c>
@@ -2050,26 +2044,23 @@
         <v>0</v>
       </c>
       <c r="R2"/>
-      <c r="S2">
-        <v>0</v>
-      </c>
-      <c r="T2" s="3">
+      <c r="S2" s="3">
         <v>11</v>
       </c>
-      <c r="U2">
+      <c r="T2">
         <v>7</v>
       </c>
-      <c r="V2" s="2">
+      <c r="U2" s="2">
         <v>7</v>
       </c>
-      <c r="Y2"/>
-      <c r="AB2"/>
-      <c r="AE2"/>
-      <c r="AG2"/>
-      <c r="AI2"/>
-      <c r="AJ2" s="6"/>
-    </row>
-    <row r="3" spans="1:37">
+      <c r="X2"/>
+      <c r="AA2"/>
+      <c r="AD2"/>
+      <c r="AF2"/>
+      <c r="AH2"/>
+      <c r="AI2" s="6"/>
+    </row>
+    <row r="3" spans="1:36">
       <c r="A3">
         <v>1</v>
       </c>
@@ -2111,26 +2102,23 @@
         <v>0</v>
       </c>
       <c r="R3"/>
-      <c r="S3">
-        <v>0</v>
-      </c>
-      <c r="T3" s="3">
+      <c r="S3" s="3">
         <v>2</v>
       </c>
-      <c r="U3">
+      <c r="T3">
         <v>4</v>
       </c>
-      <c r="V3" s="2">
+      <c r="U3" s="2">
         <v>4</v>
       </c>
-      <c r="Y3"/>
-      <c r="AB3"/>
-      <c r="AE3"/>
-      <c r="AG3"/>
-      <c r="AI3"/>
-      <c r="AJ3" s="6"/>
-    </row>
-    <row r="4" spans="1:37">
+      <c r="X3"/>
+      <c r="AA3"/>
+      <c r="AD3"/>
+      <c r="AF3"/>
+      <c r="AH3"/>
+      <c r="AI3" s="6"/>
+    </row>
+    <row r="4" spans="1:36">
       <c r="A4">
         <v>2</v>
       </c>
@@ -2170,30 +2158,27 @@
       <c r="P4">
         <v>0</v>
       </c>
-      <c r="S4">
-        <v>0</v>
-      </c>
-      <c r="T4" s="3">
+      <c r="S4" s="3">
         <v>11</v>
       </c>
-      <c r="U4">
+      <c r="T4">
         <v>15</v>
       </c>
-      <c r="V4" s="2">
+      <c r="U4" s="2">
         <v>18</v>
       </c>
+      <c r="V4">
+        <v>56</v>
+      </c>
       <c r="W4">
-        <v>56</v>
-      </c>
-      <c r="X4">
         <v>9</v>
       </c>
-      <c r="Y4" s="2">
+      <c r="X4" s="2">
         <v>12</v>
       </c>
-      <c r="AJ4" s="6"/>
-    </row>
-    <row r="5" spans="1:37">
+      <c r="AI4" s="6"/>
+    </row>
+    <row r="5" spans="1:36">
       <c r="A5">
         <v>3</v>
       </c>
@@ -2235,34 +2220,31 @@
         <v>0</v>
       </c>
       <c r="R5"/>
-      <c r="S5">
-        <v>0</v>
-      </c>
-      <c r="T5" s="3">
+      <c r="S5" s="3">
         <v>11</v>
       </c>
-      <c r="U5">
+      <c r="T5">
         <v>5</v>
       </c>
-      <c r="V5" s="2">
+      <c r="U5" s="2">
         <v>5</v>
       </c>
-      <c r="W5" s="3">
+      <c r="V5" s="3">
         <v>2</v>
       </c>
-      <c r="X5">
+      <c r="W5">
         <v>2</v>
       </c>
-      <c r="Y5" s="2">
+      <c r="X5" s="2">
         <v>2</v>
       </c>
-      <c r="AB5"/>
-      <c r="AE5"/>
-      <c r="AG5"/>
-      <c r="AI5"/>
-      <c r="AJ5" s="6"/>
-    </row>
-    <row r="6" spans="1:37">
+      <c r="AA5"/>
+      <c r="AD5"/>
+      <c r="AF5"/>
+      <c r="AH5"/>
+      <c r="AI5" s="6"/>
+    </row>
+    <row r="6" spans="1:36">
       <c r="A6">
         <v>4</v>
       </c>
@@ -2308,42 +2290,39 @@
       <c r="P6">
         <v>1</v>
       </c>
-      <c r="S6">
-        <v>0</v>
-      </c>
-      <c r="T6" s="3">
-        <v>0</v>
+      <c r="S6" s="3">
+        <v>0</v>
+      </c>
+      <c r="V6">
+        <v>2</v>
       </c>
       <c r="W6">
         <v>2</v>
       </c>
-      <c r="X6">
-        <v>2</v>
-      </c>
-      <c r="Y6" s="2">
+      <c r="X6" s="2">
         <v>7</v>
       </c>
+      <c r="Y6">
+        <v>9</v>
+      </c>
       <c r="Z6">
-        <v>9</v>
-      </c>
-      <c r="AA6">
-        <v>1</v>
-      </c>
-      <c r="AB6" s="2">
-        <v>1</v>
+        <v>1</v>
+      </c>
+      <c r="AA6" s="2">
+        <v>1</v>
+      </c>
+      <c r="AB6">
+        <v>14</v>
       </c>
       <c r="AC6">
-        <v>14</v>
-      </c>
-      <c r="AD6">
-        <v>1</v>
-      </c>
-      <c r="AE6" s="2">
-        <v>1</v>
-      </c>
-      <c r="AJ6" s="6"/>
-    </row>
-    <row r="7" spans="1:37">
+        <v>1</v>
+      </c>
+      <c r="AD6" s="2">
+        <v>1</v>
+      </c>
+      <c r="AI6" s="6"/>
+    </row>
+    <row r="7" spans="1:36">
       <c r="A7">
         <v>5</v>
       </c>
@@ -2385,37 +2364,34 @@
         <v>1</v>
       </c>
       <c r="R7"/>
-      <c r="S7">
-        <v>0</v>
-      </c>
-      <c r="T7" s="3">
+      <c r="S7" s="3">
         <v>4</v>
       </c>
-      <c r="V7"/>
-      <c r="W7" s="3">
+      <c r="U7"/>
+      <c r="V7" s="3">
         <v>21</v>
       </c>
-      <c r="X7">
+      <c r="W7">
         <v>2</v>
       </c>
-      <c r="Y7" s="2">
+      <c r="X7" s="2">
         <v>2</v>
       </c>
-      <c r="Z7" s="3">
+      <c r="Y7" s="3">
         <v>14</v>
       </c>
-      <c r="AA7">
-        <v>1</v>
-      </c>
-      <c r="AB7" s="2">
-        <v>1</v>
-      </c>
-      <c r="AE7"/>
-      <c r="AG7"/>
-      <c r="AI7"/>
-      <c r="AJ7" s="6"/>
-    </row>
-    <row r="8" spans="1:37" hidden="1">
+      <c r="Z7">
+        <v>1</v>
+      </c>
+      <c r="AA7" s="2">
+        <v>1</v>
+      </c>
+      <c r="AD7"/>
+      <c r="AF7"/>
+      <c r="AH7"/>
+      <c r="AI7" s="6"/>
+    </row>
+    <row r="8" spans="1:36" hidden="1">
       <c r="A8">
         <v>6</v>
       </c>
@@ -2456,39 +2432,39 @@
         <v>1</v>
       </c>
       <c r="R8"/>
-      <c r="T8" s="3">
+      <c r="S8" s="3">
         <v>2</v>
       </c>
-      <c r="U8">
+      <c r="T8">
         <v>7</v>
       </c>
-      <c r="V8" s="2">
+      <c r="U8" s="2">
         <v>7</v>
       </c>
-      <c r="W8" s="3">
+      <c r="V8" s="3">
         <v>3</v>
       </c>
-      <c r="X8">
-        <v>1</v>
-      </c>
-      <c r="Y8" s="2">
-        <v>1</v>
-      </c>
-      <c r="Z8" s="3">
+      <c r="W8">
+        <v>1</v>
+      </c>
+      <c r="X8" s="2">
+        <v>1</v>
+      </c>
+      <c r="Y8" s="3">
         <v>14</v>
       </c>
-      <c r="AA8">
-        <v>1</v>
-      </c>
-      <c r="AB8" s="2">
-        <v>1</v>
-      </c>
-      <c r="AE8"/>
-      <c r="AG8"/>
-      <c r="AI8"/>
-      <c r="AJ8" s="6"/>
-    </row>
-    <row r="9" spans="1:37" hidden="1">
+      <c r="Z8">
+        <v>1</v>
+      </c>
+      <c r="AA8" s="2">
+        <v>1</v>
+      </c>
+      <c r="AD8"/>
+      <c r="AF8"/>
+      <c r="AH8"/>
+      <c r="AI8" s="6"/>
+    </row>
+    <row r="9" spans="1:36" hidden="1">
       <c r="A9">
         <v>8</v>
       </c>
@@ -2527,31 +2503,31 @@
         <v>0</v>
       </c>
       <c r="R9"/>
-      <c r="T9" s="3">
+      <c r="S9" s="3">
         <v>6</v>
       </c>
-      <c r="U9">
+      <c r="T9">
         <v>3</v>
       </c>
-      <c r="V9" s="2">
+      <c r="U9" s="2">
         <v>4</v>
       </c>
-      <c r="W9" s="3">
+      <c r="V9" s="3">
         <v>2</v>
       </c>
-      <c r="X9">
+      <c r="W9">
         <v>3</v>
       </c>
-      <c r="Y9" s="2">
+      <c r="X9" s="2">
         <v>4</v>
       </c>
-      <c r="AB9"/>
-      <c r="AE9"/>
-      <c r="AG9"/>
-      <c r="AI9"/>
-      <c r="AJ9" s="6"/>
-    </row>
-    <row r="10" spans="1:37" hidden="1">
+      <c r="AA9"/>
+      <c r="AD9"/>
+      <c r="AF9"/>
+      <c r="AH9"/>
+      <c r="AI9" s="6"/>
+    </row>
+    <row r="10" spans="1:36" hidden="1">
       <c r="A10">
         <v>9</v>
       </c>
@@ -2590,31 +2566,31 @@
         <v>0</v>
       </c>
       <c r="R10"/>
-      <c r="T10" s="3">
+      <c r="S10" s="3">
         <v>7</v>
       </c>
-      <c r="U10">
+      <c r="T10">
         <v>2</v>
       </c>
-      <c r="V10" s="2">
+      <c r="U10" s="2">
         <v>3</v>
       </c>
-      <c r="W10" s="3">
+      <c r="V10" s="3">
         <v>2</v>
       </c>
-      <c r="X10">
+      <c r="W10">
         <v>2</v>
       </c>
-      <c r="Y10" s="2">
+      <c r="X10" s="2">
         <v>3</v>
       </c>
-      <c r="AB10"/>
-      <c r="AE10"/>
-      <c r="AG10"/>
-      <c r="AI10"/>
-      <c r="AJ10" s="6"/>
-    </row>
-    <row r="11" spans="1:37">
+      <c r="AA10"/>
+      <c r="AD10"/>
+      <c r="AF10"/>
+      <c r="AH10"/>
+      <c r="AI10" s="6"/>
+    </row>
+    <row r="11" spans="1:36">
       <c r="A11">
         <v>10</v>
       </c>
@@ -2654,30 +2630,27 @@
       <c r="P11">
         <v>0</v>
       </c>
-      <c r="S11">
-        <v>0</v>
-      </c>
-      <c r="T11" s="3">
+      <c r="S11" s="3">
         <v>15</v>
       </c>
-      <c r="U11">
+      <c r="T11">
         <v>2</v>
       </c>
-      <c r="V11" s="2">
+      <c r="U11" s="2">
         <v>3</v>
       </c>
-      <c r="W11" s="3">
+      <c r="V11" s="3">
         <v>2</v>
       </c>
-      <c r="X11">
+      <c r="W11">
         <v>2</v>
       </c>
-      <c r="Y11" s="2">
+      <c r="X11" s="2">
         <v>3</v>
       </c>
-      <c r="AJ11" s="6"/>
-    </row>
-    <row r="12" spans="1:37" hidden="1">
+      <c r="AI11" s="6"/>
+    </row>
+    <row r="12" spans="1:36" hidden="1">
       <c r="A12">
         <v>11</v>
       </c>
@@ -2716,34 +2689,34 @@
         <v>0</v>
       </c>
       <c r="R12"/>
-      <c r="T12" s="3">
+      <c r="S12" s="3">
         <v>11</v>
       </c>
-      <c r="U12">
+      <c r="T12">
         <v>9</v>
       </c>
-      <c r="V12" s="2">
+      <c r="U12" s="2">
         <v>13</v>
       </c>
-      <c r="W12" s="3">
+      <c r="V12" s="3">
         <v>11</v>
       </c>
-      <c r="X12">
+      <c r="W12">
         <v>9</v>
       </c>
-      <c r="Y12" s="2">
+      <c r="X12" s="2">
         <v>13</v>
       </c>
-      <c r="AB12"/>
-      <c r="AE12"/>
-      <c r="AG12"/>
-      <c r="AI12"/>
-      <c r="AJ12" s="6"/>
-      <c r="AK12" t="s">
+      <c r="AA12"/>
+      <c r="AD12"/>
+      <c r="AF12"/>
+      <c r="AH12"/>
+      <c r="AI12" s="6"/>
+      <c r="AJ12" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="13" spans="1:37">
+    <row r="13" spans="1:36">
       <c r="A13">
         <v>12</v>
       </c>
@@ -2782,34 +2755,31 @@
         <v>0</v>
       </c>
       <c r="R13"/>
-      <c r="S13">
-        <v>0</v>
-      </c>
-      <c r="T13" s="3">
+      <c r="S13" s="3">
         <v>11</v>
       </c>
-      <c r="U13">
+      <c r="T13">
         <v>11</v>
       </c>
-      <c r="V13" s="2">
+      <c r="U13" s="2">
         <v>15</v>
       </c>
-      <c r="W13" s="3">
+      <c r="V13" s="3">
         <v>2</v>
       </c>
-      <c r="X13">
+      <c r="W13">
         <v>7</v>
       </c>
-      <c r="Y13" s="2">
+      <c r="X13" s="2">
         <v>9</v>
       </c>
-      <c r="AB13"/>
-      <c r="AE13"/>
-      <c r="AG13"/>
-      <c r="AI13"/>
-      <c r="AJ13" s="6"/>
-    </row>
-    <row r="14" spans="1:37" hidden="1">
+      <c r="AA13"/>
+      <c r="AD13"/>
+      <c r="AF13"/>
+      <c r="AH13"/>
+      <c r="AI13" s="6"/>
+    </row>
+    <row r="14" spans="1:36" hidden="1">
       <c r="A14">
         <v>13</v>
       </c>
@@ -2848,23 +2818,23 @@
         <v>0</v>
       </c>
       <c r="R14"/>
-      <c r="T14" s="3">
+      <c r="S14" s="3">
         <v>6</v>
       </c>
-      <c r="U14">
+      <c r="T14">
         <v>6</v>
       </c>
-      <c r="V14" s="2">
+      <c r="U14" s="2">
         <v>8</v>
       </c>
-      <c r="Y14"/>
-      <c r="AB14"/>
-      <c r="AE14"/>
-      <c r="AG14"/>
-      <c r="AI14"/>
-      <c r="AJ14" s="6"/>
-    </row>
-    <row r="15" spans="1:37" hidden="1">
+      <c r="X14"/>
+      <c r="AA14"/>
+      <c r="AD14"/>
+      <c r="AF14"/>
+      <c r="AH14"/>
+      <c r="AI14" s="6"/>
+    </row>
+    <row r="15" spans="1:36" hidden="1">
       <c r="A15">
         <v>14</v>
       </c>
@@ -2903,23 +2873,23 @@
         <v>0</v>
       </c>
       <c r="R15"/>
-      <c r="T15" s="3">
+      <c r="S15" s="3">
         <v>18</v>
       </c>
-      <c r="U15">
+      <c r="T15">
         <v>1.4</v>
       </c>
-      <c r="V15" s="2">
+      <c r="U15" s="2">
         <v>1.8</v>
       </c>
-      <c r="Y15"/>
-      <c r="AB15"/>
-      <c r="AE15"/>
-      <c r="AG15"/>
-      <c r="AI15"/>
-      <c r="AJ15" s="6"/>
-    </row>
-    <row r="16" spans="1:37" hidden="1">
+      <c r="X15"/>
+      <c r="AA15"/>
+      <c r="AD15"/>
+      <c r="AF15"/>
+      <c r="AH15"/>
+      <c r="AI15" s="6"/>
+    </row>
+    <row r="16" spans="1:36" hidden="1">
       <c r="A16">
         <v>15</v>
       </c>
@@ -2958,31 +2928,31 @@
         <v>0</v>
       </c>
       <c r="R16"/>
-      <c r="T16" s="3">
+      <c r="S16" s="3">
         <v>6</v>
       </c>
-      <c r="U16">
+      <c r="T16">
         <v>4</v>
       </c>
-      <c r="V16" s="2">
+      <c r="U16" s="2">
         <v>5</v>
       </c>
-      <c r="W16" s="3">
+      <c r="V16" s="3">
         <v>18</v>
       </c>
-      <c r="X16">
+      <c r="W16">
         <v>0.8</v>
       </c>
-      <c r="Y16" s="2">
+      <c r="X16" s="2">
         <v>1.1000000000000001</v>
       </c>
-      <c r="AB16"/>
-      <c r="AE16"/>
-      <c r="AG16"/>
-      <c r="AI16"/>
-      <c r="AJ16" s="6"/>
-    </row>
-    <row r="17" spans="1:36">
+      <c r="AA16"/>
+      <c r="AD16"/>
+      <c r="AF16"/>
+      <c r="AH16"/>
+      <c r="AI16" s="6"/>
+    </row>
+    <row r="17" spans="1:35">
       <c r="A17">
         <v>16</v>
       </c>
@@ -3027,42 +2997,39 @@
         <v>0</v>
       </c>
       <c r="R17"/>
-      <c r="S17">
-        <v>0</v>
-      </c>
-      <c r="T17" s="3">
+      <c r="S17" s="3">
         <v>19</v>
       </c>
-      <c r="U17">
-        <v>1</v>
-      </c>
-      <c r="V17" s="2">
-        <v>1</v>
-      </c>
-      <c r="W17" s="3">
+      <c r="T17">
+        <v>1</v>
+      </c>
+      <c r="U17" s="2">
+        <v>1</v>
+      </c>
+      <c r="V17" s="3">
         <v>2</v>
       </c>
-      <c r="X17">
+      <c r="W17">
         <v>4</v>
       </c>
-      <c r="Y17" s="2">
+      <c r="X17" s="2">
         <v>6</v>
       </c>
-      <c r="Z17" s="3">
+      <c r="Y17" s="3">
         <v>21</v>
       </c>
-      <c r="AA17">
+      <c r="Z17">
         <v>2</v>
       </c>
-      <c r="AB17" s="2">
+      <c r="AA17" s="2">
         <v>3</v>
       </c>
-      <c r="AE17"/>
-      <c r="AG17"/>
-      <c r="AI17"/>
-      <c r="AJ17" s="7"/>
-    </row>
-    <row r="18" spans="1:36">
+      <c r="AD17"/>
+      <c r="AF17"/>
+      <c r="AH17"/>
+      <c r="AI17" s="7"/>
+    </row>
+    <row r="18" spans="1:35">
       <c r="A18">
         <v>18</v>
       </c>
@@ -3102,27 +3069,24 @@
       <c r="P18">
         <v>0</v>
       </c>
-      <c r="S18">
-        <v>0</v>
-      </c>
-      <c r="T18" s="3">
+      <c r="S18" s="3">
         <v>15</v>
       </c>
-      <c r="U18">
+      <c r="T18">
         <v>5</v>
       </c>
-      <c r="V18" s="2">
+      <c r="U18" s="2">
         <v>7</v>
       </c>
-      <c r="AF18">
+      <c r="AE18">
         <v>63</v>
       </c>
-      <c r="AG18" s="2">
+      <c r="AF18" s="2">
         <v>1.5</v>
       </c>
-      <c r="AJ18" s="6"/>
-    </row>
-    <row r="19" spans="1:36" hidden="1">
+      <c r="AI18" s="6"/>
+    </row>
+    <row r="19" spans="1:35" hidden="1">
       <c r="A19">
         <v>19</v>
       </c>
@@ -3161,31 +3125,31 @@
         <v>1</v>
       </c>
       <c r="R19"/>
-      <c r="T19" s="3">
+      <c r="S19" s="3">
         <v>23</v>
       </c>
-      <c r="U19">
-        <v>1</v>
-      </c>
-      <c r="V19" s="2">
-        <v>1</v>
-      </c>
-      <c r="W19" s="3">
+      <c r="T19">
+        <v>1</v>
+      </c>
+      <c r="U19" s="2">
+        <v>1</v>
+      </c>
+      <c r="V19" s="3">
         <v>7</v>
       </c>
-      <c r="X19">
-        <v>1</v>
-      </c>
-      <c r="Y19" s="2">
+      <c r="W19">
+        <v>1</v>
+      </c>
+      <c r="X19" s="2">
         <v>2</v>
       </c>
-      <c r="AB19"/>
-      <c r="AE19"/>
-      <c r="AG19"/>
-      <c r="AI19"/>
-      <c r="AJ19" s="6"/>
-    </row>
-    <row r="20" spans="1:36">
+      <c r="AA19"/>
+      <c r="AD19"/>
+      <c r="AF19"/>
+      <c r="AH19"/>
+      <c r="AI19" s="6"/>
+    </row>
+    <row r="20" spans="1:35">
       <c r="A20">
         <v>20</v>
       </c>
@@ -3228,27 +3192,24 @@
       <c r="R20" s="2">
         <v>0</v>
       </c>
-      <c r="S20">
-        <v>0</v>
-      </c>
-      <c r="T20" s="3">
+      <c r="S20" s="3">
         <v>11</v>
       </c>
-      <c r="U20">
+      <c r="T20">
         <v>24</v>
       </c>
-      <c r="V20" s="2">
+      <c r="U20" s="2">
         <v>30</v>
       </c>
-      <c r="AF20">
+      <c r="AE20">
         <v>62</v>
       </c>
-      <c r="AG20" s="2">
+      <c r="AF20" s="2">
         <v>7</v>
       </c>
-      <c r="AJ20" s="7"/>
-    </row>
-    <row r="21" spans="1:36">
+      <c r="AI20" s="7"/>
+    </row>
+    <row r="21" spans="1:35">
       <c r="A21">
         <v>21</v>
       </c>
@@ -3288,39 +3249,36 @@
       <c r="P21">
         <v>1</v>
       </c>
-      <c r="S21">
-        <v>0</v>
-      </c>
-      <c r="T21" s="3">
+      <c r="S21" s="3">
         <v>26</v>
       </c>
-      <c r="U21">
+      <c r="T21">
         <v>2</v>
       </c>
-      <c r="V21" s="2">
+      <c r="U21" s="2">
         <v>2</v>
       </c>
-      <c r="W21" s="3">
+      <c r="V21" s="3">
         <v>11</v>
       </c>
-      <c r="X21">
+      <c r="W21">
         <v>30</v>
       </c>
-      <c r="Y21" s="2">
+      <c r="X21" s="2">
         <v>42</v>
       </c>
+      <c r="Y21">
+        <v>2</v>
+      </c>
       <c r="Z21">
-        <v>2</v>
-      </c>
-      <c r="AA21">
         <v>5</v>
       </c>
-      <c r="AB21" s="2">
+      <c r="AA21" s="2">
         <v>7</v>
       </c>
-      <c r="AJ21" s="6"/>
-    </row>
-    <row r="22" spans="1:36" hidden="1">
+      <c r="AI21" s="6"/>
+    </row>
+    <row r="22" spans="1:35" hidden="1">
       <c r="A22">
         <v>22</v>
       </c>
@@ -3359,31 +3317,31 @@
         <v>1</v>
       </c>
       <c r="R22"/>
-      <c r="T22" s="3">
+      <c r="S22" s="3">
         <v>6</v>
       </c>
-      <c r="U22">
+      <c r="T22">
         <v>2</v>
       </c>
-      <c r="V22" s="2">
+      <c r="U22" s="2">
         <v>4</v>
       </c>
-      <c r="W22" s="3">
+      <c r="V22" s="3">
         <v>28</v>
       </c>
-      <c r="X22">
-        <v>1</v>
-      </c>
-      <c r="Y22" s="2">
-        <v>1</v>
-      </c>
-      <c r="AB22"/>
-      <c r="AE22"/>
-      <c r="AG22"/>
-      <c r="AI22"/>
-      <c r="AJ22" s="6"/>
-    </row>
-    <row r="23" spans="1:36" hidden="1">
+      <c r="W22">
+        <v>1</v>
+      </c>
+      <c r="X22" s="2">
+        <v>1</v>
+      </c>
+      <c r="AA22"/>
+      <c r="AD22"/>
+      <c r="AF22"/>
+      <c r="AH22"/>
+      <c r="AI22" s="6"/>
+    </row>
+    <row r="23" spans="1:35" hidden="1">
       <c r="A23">
         <v>23</v>
       </c>
@@ -3422,31 +3380,31 @@
         <v>0</v>
       </c>
       <c r="R23"/>
-      <c r="T23" s="3">
+      <c r="S23" s="3">
         <v>6</v>
       </c>
-      <c r="U23">
+      <c r="T23">
         <v>5</v>
       </c>
-      <c r="V23" s="2">
+      <c r="U23" s="2">
         <v>7</v>
       </c>
-      <c r="W23" s="3">
+      <c r="V23" s="3">
         <v>2</v>
       </c>
-      <c r="X23">
-        <v>1</v>
-      </c>
-      <c r="Y23" s="2">
-        <v>1</v>
-      </c>
-      <c r="AB23"/>
-      <c r="AE23"/>
-      <c r="AG23"/>
-      <c r="AI23"/>
-      <c r="AJ23" s="6"/>
-    </row>
-    <row r="24" spans="1:36">
+      <c r="W23">
+        <v>1</v>
+      </c>
+      <c r="X23" s="2">
+        <v>1</v>
+      </c>
+      <c r="AA23"/>
+      <c r="AD23"/>
+      <c r="AF23"/>
+      <c r="AH23"/>
+      <c r="AI23" s="6"/>
+    </row>
+    <row r="24" spans="1:35">
       <c r="A24">
         <v>24</v>
       </c>
@@ -3486,36 +3444,33 @@
       <c r="P24">
         <v>0</v>
       </c>
-      <c r="S24">
-        <v>0</v>
-      </c>
-      <c r="T24" s="3">
+      <c r="S24" s="3">
         <v>15</v>
       </c>
-      <c r="U24">
+      <c r="T24">
         <v>3</v>
       </c>
-      <c r="V24" s="2">
+      <c r="U24" s="2">
         <v>4</v>
       </c>
-      <c r="W24" s="3">
+      <c r="V24" s="3">
         <v>11</v>
       </c>
-      <c r="X24">
+      <c r="W24">
         <v>8</v>
       </c>
-      <c r="Y24" s="2">
+      <c r="X24" s="2">
         <v>11</v>
       </c>
-      <c r="AF24">
+      <c r="AE24">
         <v>63</v>
       </c>
-      <c r="AG24" s="2">
+      <c r="AF24" s="2">
         <v>3</v>
       </c>
-      <c r="AJ24" s="6"/>
-    </row>
-    <row r="25" spans="1:36" hidden="1">
+      <c r="AI24" s="6"/>
+    </row>
+    <row r="25" spans="1:35" hidden="1">
       <c r="A25">
         <v>25</v>
       </c>
@@ -3554,23 +3509,23 @@
         <v>0</v>
       </c>
       <c r="R25"/>
-      <c r="T25" s="3">
+      <c r="S25" s="3">
         <v>7</v>
       </c>
-      <c r="U25">
+      <c r="T25">
         <v>3</v>
       </c>
-      <c r="V25" s="2">
+      <c r="U25" s="2">
         <v>5</v>
       </c>
-      <c r="Y25"/>
-      <c r="AB25"/>
-      <c r="AE25"/>
-      <c r="AG25"/>
-      <c r="AI25"/>
-      <c r="AJ25" s="6"/>
-    </row>
-    <row r="26" spans="1:36" hidden="1">
+      <c r="X25"/>
+      <c r="AA25"/>
+      <c r="AD25"/>
+      <c r="AF25"/>
+      <c r="AH25"/>
+      <c r="AI25" s="6"/>
+    </row>
+    <row r="26" spans="1:35" hidden="1">
       <c r="A26">
         <v>26</v>
       </c>
@@ -3609,31 +3564,31 @@
         <v>0</v>
       </c>
       <c r="R26"/>
-      <c r="T26" s="3">
+      <c r="S26" s="3">
         <v>7</v>
       </c>
-      <c r="U26">
+      <c r="T26">
         <v>3</v>
       </c>
-      <c r="V26" s="2">
+      <c r="U26" s="2">
         <v>4</v>
       </c>
-      <c r="W26" s="3">
+      <c r="V26" s="3">
         <v>2</v>
       </c>
-      <c r="X26">
+      <c r="W26">
         <v>4</v>
       </c>
-      <c r="Y26" s="2">
+      <c r="X26" s="2">
         <v>6</v>
       </c>
-      <c r="AB26"/>
-      <c r="AE26"/>
-      <c r="AG26"/>
-      <c r="AI26"/>
-      <c r="AJ26" s="6"/>
-    </row>
-    <row r="27" spans="1:36">
+      <c r="AA26"/>
+      <c r="AD26"/>
+      <c r="AF26"/>
+      <c r="AH26"/>
+      <c r="AI26" s="6"/>
+    </row>
+    <row r="27" spans="1:35">
       <c r="A27">
         <v>27</v>
       </c>
@@ -3676,39 +3631,36 @@
       <c r="R27" s="2">
         <v>0</v>
       </c>
-      <c r="S27">
-        <v>0</v>
-      </c>
-      <c r="T27" s="3">
+      <c r="S27" s="3">
         <v>11</v>
       </c>
-      <c r="U27">
+      <c r="T27">
         <v>12</v>
       </c>
-      <c r="V27" s="2">
+      <c r="U27" s="2">
         <v>18</v>
       </c>
-      <c r="W27" s="3">
+      <c r="V27" s="3">
         <v>56</v>
       </c>
-      <c r="X27">
+      <c r="W27">
         <v>24</v>
       </c>
-      <c r="Y27" s="2">
+      <c r="X27" s="2">
         <v>30</v>
       </c>
+      <c r="Y27">
+        <v>57</v>
+      </c>
       <c r="Z27">
-        <v>57</v>
-      </c>
-      <c r="AA27">
         <v>36</v>
       </c>
-      <c r="AB27" s="2">
+      <c r="AA27" s="2">
         <v>44</v>
       </c>
-      <c r="AJ27" s="7"/>
-    </row>
-    <row r="28" spans="1:36">
+      <c r="AI27" s="7"/>
+    </row>
+    <row r="28" spans="1:35">
       <c r="A28">
         <v>28</v>
       </c>
@@ -3748,27 +3700,24 @@
       <c r="P28">
         <v>0</v>
       </c>
-      <c r="S28">
-        <v>0</v>
-      </c>
-      <c r="T28" s="3">
+      <c r="S28" s="3">
         <v>2</v>
       </c>
-      <c r="U28">
+      <c r="T28">
         <v>6</v>
       </c>
-      <c r="V28" s="2">
+      <c r="U28" s="2">
         <v>8</v>
       </c>
-      <c r="AF28">
+      <c r="AE28">
         <v>21</v>
       </c>
-      <c r="AG28" s="2">
+      <c r="AF28" s="2">
         <v>12</v>
       </c>
-      <c r="AJ28" s="6"/>
-    </row>
-    <row r="29" spans="1:36">
+      <c r="AI28" s="6"/>
+    </row>
+    <row r="29" spans="1:35">
       <c r="A29">
         <v>30</v>
       </c>
@@ -3813,42 +3762,39 @@
         <v>0</v>
       </c>
       <c r="R29"/>
-      <c r="S29">
-        <v>0</v>
-      </c>
-      <c r="T29" s="3">
+      <c r="S29" s="3">
         <v>32</v>
       </c>
-      <c r="U29">
+      <c r="T29">
         <v>30</v>
       </c>
-      <c r="V29" s="2">
+      <c r="U29" s="2">
         <v>30</v>
       </c>
-      <c r="W29" s="3">
+      <c r="V29" s="3">
         <v>2</v>
       </c>
-      <c r="X29">
+      <c r="W29">
         <v>3</v>
       </c>
-      <c r="Y29" s="2">
+      <c r="X29" s="2">
         <v>5</v>
       </c>
-      <c r="Z29" s="3">
+      <c r="Y29" s="3">
         <v>21</v>
       </c>
-      <c r="AA29">
+      <c r="Z29">
         <v>2</v>
       </c>
-      <c r="AB29" s="2">
+      <c r="AA29" s="2">
         <v>3</v>
       </c>
-      <c r="AE29"/>
-      <c r="AG29"/>
-      <c r="AI29"/>
-      <c r="AJ29" s="6"/>
-    </row>
-    <row r="30" spans="1:36">
+      <c r="AD29"/>
+      <c r="AF29"/>
+      <c r="AH29"/>
+      <c r="AI29" s="6"/>
+    </row>
+    <row r="30" spans="1:35">
       <c r="A30">
         <v>31</v>
       </c>
@@ -3893,34 +3839,31 @@
         <v>0</v>
       </c>
       <c r="R30"/>
-      <c r="S30">
-        <v>0</v>
-      </c>
-      <c r="T30" s="3">
+      <c r="S30" s="3">
         <v>33</v>
       </c>
-      <c r="U30">
+      <c r="T30">
         <v>50</v>
       </c>
-      <c r="V30" s="2">
+      <c r="U30" s="2">
         <v>70</v>
       </c>
-      <c r="W30" s="3">
+      <c r="V30" s="3">
         <v>2</v>
       </c>
-      <c r="X30">
+      <c r="W30">
         <v>2</v>
       </c>
-      <c r="Y30" s="2">
+      <c r="X30" s="2">
         <v>4</v>
       </c>
-      <c r="AB30"/>
-      <c r="AE30"/>
-      <c r="AG30"/>
-      <c r="AI30"/>
-      <c r="AJ30" s="7"/>
-    </row>
-    <row r="31" spans="1:36">
+      <c r="AA30"/>
+      <c r="AD30"/>
+      <c r="AF30"/>
+      <c r="AH30"/>
+      <c r="AI30" s="7"/>
+    </row>
+    <row r="31" spans="1:35">
       <c r="A31">
         <v>32</v>
       </c>
@@ -3962,34 +3905,31 @@
         <v>1</v>
       </c>
       <c r="R31"/>
-      <c r="S31">
-        <v>0</v>
-      </c>
-      <c r="T31" s="3">
+      <c r="S31" s="3">
         <v>33</v>
       </c>
-      <c r="U31">
+      <c r="T31">
         <v>20</v>
       </c>
-      <c r="V31" s="2">
+      <c r="U31" s="2">
         <v>30</v>
       </c>
-      <c r="W31" s="3">
+      <c r="V31" s="3">
         <v>35</v>
       </c>
-      <c r="X31">
-        <v>1</v>
-      </c>
-      <c r="Y31" s="2">
-        <v>1</v>
-      </c>
-      <c r="AB31"/>
-      <c r="AE31"/>
-      <c r="AG31"/>
-      <c r="AI31"/>
-      <c r="AJ31" s="7"/>
-    </row>
-    <row r="32" spans="1:36">
+      <c r="W31">
+        <v>1</v>
+      </c>
+      <c r="X31" s="2">
+        <v>1</v>
+      </c>
+      <c r="AA31"/>
+      <c r="AD31"/>
+      <c r="AF31"/>
+      <c r="AH31"/>
+      <c r="AI31" s="7"/>
+    </row>
+    <row r="32" spans="1:35">
       <c r="A32">
         <v>33</v>
       </c>
@@ -4034,17 +3974,14 @@
         <v>1</v>
       </c>
       <c r="R32"/>
-      <c r="S32">
-        <v>0</v>
-      </c>
-      <c r="V32"/>
-      <c r="Y32"/>
-      <c r="AB32"/>
-      <c r="AE32"/>
-      <c r="AG32"/>
-      <c r="AI32"/>
-    </row>
-    <row r="33" spans="1:35">
+      <c r="U32"/>
+      <c r="X32"/>
+      <c r="AA32"/>
+      <c r="AD32"/>
+      <c r="AF32"/>
+      <c r="AH32"/>
+    </row>
+    <row r="33" spans="1:34">
       <c r="A33">
         <v>34</v>
       </c>
@@ -4084,35 +4021,32 @@
       <c r="P33">
         <v>1</v>
       </c>
-      <c r="S33">
-        <v>0</v>
-      </c>
-      <c r="T33" s="3">
+      <c r="S33" s="3">
         <v>11</v>
       </c>
-      <c r="U33">
+      <c r="T33">
         <v>38</v>
       </c>
-      <c r="V33" s="2">
+      <c r="U33" s="2">
         <v>52</v>
       </c>
+      <c r="V33">
+        <v>78</v>
+      </c>
       <c r="W33">
-        <v>78</v>
-      </c>
-      <c r="X33">
-        <v>1</v>
-      </c>
-      <c r="Y33" s="2">
-        <v>1</v>
-      </c>
-      <c r="AF33">
+        <v>1</v>
+      </c>
+      <c r="X33" s="2">
+        <v>1</v>
+      </c>
+      <c r="AE33">
         <v>64</v>
       </c>
-      <c r="AG33" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34" spans="1:35">
+      <c r="AF33" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:34">
       <c r="A34">
         <v>35</v>
       </c>
@@ -4152,29 +4086,26 @@
       <c r="P34">
         <v>1</v>
       </c>
-      <c r="S34">
-        <v>0</v>
-      </c>
-      <c r="T34" s="3">
+      <c r="S34" s="3">
         <v>15</v>
       </c>
-      <c r="U34">
+      <c r="T34">
         <v>3</v>
       </c>
-      <c r="V34" s="2">
+      <c r="U34" s="2">
         <v>4</v>
       </c>
+      <c r="V34">
+        <v>52</v>
+      </c>
       <c r="W34">
-        <v>52</v>
-      </c>
-      <c r="X34">
         <v>3</v>
       </c>
-      <c r="Y34" s="2">
+      <c r="X34" s="2">
         <v>4</v>
       </c>
     </row>
-    <row r="35" spans="1:35">
+    <row r="35" spans="1:34">
       <c r="A35">
         <v>36</v>
       </c>
@@ -4214,29 +4145,26 @@
       <c r="P35">
         <v>0</v>
       </c>
-      <c r="S35">
-        <v>0</v>
-      </c>
-      <c r="T35" s="3">
+      <c r="S35" s="3">
         <v>45</v>
       </c>
-      <c r="U35">
-        <v>1</v>
-      </c>
-      <c r="V35" s="2">
+      <c r="T35">
+        <v>1</v>
+      </c>
+      <c r="U35" s="2">
         <v>3</v>
       </c>
+      <c r="V35">
+        <v>74</v>
+      </c>
       <c r="W35">
-        <v>74</v>
-      </c>
-      <c r="X35">
-        <v>1</v>
-      </c>
-      <c r="Y35" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="36" spans="1:35">
+        <v>1</v>
+      </c>
+      <c r="X35" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:34">
       <c r="A36">
         <v>37</v>
       </c>
@@ -4276,29 +4204,26 @@
       <c r="P36">
         <v>0</v>
       </c>
-      <c r="S36">
-        <v>0</v>
-      </c>
-      <c r="T36" s="3">
+      <c r="S36" s="3">
         <v>15</v>
       </c>
-      <c r="U36">
+      <c r="T36">
         <v>3</v>
       </c>
-      <c r="V36" s="2">
+      <c r="U36" s="2">
         <v>4</v>
       </c>
-      <c r="W36" s="3">
+      <c r="V36" s="3">
         <v>2</v>
       </c>
-      <c r="X36">
+      <c r="W36">
         <v>6</v>
       </c>
-      <c r="Y36" s="2">
+      <c r="X36" s="2">
         <v>8</v>
       </c>
     </row>
-    <row r="37" spans="1:35" hidden="1">
+    <row r="37" spans="1:34" hidden="1">
       <c r="A37">
         <v>38</v>
       </c>
@@ -4337,30 +4262,30 @@
         <v>0</v>
       </c>
       <c r="R37"/>
-      <c r="T37" s="3">
+      <c r="S37" s="3">
         <v>7</v>
       </c>
-      <c r="U37">
+      <c r="T37">
         <v>3</v>
       </c>
-      <c r="V37" s="2">
+      <c r="U37" s="2">
         <v>4</v>
       </c>
-      <c r="W37" s="3">
+      <c r="V37" s="3">
         <v>2</v>
       </c>
-      <c r="X37">
+      <c r="W37">
         <v>6</v>
       </c>
-      <c r="Y37" s="2">
+      <c r="X37" s="2">
         <v>8</v>
       </c>
-      <c r="AB37"/>
-      <c r="AE37"/>
-      <c r="AG37"/>
-      <c r="AI37"/>
-    </row>
-    <row r="38" spans="1:35">
+      <c r="AA37"/>
+      <c r="AD37"/>
+      <c r="AF37"/>
+      <c r="AH37"/>
+    </row>
+    <row r="38" spans="1:34">
       <c r="A38">
         <v>39</v>
       </c>
@@ -4402,33 +4327,30 @@
         <v>1</v>
       </c>
       <c r="R38"/>
-      <c r="S38">
-        <v>0</v>
-      </c>
-      <c r="T38" s="3">
+      <c r="S38" s="3">
         <v>21</v>
       </c>
-      <c r="U38">
+      <c r="T38">
         <v>4</v>
       </c>
-      <c r="V38" s="2">
+      <c r="U38" s="2">
         <v>5</v>
       </c>
-      <c r="W38" s="3">
+      <c r="V38" s="3">
         <v>2</v>
       </c>
-      <c r="X38">
+      <c r="W38">
         <v>3</v>
       </c>
-      <c r="Y38" s="2">
+      <c r="X38" s="2">
         <v>5</v>
       </c>
-      <c r="AB38"/>
-      <c r="AE38"/>
-      <c r="AG38"/>
-      <c r="AI38"/>
-    </row>
-    <row r="39" spans="1:35">
+      <c r="AA38"/>
+      <c r="AD38"/>
+      <c r="AF38"/>
+      <c r="AH38"/>
+    </row>
+    <row r="39" spans="1:34">
       <c r="A39">
         <v>40</v>
       </c>
@@ -4470,33 +4392,30 @@
         <v>1</v>
       </c>
       <c r="R39"/>
-      <c r="S39">
-        <v>0</v>
-      </c>
-      <c r="T39" s="3">
+      <c r="S39" s="3">
         <v>76</v>
       </c>
-      <c r="U39">
-        <v>1</v>
-      </c>
-      <c r="V39" s="2">
+      <c r="T39">
+        <v>1</v>
+      </c>
+      <c r="U39" s="2">
         <v>2</v>
       </c>
-      <c r="W39" s="3">
+      <c r="V39" s="3">
         <v>2</v>
       </c>
-      <c r="X39">
+      <c r="W39">
         <v>6</v>
       </c>
-      <c r="Y39" s="2">
+      <c r="X39" s="2">
         <v>7</v>
       </c>
-      <c r="AB39"/>
-      <c r="AE39"/>
-      <c r="AG39"/>
-      <c r="AI39"/>
-    </row>
-    <row r="40" spans="1:35" hidden="1">
+      <c r="AA39"/>
+      <c r="AD39"/>
+      <c r="AF39"/>
+      <c r="AH39"/>
+    </row>
+    <row r="40" spans="1:34" hidden="1">
       <c r="A40">
         <v>41</v>
       </c>
@@ -4535,30 +4454,30 @@
         <v>1</v>
       </c>
       <c r="R40"/>
-      <c r="T40" s="3">
+      <c r="S40" s="3">
         <v>7</v>
       </c>
-      <c r="U40">
+      <c r="T40">
         <v>4</v>
       </c>
-      <c r="V40" s="2">
+      <c r="U40" s="2">
         <v>5</v>
       </c>
-      <c r="W40" s="3">
+      <c r="V40" s="3">
         <v>38</v>
       </c>
-      <c r="X40">
+      <c r="W40">
         <v>4</v>
       </c>
-      <c r="Y40" s="2">
+      <c r="X40" s="2">
         <v>5</v>
       </c>
-      <c r="AB40"/>
-      <c r="AE40"/>
-      <c r="AG40"/>
-      <c r="AI40"/>
-    </row>
-    <row r="41" spans="1:35" hidden="1">
+      <c r="AA40"/>
+      <c r="AD40"/>
+      <c r="AF40"/>
+      <c r="AH40"/>
+    </row>
+    <row r="41" spans="1:34" hidden="1">
       <c r="A41">
         <v>42</v>
       </c>
@@ -4597,30 +4516,30 @@
         <v>0</v>
       </c>
       <c r="R41"/>
-      <c r="T41" s="3">
+      <c r="S41" s="3">
         <v>6</v>
       </c>
-      <c r="U41">
+      <c r="T41">
         <v>3</v>
       </c>
-      <c r="V41" s="2">
+      <c r="U41" s="2">
         <v>3</v>
       </c>
-      <c r="W41" s="3">
+      <c r="V41" s="3">
         <v>39</v>
       </c>
-      <c r="X41">
+      <c r="W41">
         <v>2</v>
       </c>
-      <c r="Y41" s="2">
+      <c r="X41" s="2">
         <v>3</v>
       </c>
-      <c r="AB41"/>
-      <c r="AE41"/>
-      <c r="AG41"/>
-      <c r="AI41"/>
-    </row>
-    <row r="42" spans="1:35" hidden="1">
+      <c r="AA41"/>
+      <c r="AD41"/>
+      <c r="AF41"/>
+      <c r="AH41"/>
+    </row>
+    <row r="42" spans="1:34" hidden="1">
       <c r="A42">
         <v>43</v>
       </c>
@@ -4659,30 +4578,30 @@
         <v>1</v>
       </c>
       <c r="R42"/>
-      <c r="T42" s="3">
+      <c r="S42" s="3">
         <v>7</v>
       </c>
-      <c r="U42">
-        <v>1</v>
-      </c>
-      <c r="V42" s="2">
+      <c r="T42">
+        <v>1</v>
+      </c>
+      <c r="U42" s="2">
         <v>3</v>
       </c>
-      <c r="W42" s="3">
+      <c r="V42" s="3">
         <v>41</v>
       </c>
-      <c r="X42">
-        <v>1</v>
-      </c>
-      <c r="Y42" s="2">
-        <v>1</v>
-      </c>
-      <c r="AB42"/>
-      <c r="AE42"/>
-      <c r="AG42"/>
-      <c r="AI42"/>
-    </row>
-    <row r="43" spans="1:35" hidden="1">
+      <c r="W42">
+        <v>1</v>
+      </c>
+      <c r="X42" s="2">
+        <v>1</v>
+      </c>
+      <c r="AA42"/>
+      <c r="AD42"/>
+      <c r="AF42"/>
+      <c r="AH42"/>
+    </row>
+    <row r="43" spans="1:34" hidden="1">
       <c r="A43">
         <v>44</v>
       </c>
@@ -4721,38 +4640,38 @@
         <v>1</v>
       </c>
       <c r="R43"/>
-      <c r="T43" s="3">
+      <c r="S43" s="3">
         <v>6</v>
       </c>
-      <c r="U43">
+      <c r="T43">
         <v>5</v>
       </c>
-      <c r="V43" s="2">
+      <c r="U43" s="2">
         <v>5</v>
       </c>
-      <c r="W43" s="3">
+      <c r="V43" s="3">
         <v>14</v>
       </c>
-      <c r="X43">
-        <v>1</v>
-      </c>
-      <c r="Y43" s="2">
-        <v>1</v>
-      </c>
-      <c r="Z43" s="3">
+      <c r="W43">
+        <v>1</v>
+      </c>
+      <c r="X43" s="2">
+        <v>1</v>
+      </c>
+      <c r="Y43" s="3">
         <v>18</v>
       </c>
-      <c r="AA43">
+      <c r="Z43">
         <v>0.9</v>
       </c>
-      <c r="AB43" s="2">
+      <c r="AA43" s="2">
         <v>1.2</v>
       </c>
-      <c r="AE43"/>
-      <c r="AG43"/>
-      <c r="AI43"/>
-    </row>
-    <row r="44" spans="1:35">
+      <c r="AD43"/>
+      <c r="AF43"/>
+      <c r="AH43"/>
+    </row>
+    <row r="44" spans="1:34">
       <c r="A44">
         <v>45</v>
       </c>
@@ -4792,29 +4711,26 @@
       <c r="P44">
         <v>1</v>
       </c>
-      <c r="S44">
-        <v>0</v>
-      </c>
-      <c r="T44" s="3">
+      <c r="S44" s="3">
         <v>15</v>
       </c>
-      <c r="U44">
+      <c r="T44">
         <v>2</v>
       </c>
-      <c r="V44" s="2">
+      <c r="U44" s="2">
         <v>2</v>
       </c>
-      <c r="W44" s="3">
+      <c r="V44" s="3">
         <v>42</v>
       </c>
-      <c r="X44">
+      <c r="W44">
         <v>8</v>
       </c>
-      <c r="Y44" s="2">
+      <c r="X44" s="2">
         <v>12</v>
       </c>
     </row>
-    <row r="45" spans="1:35" hidden="1">
+    <row r="45" spans="1:34" hidden="1">
       <c r="A45">
         <v>46</v>
       </c>
@@ -4853,38 +4769,38 @@
         <v>1</v>
       </c>
       <c r="R45"/>
-      <c r="T45" s="3">
+      <c r="S45" s="3">
         <v>7</v>
       </c>
-      <c r="U45">
+      <c r="T45">
         <v>7</v>
       </c>
-      <c r="V45" s="2">
+      <c r="U45" s="2">
         <v>9</v>
       </c>
-      <c r="W45" s="3">
+      <c r="V45" s="3">
         <v>26</v>
       </c>
-      <c r="X45">
+      <c r="W45">
         <v>2</v>
       </c>
-      <c r="Y45" s="2">
+      <c r="X45" s="2">
         <v>2</v>
       </c>
-      <c r="Z45" s="3">
+      <c r="Y45" s="3">
         <v>2</v>
       </c>
-      <c r="AA45">
+      <c r="Z45">
         <v>7</v>
       </c>
-      <c r="AB45" s="2">
+      <c r="AA45" s="2">
         <v>8</v>
       </c>
-      <c r="AE45"/>
-      <c r="AG45"/>
-      <c r="AI45"/>
-    </row>
-    <row r="46" spans="1:35">
+      <c r="AD45"/>
+      <c r="AF45"/>
+      <c r="AH45"/>
+    </row>
+    <row r="46" spans="1:34">
       <c r="A46">
         <v>47</v>
       </c>
@@ -4929,41 +4845,38 @@
         <v>1</v>
       </c>
       <c r="R46"/>
-      <c r="S46">
-        <v>0</v>
-      </c>
-      <c r="T46" s="3">
+      <c r="S46" s="3">
         <v>32</v>
       </c>
-      <c r="U46">
+      <c r="T46">
         <v>40</v>
       </c>
-      <c r="V46" s="2">
+      <c r="U46" s="2">
         <v>40</v>
       </c>
-      <c r="W46" s="3">
+      <c r="V46" s="3">
         <v>33</v>
       </c>
-      <c r="X46">
+      <c r="W46">
         <v>30</v>
       </c>
-      <c r="Y46" s="2">
+      <c r="X46" s="2">
         <v>30</v>
       </c>
-      <c r="Z46" s="3">
+      <c r="Y46" s="3">
         <v>19</v>
       </c>
-      <c r="AA46">
-        <v>1</v>
-      </c>
-      <c r="AB46" s="2">
-        <v>1</v>
-      </c>
-      <c r="AE46"/>
-      <c r="AG46"/>
-      <c r="AI46"/>
-    </row>
-    <row r="47" spans="1:35" hidden="1">
+      <c r="Z46">
+        <v>1</v>
+      </c>
+      <c r="AA46" s="2">
+        <v>1</v>
+      </c>
+      <c r="AD46"/>
+      <c r="AF46"/>
+      <c r="AH46"/>
+    </row>
+    <row r="47" spans="1:34" hidden="1">
       <c r="A47">
         <v>48</v>
       </c>
@@ -5002,22 +4915,22 @@
         <v>0</v>
       </c>
       <c r="R47"/>
-      <c r="T47" s="3">
+      <c r="S47" s="3">
         <v>11</v>
       </c>
-      <c r="U47">
+      <c r="T47">
         <v>10</v>
       </c>
-      <c r="V47" s="2">
+      <c r="U47" s="2">
         <v>14</v>
       </c>
-      <c r="Y47"/>
-      <c r="AB47"/>
-      <c r="AE47"/>
-      <c r="AG47"/>
-      <c r="AI47"/>
-    </row>
-    <row r="48" spans="1:35" hidden="1">
+      <c r="X47"/>
+      <c r="AA47"/>
+      <c r="AD47"/>
+      <c r="AF47"/>
+      <c r="AH47"/>
+    </row>
+    <row r="48" spans="1:34" hidden="1">
       <c r="A48">
         <v>49</v>
       </c>
@@ -5056,30 +4969,30 @@
         <v>0</v>
       </c>
       <c r="R48"/>
-      <c r="T48" s="3">
+      <c r="S48" s="3">
         <v>11</v>
       </c>
-      <c r="U48">
+      <c r="T48">
         <v>8</v>
       </c>
-      <c r="V48" s="2">
+      <c r="U48" s="2">
         <v>11</v>
       </c>
-      <c r="W48" s="3">
+      <c r="V48" s="3">
         <v>6</v>
       </c>
-      <c r="X48">
+      <c r="W48">
         <v>3</v>
       </c>
-      <c r="Y48" s="2">
+      <c r="X48" s="2">
         <v>3</v>
       </c>
-      <c r="AB48"/>
-      <c r="AE48"/>
-      <c r="AG48"/>
-      <c r="AI48"/>
-    </row>
-    <row r="49" spans="1:35">
+      <c r="AA48"/>
+      <c r="AD48"/>
+      <c r="AF48"/>
+      <c r="AH48"/>
+    </row>
+    <row r="49" spans="1:34">
       <c r="A49">
         <v>50</v>
       </c>
@@ -5119,29 +5032,26 @@
       <c r="P49">
         <v>0</v>
       </c>
-      <c r="S49">
-        <v>0</v>
-      </c>
-      <c r="T49" s="3">
+      <c r="S49" s="3">
         <v>11</v>
       </c>
-      <c r="U49">
+      <c r="T49">
         <v>7</v>
       </c>
-      <c r="V49" s="2">
+      <c r="U49" s="2">
         <v>11</v>
       </c>
-      <c r="W49" s="3">
+      <c r="V49" s="3">
         <v>45</v>
       </c>
-      <c r="X49">
+      <c r="W49">
         <v>2</v>
       </c>
-      <c r="Y49" s="2">
+      <c r="X49" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="50" spans="1:35" hidden="1">
+    <row r="50" spans="1:34" hidden="1">
       <c r="A50">
         <v>51</v>
       </c>
@@ -5180,30 +5090,30 @@
         <v>1</v>
       </c>
       <c r="R50"/>
-      <c r="T50" s="3">
+      <c r="S50" s="3">
         <v>6</v>
       </c>
-      <c r="U50">
+      <c r="T50">
         <v>5</v>
       </c>
-      <c r="V50" s="2">
+      <c r="U50" s="2">
         <v>7</v>
       </c>
-      <c r="W50" s="3">
+      <c r="V50" s="3">
         <v>18</v>
       </c>
-      <c r="X50">
+      <c r="W50">
         <v>1.1000000000000001</v>
       </c>
-      <c r="Y50" s="2">
+      <c r="X50" s="2">
         <v>1.7</v>
       </c>
-      <c r="AB50"/>
-      <c r="AE50"/>
-      <c r="AG50"/>
-      <c r="AI50"/>
-    </row>
-    <row r="51" spans="1:35" hidden="1">
+      <c r="AA50"/>
+      <c r="AD50"/>
+      <c r="AF50"/>
+      <c r="AH50"/>
+    </row>
+    <row r="51" spans="1:34" hidden="1">
       <c r="A51">
         <v>52</v>
       </c>
@@ -5242,30 +5152,30 @@
         <v>1</v>
       </c>
       <c r="R51"/>
-      <c r="T51" s="3">
+      <c r="S51" s="3">
         <v>6</v>
       </c>
-      <c r="U51">
-        <v>1</v>
-      </c>
-      <c r="V51" s="2">
+      <c r="T51">
+        <v>1</v>
+      </c>
+      <c r="U51" s="2">
         <v>3</v>
       </c>
-      <c r="W51" s="3">
+      <c r="V51" s="3">
         <v>49</v>
       </c>
-      <c r="X51">
-        <v>1</v>
-      </c>
-      <c r="Y51" s="2">
-        <v>1</v>
-      </c>
-      <c r="AB51"/>
-      <c r="AE51"/>
-      <c r="AG51"/>
-      <c r="AI51"/>
-    </row>
-    <row r="52" spans="1:35">
+      <c r="W51">
+        <v>1</v>
+      </c>
+      <c r="X51" s="2">
+        <v>1</v>
+      </c>
+      <c r="AA51"/>
+      <c r="AD51"/>
+      <c r="AF51"/>
+      <c r="AH51"/>
+    </row>
+    <row r="52" spans="1:34">
       <c r="A52">
         <v>53</v>
       </c>
@@ -5307,33 +5217,30 @@
         <v>1</v>
       </c>
       <c r="R52"/>
-      <c r="S52">
-        <v>0</v>
-      </c>
-      <c r="T52" s="3">
+      <c r="S52" s="3">
         <v>9</v>
       </c>
-      <c r="U52">
+      <c r="T52">
         <v>2</v>
       </c>
-      <c r="V52" s="2">
+      <c r="U52" s="2">
         <v>2</v>
       </c>
-      <c r="W52" s="3">
+      <c r="V52" s="3">
         <v>21</v>
       </c>
-      <c r="X52">
+      <c r="W52">
         <v>2</v>
       </c>
-      <c r="Y52" s="2">
+      <c r="X52" s="2">
         <v>2</v>
       </c>
-      <c r="AB52"/>
-      <c r="AE52"/>
-      <c r="AG52"/>
-      <c r="AI52"/>
-    </row>
-    <row r="53" spans="1:35">
+      <c r="AA52"/>
+      <c r="AD52"/>
+      <c r="AF52"/>
+      <c r="AH52"/>
+    </row>
+    <row r="53" spans="1:34">
       <c r="A53">
         <v>54</v>
       </c>
@@ -5377,28 +5284,25 @@
         <v>6</v>
       </c>
       <c r="S53">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="T53">
-        <v>50</v>
-      </c>
-      <c r="U53">
         <v>3</v>
       </c>
-      <c r="V53" s="2">
+      <c r="U53" s="2">
         <v>4</v>
       </c>
+      <c r="V53">
+        <v>51</v>
+      </c>
       <c r="W53">
-        <v>51</v>
-      </c>
-      <c r="X53">
         <v>-0.5</v>
       </c>
-      <c r="Y53" s="2">
+      <c r="X53" s="2">
         <v>-0.5</v>
       </c>
     </row>
-    <row r="54" spans="1:35">
+    <row r="54" spans="1:34">
       <c r="A54">
         <v>55</v>
       </c>
@@ -5442,37 +5346,34 @@
         <v>1</v>
       </c>
       <c r="S54">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="T54">
-        <v>15</v>
-      </c>
-      <c r="U54">
         <v>3</v>
       </c>
-      <c r="V54" s="2">
+      <c r="U54" s="2">
         <v>4</v>
       </c>
+      <c r="V54">
+        <v>14</v>
+      </c>
       <c r="W54">
-        <v>14</v>
-      </c>
-      <c r="X54">
-        <v>1</v>
-      </c>
-      <c r="Y54" s="2">
-        <v>1</v>
+        <v>1</v>
+      </c>
+      <c r="X54" s="2">
+        <v>1</v>
+      </c>
+      <c r="Y54">
+        <v>52</v>
       </c>
       <c r="Z54">
-        <v>52</v>
-      </c>
-      <c r="AA54">
         <v>3</v>
       </c>
-      <c r="AB54" s="2">
+      <c r="AA54" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="55" spans="1:35">
+    <row r="55" spans="1:34">
       <c r="A55">
         <v>56</v>
       </c>
@@ -5513,29 +5414,26 @@
         <v>1</v>
       </c>
       <c r="S55">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="T55">
-        <v>15</v>
-      </c>
-      <c r="U55">
-        <v>1</v>
-      </c>
-      <c r="V55" s="2">
+        <v>1</v>
+      </c>
+      <c r="U55" s="2">
         <v>3</v>
       </c>
+      <c r="V55">
+        <v>60</v>
+      </c>
       <c r="W55">
-        <v>60</v>
-      </c>
-      <c r="X55">
-        <v>1</v>
-      </c>
-      <c r="Y55" s="2">
-        <v>1</v>
-      </c>
-      <c r="AH55" s="2"/>
-    </row>
-    <row r="56" spans="1:35">
+        <v>1</v>
+      </c>
+      <c r="X55" s="2">
+        <v>1</v>
+      </c>
+      <c r="AG55" s="2"/>
+    </row>
+    <row r="56" spans="1:34">
       <c r="A56">
         <v>57</v>
       </c>
@@ -5579,38 +5477,35 @@
         <v>1</v>
       </c>
       <c r="S56">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="T56">
-        <v>45</v>
-      </c>
-      <c r="U56">
         <v>3</v>
       </c>
-      <c r="V56" s="2">
+      <c r="U56" s="2">
         <v>4</v>
       </c>
+      <c r="V56">
+        <v>11</v>
+      </c>
       <c r="W56">
-        <v>11</v>
-      </c>
-      <c r="X56">
         <v>12</v>
       </c>
-      <c r="Y56" s="2">
+      <c r="X56" s="2">
         <v>18</v>
       </c>
+      <c r="Y56">
+        <v>14</v>
+      </c>
       <c r="Z56">
-        <v>14</v>
-      </c>
-      <c r="AA56">
-        <v>1</v>
-      </c>
-      <c r="AB56" s="2">
-        <v>1</v>
-      </c>
-      <c r="AH56" s="2"/>
-    </row>
-    <row r="57" spans="1:35">
+        <v>1</v>
+      </c>
+      <c r="AA56" s="2">
+        <v>1</v>
+      </c>
+      <c r="AG56" s="2"/>
+    </row>
+    <row r="57" spans="1:34">
       <c r="A57">
         <v>58</v>
       </c>
@@ -5654,37 +5549,34 @@
         <v>1</v>
       </c>
       <c r="S57">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="T57">
+        <v>5</v>
+      </c>
+      <c r="U57" s="2">
+        <v>6</v>
+      </c>
+      <c r="V57">
         <v>2</v>
       </c>
-      <c r="U57">
+      <c r="W57">
         <v>5</v>
       </c>
-      <c r="V57" s="2">
+      <c r="X57" s="2">
         <v>6</v>
       </c>
-      <c r="W57">
-        <v>2</v>
-      </c>
-      <c r="X57">
-        <v>5</v>
-      </c>
-      <c r="Y57" s="2">
-        <v>6</v>
+      <c r="Y57">
+        <v>66</v>
       </c>
       <c r="Z57">
-        <v>66</v>
-      </c>
-      <c r="AA57">
         <v>0.6</v>
       </c>
-      <c r="AB57" s="2">
+      <c r="AA57" s="2">
         <v>1.2</v>
       </c>
     </row>
-    <row r="58" spans="1:35">
+    <row r="58" spans="1:34">
       <c r="A58">
         <v>59</v>
       </c>
@@ -5725,19 +5617,16 @@
         <v>0</v>
       </c>
       <c r="S58">
-        <v>0</v>
+        <v>66</v>
       </c>
       <c r="T58">
-        <v>66</v>
-      </c>
-      <c r="U58">
         <v>1.2</v>
       </c>
-      <c r="V58" s="2">
+      <c r="U58" s="2">
         <v>1.7</v>
       </c>
     </row>
-    <row r="59" spans="1:35">
+    <row r="59" spans="1:34">
       <c r="A59">
         <v>60</v>
       </c>
@@ -5778,28 +5667,25 @@
         <v>0</v>
       </c>
       <c r="S59">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="T59">
-        <v>2</v>
-      </c>
-      <c r="U59">
         <v>7</v>
       </c>
-      <c r="V59" s="2">
+      <c r="U59" s="2">
         <v>9</v>
       </c>
+      <c r="V59">
+        <v>66</v>
+      </c>
       <c r="W59">
-        <v>66</v>
-      </c>
-      <c r="X59">
         <v>0.9</v>
       </c>
-      <c r="Y59" s="2">
+      <c r="X59" s="2">
         <v>1.4</v>
       </c>
     </row>
-    <row r="60" spans="1:35">
+    <row r="60" spans="1:34">
       <c r="A60">
         <v>61</v>
       </c>
@@ -5840,28 +5726,25 @@
         <v>1</v>
       </c>
       <c r="S60">
-        <v>0</v>
+        <v>66</v>
       </c>
       <c r="T60">
-        <v>66</v>
-      </c>
-      <c r="U60">
         <v>3</v>
       </c>
-      <c r="V60" s="2">
+      <c r="U60" s="2">
         <v>4</v>
       </c>
+      <c r="V60">
+        <v>67</v>
+      </c>
       <c r="W60">
-        <v>67</v>
-      </c>
-      <c r="X60">
         <v>-1</v>
       </c>
-      <c r="Y60" s="2">
+      <c r="X60" s="2">
         <v>-1</v>
       </c>
     </row>
-    <row r="61" spans="1:35">
+    <row r="61" spans="1:34">
       <c r="A61">
         <v>62</v>
       </c>
@@ -5905,28 +5788,25 @@
         <v>1</v>
       </c>
       <c r="S61">
-        <v>0</v>
+        <v>66</v>
       </c>
       <c r="T61">
-        <v>66</v>
-      </c>
-      <c r="U61">
         <v>1.2</v>
       </c>
-      <c r="V61" s="2">
+      <c r="U61" s="2">
         <v>1.5</v>
       </c>
+      <c r="V61">
+        <v>62</v>
+      </c>
       <c r="W61">
-        <v>62</v>
-      </c>
-      <c r="X61">
-        <v>1</v>
-      </c>
-      <c r="Y61" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="62" spans="1:35" hidden="1">
+        <v>1</v>
+      </c>
+      <c r="X61" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62" spans="1:34" hidden="1">
       <c r="A62">
         <v>63</v>
       </c>
@@ -5969,26 +5849,26 @@
       <c r="P62">
         <v>1</v>
       </c>
+      <c r="S62">
+        <v>15</v>
+      </c>
       <c r="T62">
-        <v>15</v>
-      </c>
-      <c r="U62">
         <v>6</v>
       </c>
-      <c r="V62" s="2">
+      <c r="U62" s="2">
         <v>8</v>
       </c>
+      <c r="V62">
+        <v>45</v>
+      </c>
       <c r="W62">
-        <v>45</v>
-      </c>
-      <c r="X62">
         <v>6</v>
       </c>
-      <c r="Y62" s="2">
+      <c r="X62" s="2">
         <v>8</v>
       </c>
     </row>
-    <row r="63" spans="1:35" hidden="1">
+    <row r="63" spans="1:34" hidden="1">
       <c r="A63">
         <v>64</v>
       </c>
@@ -6034,44 +5914,44 @@
       <c r="R63" s="2">
         <v>14</v>
       </c>
+      <c r="S63">
+        <v>33</v>
+      </c>
       <c r="T63">
-        <v>33</v>
-      </c>
-      <c r="U63">
         <v>-30</v>
       </c>
-      <c r="V63" s="2">
+      <c r="U63" s="2">
         <v>-30</v>
       </c>
+      <c r="V63">
+        <v>11</v>
+      </c>
       <c r="W63">
-        <v>11</v>
-      </c>
-      <c r="X63">
         <v>32</v>
       </c>
-      <c r="Y63" s="2">
+      <c r="X63" s="2">
         <v>40</v>
       </c>
+      <c r="Y63">
+        <v>2</v>
+      </c>
       <c r="Z63">
+        <v>15</v>
+      </c>
+      <c r="AA63" s="2">
+        <v>18</v>
+      </c>
+      <c r="AB63">
+        <v>66</v>
+      </c>
+      <c r="AC63">
+        <v>1.5</v>
+      </c>
+      <c r="AD63" s="2">
         <v>2</v>
       </c>
-      <c r="AA63">
-        <v>15</v>
-      </c>
-      <c r="AB63" s="2">
-        <v>18</v>
-      </c>
-      <c r="AC63">
-        <v>66</v>
-      </c>
-      <c r="AD63">
-        <v>1.5</v>
-      </c>
-      <c r="AE63" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="64" spans="1:35" hidden="1">
+    </row>
+    <row r="64" spans="1:34" hidden="1">
       <c r="A64">
         <v>65</v>
       </c>
@@ -6108,26 +5988,26 @@
       <c r="P64">
         <v>1</v>
       </c>
+      <c r="S64">
+        <v>33</v>
+      </c>
       <c r="T64">
-        <v>33</v>
-      </c>
-      <c r="U64">
         <v>50</v>
       </c>
-      <c r="V64" s="2">
+      <c r="U64" s="2">
         <v>50</v>
       </c>
+      <c r="V64">
+        <v>68</v>
+      </c>
       <c r="W64">
-        <v>68</v>
-      </c>
-      <c r="X64">
         <v>0.1</v>
       </c>
-      <c r="Y64" s="2">
+      <c r="X64" s="2">
         <v>0.15</v>
       </c>
     </row>
-    <row r="65" spans="1:31" hidden="1">
+    <row r="65" spans="1:30" hidden="1">
       <c r="A65">
         <v>66</v>
       </c>
@@ -6164,26 +6044,26 @@
       <c r="P65">
         <v>1</v>
       </c>
+      <c r="S65">
+        <v>19</v>
+      </c>
       <c r="T65">
-        <v>19</v>
-      </c>
-      <c r="U65">
-        <v>1</v>
-      </c>
-      <c r="V65" s="2">
-        <v>1</v>
+        <v>1</v>
+      </c>
+      <c r="U65" s="2">
+        <v>1</v>
+      </c>
+      <c r="V65">
+        <v>69</v>
       </c>
       <c r="W65">
-        <v>69</v>
-      </c>
-      <c r="X65">
-        <v>1</v>
-      </c>
-      <c r="Y65" s="2">
+        <v>1</v>
+      </c>
+      <c r="X65" s="2">
         <v>1.5</v>
       </c>
     </row>
-    <row r="66" spans="1:31" hidden="1">
+    <row r="66" spans="1:30" hidden="1">
       <c r="A66">
         <v>67</v>
       </c>
@@ -6220,44 +6100,44 @@
       <c r="P66">
         <v>1</v>
       </c>
+      <c r="S66">
+        <v>11</v>
+      </c>
       <c r="T66">
-        <v>11</v>
-      </c>
-      <c r="U66">
         <v>12</v>
       </c>
-      <c r="V66" s="2">
+      <c r="U66" s="2">
         <v>15</v>
       </c>
+      <c r="V66">
+        <v>9</v>
+      </c>
       <c r="W66">
-        <v>9</v>
-      </c>
-      <c r="X66">
-        <v>1</v>
-      </c>
-      <c r="Y66" s="2">
-        <v>1</v>
+        <v>1</v>
+      </c>
+      <c r="X66" s="2">
+        <v>1</v>
+      </c>
+      <c r="Y66">
+        <v>14</v>
       </c>
       <c r="Z66">
-        <v>14</v>
-      </c>
-      <c r="AA66">
-        <v>1</v>
-      </c>
-      <c r="AB66" s="2">
-        <v>1</v>
+        <v>1</v>
+      </c>
+      <c r="AA66" s="2">
+        <v>1</v>
+      </c>
+      <c r="AB66">
+        <v>2</v>
       </c>
       <c r="AC66">
-        <v>2</v>
-      </c>
-      <c r="AD66">
         <v>5</v>
       </c>
-      <c r="AE66" s="2">
+      <c r="AD66" s="2">
         <v>7</v>
       </c>
     </row>
-    <row r="67" spans="1:31" hidden="1">
+    <row r="67" spans="1:30" hidden="1">
       <c r="A67">
         <v>68</v>
       </c>
@@ -6297,35 +6177,35 @@
       <c r="P67">
         <v>1</v>
       </c>
+      <c r="S67">
+        <v>9</v>
+      </c>
       <c r="T67">
-        <v>9</v>
-      </c>
-      <c r="U67">
         <v>2</v>
       </c>
-      <c r="V67" s="2">
+      <c r="U67" s="2">
         <v>2</v>
       </c>
+      <c r="V67">
+        <v>14</v>
+      </c>
       <c r="W67">
-        <v>14</v>
-      </c>
-      <c r="X67">
-        <v>1</v>
-      </c>
-      <c r="Y67" s="2">
-        <v>1</v>
+        <v>1</v>
+      </c>
+      <c r="X67" s="2">
+        <v>1</v>
+      </c>
+      <c r="Y67">
+        <v>70</v>
       </c>
       <c r="Z67">
-        <v>70</v>
-      </c>
-      <c r="AA67">
-        <v>1</v>
-      </c>
-      <c r="AB67" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="68" spans="1:31" hidden="1">
+        <v>1</v>
+      </c>
+      <c r="AA67" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68" spans="1:30" hidden="1">
       <c r="A68">
         <v>69</v>
       </c>
@@ -6362,26 +6242,26 @@
       <c r="P68">
         <v>1</v>
       </c>
+      <c r="S68">
+        <v>3</v>
+      </c>
       <c r="T68">
-        <v>3</v>
-      </c>
-      <c r="U68">
-        <v>1</v>
-      </c>
-      <c r="V68" s="2">
-        <v>1</v>
+        <v>1</v>
+      </c>
+      <c r="U68" s="2">
+        <v>1</v>
+      </c>
+      <c r="V68">
+        <v>72</v>
       </c>
       <c r="W68">
-        <v>72</v>
-      </c>
-      <c r="X68">
-        <v>1</v>
-      </c>
-      <c r="Y68" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="69" spans="1:31">
+        <v>1</v>
+      </c>
+      <c r="X68" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69" spans="1:30">
       <c r="A69">
         <v>70</v>
       </c>
@@ -6422,19 +6302,16 @@
         <v>0</v>
       </c>
       <c r="S69">
-        <v>0</v>
+        <v>66</v>
       </c>
       <c r="T69">
-        <v>66</v>
-      </c>
-      <c r="U69">
         <v>0.7</v>
       </c>
-      <c r="V69" s="2">
+      <c r="U69" s="2">
         <v>0.9</v>
       </c>
     </row>
-    <row r="70" spans="1:31">
+    <row r="70" spans="1:30">
       <c r="A70">
         <v>71</v>
       </c>
@@ -6472,19 +6349,16 @@
         <v>0</v>
       </c>
       <c r="S70">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="T70">
-        <v>11</v>
-      </c>
-      <c r="U70">
         <v>18</v>
       </c>
-      <c r="V70" s="2">
+      <c r="U70" s="2">
         <v>22</v>
       </c>
     </row>
-    <row r="71" spans="1:31" hidden="1">
+    <row r="71" spans="1:30" hidden="1">
       <c r="A71">
         <v>72</v>
       </c>
@@ -6521,26 +6395,26 @@
       <c r="P71">
         <v>1</v>
       </c>
+      <c r="S71">
+        <v>33</v>
+      </c>
       <c r="T71">
-        <v>33</v>
-      </c>
-      <c r="U71">
         <v>50</v>
       </c>
-      <c r="V71" s="2">
+      <c r="U71" s="2">
         <v>100</v>
       </c>
+      <c r="V71">
+        <v>14</v>
+      </c>
       <c r="W71">
-        <v>14</v>
-      </c>
-      <c r="X71">
-        <v>1</v>
-      </c>
-      <c r="Y71" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="72" spans="1:31" hidden="1">
+        <v>1</v>
+      </c>
+      <c r="X71" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72" spans="1:30" hidden="1">
       <c r="A72">
         <v>73</v>
       </c>
@@ -6577,26 +6451,26 @@
       <c r="P72">
         <v>1</v>
       </c>
+      <c r="S72">
+        <v>38</v>
+      </c>
       <c r="T72">
-        <v>38</v>
-      </c>
-      <c r="U72">
         <v>5</v>
       </c>
-      <c r="V72" s="2">
+      <c r="U72" s="2">
         <v>6</v>
       </c>
+      <c r="V72">
+        <v>2</v>
+      </c>
       <c r="W72">
-        <v>2</v>
-      </c>
-      <c r="X72">
         <v>5</v>
       </c>
-      <c r="Y72" s="2">
+      <c r="X72" s="2">
         <v>6</v>
       </c>
     </row>
-    <row r="73" spans="1:31">
+    <row r="73" spans="1:30">
       <c r="A73">
         <v>74</v>
       </c>
@@ -6637,28 +6511,25 @@
         <v>0</v>
       </c>
       <c r="S73">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="T73">
-        <v>45</v>
-      </c>
-      <c r="U73">
         <v>2</v>
       </c>
-      <c r="V73" s="2">
+      <c r="U73" s="2">
         <v>3</v>
+      </c>
+      <c r="V73">
+        <v>2</v>
       </c>
       <c r="W73">
         <v>2</v>
       </c>
-      <c r="X73">
-        <v>2</v>
-      </c>
-      <c r="Y73" s="2">
+      <c r="X73" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="74" spans="1:31">
+    <row r="74" spans="1:30">
       <c r="A74">
         <v>75</v>
       </c>
@@ -6699,29 +6570,26 @@
         <v>0</v>
       </c>
       <c r="S74">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="T74">
-        <v>11</v>
-      </c>
-      <c r="U74">
         <v>5</v>
       </c>
-      <c r="V74" s="2">
+      <c r="U74" s="2">
         <v>8</v>
       </c>
+      <c r="V74">
+        <v>66</v>
+      </c>
       <c r="W74">
-        <v>66</v>
-      </c>
-      <c r="X74">
         <v>0.6</v>
       </c>
-      <c r="Y74" s="2">
+      <c r="X74" s="2">
         <v>0.8</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AK74" xr:uid="{00000000-0009-0000-0000-000000000000}">
+  <autoFilter ref="A1:AJ74" xr:uid="{00000000-0009-0000-0000-000000000000}">
     <filterColumn colId="6">
       <filters>
         <filter val="C"/>
@@ -8476,7 +8344,7 @@
         <v>9</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="I1" t="s">
         <v>18</v>

</xml_diff>